<commit_message>
push fleet model update aircraft nomenclature
</commit_message>
<xml_diff>
--- a/aeromaps/utils/calibration_notebooks/fleet_calibrated_inputs_processed_here/aircraft_type_key_parameters.xlsx
+++ b/aeromaps/utils/calibration_notebooks/fleet_calibrated_inputs_processed_here/aircraft_type_key_parameters.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J112"/>
+  <dimension ref="A1:J108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -494,16 +494,16 @@
         <v>371571726.8318613</v>
       </c>
       <c r="F2" t="n">
-        <v>1.904737906228883</v>
+        <v>1.178449744963836</v>
       </c>
       <c r="G2" t="n">
-        <v>1993803.690489483</v>
+        <v>1997786.487702498</v>
       </c>
       <c r="H2" t="n">
-        <v>279132516.6685275</v>
+        <v>279690108.2783498</v>
       </c>
       <c r="I2" t="n">
-        <v>6307623013.427601</v>
+        <v>6320223041.945186</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -528,16 +528,16 @@
         <v>524826906.5019609</v>
       </c>
       <c r="F3" t="n">
-        <v>1.412938209082142</v>
+        <v>0.8524547275953843</v>
       </c>
       <c r="G3" t="n">
-        <v>2155750.270211081</v>
+        <v>2160056.56987795</v>
       </c>
       <c r="H3" t="n">
-        <v>394261039.3861879</v>
+        <v>395048610.2871538</v>
       </c>
       <c r="I3" t="n">
-        <v>798879917202.859</v>
+        <v>800475749692.7611</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -562,16 +562,16 @@
         <v>641773498.6793677</v>
       </c>
       <c r="F4" t="n">
-        <v>1.446328441586544</v>
+        <v>0.8330292323059032</v>
       </c>
       <c r="G4" t="n">
-        <v>2429533.824087007</v>
+        <v>2434387.030342798</v>
       </c>
       <c r="H4" t="n">
-        <v>482113785.5265285</v>
+        <v>483076849.9698891</v>
       </c>
       <c r="I4" t="n">
-        <v>746770436479.7814</v>
+        <v>748262175725.4059</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -596,19 +596,19 @@
         <v>915711708.154284</v>
       </c>
       <c r="F5" t="n">
-        <v>2.170477416625605</v>
+        <v>1.229639562991454</v>
       </c>
       <c r="G5" t="n">
-        <v>2565936.795986042</v>
+        <v>2571062.479105487</v>
       </c>
       <c r="H5" t="n">
-        <v>687901945.1219021</v>
+        <v>689276089.4084879</v>
       </c>
       <c r="I5" t="n">
-        <v>13188562215.41278</v>
+        <v>13214907521.66625</v>
       </c>
       <c r="J5" t="n">
-        <v>-1.259580082256914</v>
+        <v>-0.722863936181168</v>
       </c>
     </row>
     <row r="6">
@@ -630,19 +630,19 @@
         <v>814938508.190392</v>
       </c>
       <c r="F6" t="n">
-        <v>2.111221625367664</v>
+        <v>1.174570952133184</v>
       </c>
       <c r="G6" t="n">
-        <v>2650400.673604153</v>
+        <v>2655695.080704791</v>
       </c>
       <c r="H6" t="n">
-        <v>612198992.2667445</v>
+        <v>613421913.2854193</v>
       </c>
       <c r="I6" t="n">
-        <v>11354047191.18516</v>
+        <v>11376727893.26491</v>
       </c>
       <c r="J6" t="n">
-        <v>-1.038083426852898</v>
+        <v>-0.4353897039194094</v>
       </c>
     </row>
     <row r="7">
@@ -664,19 +664,19 @@
         <v>288887383.8273833</v>
       </c>
       <c r="F7" t="n">
-        <v>2.782981495402267</v>
+        <v>1.680027915024445</v>
       </c>
       <c r="G7" t="n">
-        <v>2281070.3172418</v>
+        <v>2285626.954660789</v>
       </c>
       <c r="H7" t="n">
-        <v>217018294.607796</v>
+        <v>217451807.6276887</v>
       </c>
       <c r="I7" t="n">
-        <v>4993085395.383477</v>
+        <v>5003059520.063828</v>
       </c>
       <c r="J7" t="n">
-        <v>-2.442436684757639</v>
+        <v>-2.718118701741198</v>
       </c>
     </row>
     <row r="8">
@@ -698,19 +698,19 @@
         <v>346880743.7460527</v>
       </c>
       <c r="F8" t="n">
-        <v>2.120925647002421</v>
+        <v>1.343098767003529</v>
       </c>
       <c r="G8" t="n">
-        <v>1993803.690489483</v>
+        <v>1997786.487702498</v>
       </c>
       <c r="H8" t="n">
-        <v>260584129.5064426</v>
+        <v>261104669.0910091</v>
       </c>
       <c r="I8" t="n">
-        <v>232455692953.8527</v>
+        <v>232920043526.8115</v>
       </c>
       <c r="J8" t="n">
-        <v>-1.127859907872356</v>
+        <v>-1.101696162447163</v>
       </c>
     </row>
     <row r="9">
@@ -732,19 +732,19 @@
         <v>453313595.4366798</v>
       </c>
       <c r="F9" t="n">
-        <v>1.865365362252669</v>
+        <v>1.129040999847672</v>
       </c>
       <c r="G9" t="n">
-        <v>2161144.726974176</v>
+        <v>2165461.802540128</v>
       </c>
       <c r="H9" t="n">
-        <v>340538732.0859234</v>
+        <v>341218987.9804959</v>
       </c>
       <c r="I9" t="n">
-        <v>1167940425019.813</v>
+        <v>1170273488145.298</v>
       </c>
       <c r="J9" t="n">
-        <v>-0.7146336173998215</v>
+        <v>-0.5621891901178458</v>
       </c>
     </row>
     <row r="10">
@@ -766,19 +766,19 @@
         <v>560616094.5019472</v>
       </c>
       <c r="F10" t="n">
-        <v>2.025617642195404</v>
+        <v>1.213652392088143</v>
       </c>
       <c r="G10" t="n">
-        <v>2262400.938350429</v>
+        <v>2266920.282052604</v>
       </c>
       <c r="H10" t="n">
-        <v>421146632.1118146</v>
+        <v>421987909.3351676</v>
       </c>
       <c r="I10" t="n">
-        <v>625619629066.2284</v>
+        <v>626869358980.4314</v>
       </c>
       <c r="J10" t="n">
-        <v>0.001830711561807127</v>
+        <v>-0.2196441321817518</v>
       </c>
     </row>
     <row r="11">
@@ -800,19 +800,19 @@
         <v>1224179199.890376</v>
       </c>
       <c r="F11" t="n">
-        <v>2.210340183143528</v>
+        <v>1.158197581335016</v>
       </c>
       <c r="G11" t="n">
-        <v>3500576.393797548</v>
+        <v>3507569.101239946</v>
       </c>
       <c r="H11" t="n">
-        <v>919629229.683803</v>
+        <v>921466269.4838915</v>
       </c>
       <c r="I11" t="n">
-        <v>394964101839.0745</v>
+        <v>395753077168.767</v>
       </c>
       <c r="J11" t="n">
-        <v>-1.344367604773331</v>
+        <v>-1.447335696156048</v>
       </c>
     </row>
     <row r="12">
@@ -834,19 +834,19 @@
         <v>1384950473.663155</v>
       </c>
       <c r="F12" t="n">
-        <v>2.085453342415542</v>
+        <v>1.148368652583524</v>
       </c>
       <c r="G12" t="n">
-        <v>3606081.399511821</v>
+        <v>3613284.862428653</v>
       </c>
       <c r="H12" t="n">
-        <v>1040404000.786093</v>
+        <v>1042482298.75219</v>
       </c>
       <c r="I12" t="n">
-        <v>635287214309.1821</v>
+        <v>636556256070.2565</v>
       </c>
       <c r="J12" t="n">
-        <v>-0.5100694580772367</v>
+        <v>-0.5836565905168096</v>
       </c>
     </row>
     <row r="13">
@@ -868,16 +868,16 @@
         <v>1165707493.905956</v>
       </c>
       <c r="F13" t="n">
-        <v>2.319533741877407</v>
+        <v>1.206911147835214</v>
       </c>
       <c r="G13" t="n">
-        <v>3574302.249524496</v>
+        <v>3581442.23081041</v>
       </c>
       <c r="H13" t="n">
-        <v>875704051.1335014</v>
+        <v>877453346.5485505</v>
       </c>
       <c r="I13" t="n">
-        <v>5932019800.001555</v>
+        <v>5943869528.256999</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -902,16 +902,16 @@
         <v>1300462062.965058</v>
       </c>
       <c r="F14" t="n">
-        <v>2.079182424675519</v>
+        <v>1.081850374244981</v>
       </c>
       <c r="G14" t="n">
-        <v>3574302.249524496</v>
+        <v>3581442.23081041</v>
       </c>
       <c r="H14" t="n">
-        <v>976934525.0308623</v>
+        <v>978886037.1692698</v>
       </c>
       <c r="I14" t="n">
-        <v>134983057807.5723</v>
+        <v>135252698268.6693</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -936,19 +936,19 @@
         <v>1338821871.007196</v>
       </c>
       <c r="F15" t="n">
-        <v>2.471666250499918</v>
+        <v>1.225404189833046</v>
       </c>
       <c r="G15" t="n">
-        <v>3623241.455703219</v>
+        <v>3630479.197332795</v>
       </c>
       <c r="H15" t="n">
-        <v>1005751221.739783</v>
+        <v>1007760297.749643</v>
       </c>
       <c r="I15" t="n">
-        <v>4508214853.748553</v>
+        <v>4517220407.124161</v>
       </c>
       <c r="J15" t="n">
-        <v>-1.341103609368384</v>
+        <v>-0.9563513210372246</v>
       </c>
     </row>
     <row r="16">
@@ -970,19 +970,19 @@
         <v>1350130690.79833</v>
       </c>
       <c r="F16" t="n">
-        <v>2.530187724259435</v>
+        <v>1.260179397395529</v>
       </c>
       <c r="G16" t="n">
-        <v>3659095.448890476</v>
+        <v>3666404.812006572</v>
       </c>
       <c r="H16" t="n">
-        <v>1014246645.640209</v>
+        <v>1016272692.002163</v>
       </c>
       <c r="I16" t="n">
-        <v>55237081051.80188</v>
+        <v>55347421951.21822</v>
       </c>
       <c r="J16" t="n">
-        <v>-1.609200840750934</v>
+        <v>-1.411448629326703</v>
       </c>
     </row>
     <row r="17">
@@ -1004,19 +1004,19 @@
         <v>1042530264.242206</v>
       </c>
       <c r="F17" t="n">
-        <v>4.259262412067179</v>
+        <v>2.076914867607091</v>
       </c>
       <c r="G17" t="n">
-        <v>3830453.712047529</v>
+        <v>3838105.378278112</v>
       </c>
       <c r="H17" t="n">
-        <v>783170718.7256291</v>
+        <v>784735170.7179365</v>
       </c>
       <c r="I17" t="n">
-        <v>14388464678.14303</v>
+        <v>14417206894.48712</v>
       </c>
       <c r="J17" t="n">
-        <v>-1.664820494382353</v>
+        <v>-1.822473864884408</v>
       </c>
     </row>
     <row r="18">
@@ -1038,19 +1038,19 @@
         <v>1464744673.093225</v>
       </c>
       <c r="F18" t="n">
-        <v>2.801019561395783</v>
+        <v>1.428662850478296</v>
       </c>
       <c r="G18" t="n">
-        <v>3634550.173053185</v>
+        <v>3641810.50483452</v>
       </c>
       <c r="H18" t="n">
-        <v>1100347086.048187</v>
+        <v>1102545125.568611</v>
       </c>
       <c r="I18" t="n">
-        <v>46522164741.67451</v>
+        <v>46615096833.71568</v>
       </c>
       <c r="J18" t="n">
-        <v>-1.928245312921163</v>
+        <v>-2.063959410459421</v>
       </c>
     </row>
     <row r="19">
@@ -1072,19 +1072,19 @@
         <v>1441813781.26995</v>
       </c>
       <c r="F19" t="n">
-        <v>2.125373803679078</v>
+        <v>1.097180837791816</v>
       </c>
       <c r="G19" t="n">
-        <v>3661127.954609676</v>
+        <v>3668441.377833672</v>
       </c>
       <c r="H19" t="n">
-        <v>1083120916.558222</v>
+        <v>1085284545.298807</v>
       </c>
       <c r="I19" t="n">
-        <v>562531554576.3455</v>
+        <v>563655260545.2366</v>
       </c>
       <c r="J19" t="n">
-        <v>0.8239271828251541</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -1106,16 +1106,16 @@
         <v>1654137551.758496</v>
       </c>
       <c r="F20" t="n">
-        <v>2.001308765589342</v>
+        <v>0.9984880328710761</v>
       </c>
       <c r="G20" t="n">
-        <v>3665663.813677243</v>
+        <v>3672986.297676349</v>
       </c>
       <c r="H20" t="n">
-        <v>1242623010.300239</v>
+        <v>1245105258.420182</v>
       </c>
       <c r="I20" t="n">
-        <v>111439263571.0907</v>
+        <v>111661873244.4947</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1140,19 +1140,19 @@
         <v>2317785585.396739</v>
       </c>
       <c r="F21" t="n">
-        <v>2.819298712196609</v>
+        <v>1.412066518413993</v>
       </c>
       <c r="G21" t="n">
-        <v>3685597.080659749</v>
+        <v>3692959.383102648</v>
       </c>
       <c r="H21" t="n">
-        <v>1741169407.764402</v>
+        <v>1744647545.906944</v>
       </c>
       <c r="I21" t="n">
-        <v>354928369289.347</v>
+        <v>355637369742.4854</v>
       </c>
       <c r="J21" t="n">
-        <v>-1.245911163120915</v>
+        <v>-1.80793649262165</v>
       </c>
     </row>
     <row r="22">
@@ -1174,16 +1174,16 @@
         <v>135894357.2431726</v>
       </c>
       <c r="F22" t="n">
-        <v>3.902026249335376</v>
+        <v>2.729543634431751</v>
       </c>
       <c r="G22" t="n">
-        <v>1276083.835204698</v>
+        <v>1278632.924248254</v>
       </c>
       <c r="H22" t="n">
-        <v>102086706.8163758</v>
+        <v>102290633.9398603</v>
       </c>
       <c r="I22" t="n">
-        <v>14969431509.27357</v>
+        <v>14999334257.66347</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1195,32 +1195,32 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>AN24</t>
+          <t>AT43</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>52</v>
+        <v>41.49033614059356</v>
       </c>
       <c r="D23" t="n">
-        <v>1101395.512311833</v>
+        <v>975824.3201168067</v>
       </c>
       <c r="E23" t="n">
-        <v>57272566.64021534</v>
+        <v>40487279.05581249</v>
       </c>
       <c r="F23" t="n">
-        <v>3.699540219623766</v>
+        <v>2.41333855030665</v>
       </c>
       <c r="G23" t="n">
-        <v>827391.5343891077</v>
+        <v>734524.1579094057</v>
       </c>
       <c r="H23" t="n">
-        <v>43024359.78823362</v>
+        <v>30475654.21504767</v>
       </c>
       <c r="I23" t="n">
-        <v>2684182077.837289</v>
+        <v>1376416694.881595</v>
       </c>
       <c r="J23" t="n">
-        <v>0.9946554822623437</v>
+        <v>-0.174175411036816</v>
       </c>
     </row>
     <row r="24">
@@ -1229,32 +1229,32 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>AT43</t>
+          <t>AT45</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>41.49033614059356</v>
+        <v>42</v>
       </c>
       <c r="D24" t="n">
-        <v>975824.3201168067</v>
+        <v>610417.8060183238</v>
       </c>
       <c r="E24" t="n">
-        <v>40487279.05581249</v>
+        <v>25637547.8527696</v>
       </c>
       <c r="F24" t="n">
-        <v>3.308508974203637</v>
+        <v>4.028249795385581</v>
       </c>
       <c r="G24" t="n">
-        <v>733059.8068453545</v>
+        <v>459474.7391465366</v>
       </c>
       <c r="H24" t="n">
-        <v>30414897.79717235</v>
+        <v>19297939.04415454</v>
       </c>
       <c r="I24" t="n">
-        <v>1373672663.619962</v>
+        <v>1500994192.873917</v>
       </c>
       <c r="J24" t="n">
-        <v>-0.8110095425798591</v>
+        <v>-0.3168705169290315</v>
       </c>
     </row>
     <row r="25">
@@ -1263,32 +1263,32 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>AT45</t>
+          <t>AT46</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D25" t="n">
         <v>610417.8060183238</v>
       </c>
       <c r="E25" t="n">
-        <v>25637547.8527696</v>
+        <v>27468801.27082457</v>
       </c>
       <c r="F25" t="n">
-        <v>4.828333565796324</v>
+        <v>3.759699809026542</v>
       </c>
       <c r="G25" t="n">
-        <v>458558.7279902952</v>
+        <v>459474.7391465366</v>
       </c>
       <c r="H25" t="n">
-        <v>19259466.5755924</v>
+        <v>20676363.26159415</v>
       </c>
       <c r="I25" t="n">
-        <v>1498001803.284273</v>
+        <v>1375461467.696546</v>
       </c>
       <c r="J25" t="n">
-        <v>-0.5521200614288333</v>
+        <v>-1.925763987349056</v>
       </c>
     </row>
     <row r="26">
@@ -1297,32 +1297,32 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>AT46</t>
+          <t>AT72</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>45</v>
+        <v>65.08528472924029</v>
       </c>
       <c r="D26" t="n">
-        <v>610417.8060183238</v>
+        <v>1118751.395250489</v>
       </c>
       <c r="E26" t="n">
-        <v>27468801.27082457</v>
+        <v>72814253.10111289</v>
       </c>
       <c r="F26" t="n">
-        <v>4.506444661409902</v>
+        <v>1.587888411702909</v>
       </c>
       <c r="G26" t="n">
-        <v>458558.7279902952</v>
+        <v>842108.4713362895</v>
       </c>
       <c r="H26" t="n">
-        <v>20635142.75956328</v>
+        <v>54808869.62982767</v>
       </c>
       <c r="I26" t="n">
-        <v>1372719340.780645</v>
+        <v>1125912787.639718</v>
       </c>
       <c r="J26" t="n">
-        <v>-0.7848221100116923</v>
+        <v>-0.7195512626524666</v>
       </c>
     </row>
     <row r="27">
@@ -1331,32 +1331,32 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>AT72</t>
+          <t>AT75</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>65.08528472924029</v>
+        <v>70</v>
       </c>
       <c r="D27" t="n">
         <v>1118751.395250489</v>
       </c>
       <c r="E27" t="n">
-        <v>72814253.10111289</v>
+        <v>78312597.6675342</v>
       </c>
       <c r="F27" t="n">
-        <v>2.388202366416432</v>
+        <v>1.476402419913499</v>
       </c>
       <c r="G27" t="n">
-        <v>840429.6396426423</v>
+        <v>842108.4713362895</v>
       </c>
       <c r="H27" t="n">
-        <v>54699602.39103416</v>
+        <v>58947592.99354025</v>
       </c>
       <c r="I27" t="n">
-        <v>1123668162.23039</v>
+        <v>13267197882.07699</v>
       </c>
       <c r="J27" t="n">
-        <v>-1.195175209322294</v>
+        <v>-0.9215612225492077</v>
       </c>
     </row>
     <row r="28">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>AT75</t>
+          <t>AT76</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -1378,19 +1378,19 @@
         <v>78312597.6675342</v>
       </c>
       <c r="F28" t="n">
-        <v>2.220526157275127</v>
+        <v>1.476402419913499</v>
       </c>
       <c r="G28" t="n">
-        <v>840429.6396426423</v>
+        <v>842108.4713362895</v>
       </c>
       <c r="H28" t="n">
-        <v>58830074.77498494</v>
+        <v>58947592.99354025</v>
       </c>
       <c r="I28" t="n">
-        <v>13240748329.49741</v>
+        <v>32987768536.4073</v>
       </c>
       <c r="J28" t="n">
-        <v>-0.9215824911147686</v>
+        <v>-0.5724967379994873</v>
       </c>
     </row>
     <row r="29">
@@ -1399,32 +1399,32 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>AT76</t>
+          <t>B190</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>70</v>
+        <v>17.08109334942567</v>
       </c>
       <c r="D29" t="n">
-        <v>1118751.395250489</v>
+        <v>1191751.053870659</v>
       </c>
       <c r="E29" t="n">
-        <v>78312597.6675342</v>
+        <v>20356411.00044115</v>
       </c>
       <c r="F29" t="n">
-        <v>2.220526157275127</v>
+        <v>2.967918644423394</v>
       </c>
       <c r="G29" t="n">
-        <v>840429.6396426423</v>
+        <v>897056.8997267976</v>
       </c>
       <c r="H29" t="n">
-        <v>58830074.77498494</v>
+        <v>15322712.64397981</v>
       </c>
       <c r="I29" t="n">
-        <v>32922003954.75698</v>
+        <v>5633988246.872105</v>
       </c>
       <c r="J29" t="n">
-        <v>0.451652430105666</v>
+        <v>0.996188660394359</v>
       </c>
     </row>
     <row r="30">
@@ -1433,32 +1433,32 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>B190</t>
+          <t>B38M</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>17.08109334942567</v>
+        <v>171.9250535865172</v>
       </c>
       <c r="D30" t="n">
-        <v>1191751.053870659</v>
+        <v>2879411.841229504</v>
       </c>
       <c r="E30" t="n">
-        <v>20356411.00044115</v>
+        <v>495043035.1010346</v>
       </c>
       <c r="F30" t="n">
-        <v>4.649774328792322</v>
+        <v>0.8763039646656254</v>
       </c>
       <c r="G30" t="n">
-        <v>895268.5225693081</v>
+        <v>2167395.825613678</v>
       </c>
       <c r="H30" t="n">
-        <v>15292165.20680875</v>
+        <v>372629643.4618254</v>
       </c>
       <c r="I30" t="n">
-        <v>5622756299.501387</v>
+        <v>518543180203.8316</v>
       </c>
       <c r="J30" t="n">
-        <v>0.3468514888100748</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -1467,29 +1467,29 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>B38M</t>
+          <t>B39M</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>171.9250535865172</v>
+        <v>178.0546134379522</v>
       </c>
       <c r="D31" t="n">
-        <v>2879411.841229504</v>
+        <v>3203937.581275163</v>
       </c>
       <c r="E31" t="n">
-        <v>495043035.1010346</v>
+        <v>570475867.5132767</v>
       </c>
       <c r="F31" t="n">
-        <v>1.440499062680862</v>
+        <v>0.7851654512067765</v>
       </c>
       <c r="G31" t="n">
-        <v>2163074.894369578</v>
+        <v>2411673.397931646</v>
       </c>
       <c r="H31" t="n">
-        <v>371886767.1261396</v>
+        <v>429409574.6073118</v>
       </c>
       <c r="I31" t="n">
-        <v>517509409905.7257</v>
+        <v>97906834720.49709</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1501,29 +1501,29 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>B39M</t>
+          <t>B3XM</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>178.0546134379522</v>
+        <v>190</v>
       </c>
       <c r="D32" t="n">
         <v>3203937.581275163</v>
       </c>
       <c r="E32" t="n">
-        <v>570475867.5132767</v>
+        <v>608748140.4422809</v>
       </c>
       <c r="F32" t="n">
-        <v>1.329917904959669</v>
+        <v>0.7358017415760942</v>
       </c>
       <c r="G32" t="n">
-        <v>2406865.473687933</v>
+        <v>2411673.397931646</v>
       </c>
       <c r="H32" t="n">
-        <v>428553501.5146586</v>
+        <v>458217945.6070126</v>
       </c>
       <c r="I32" t="n">
-        <v>97711647161.23572</v>
+        <v>458217945.6070126</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1535,32 +1535,32 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>B3XM</t>
+          <t>B461</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>190</v>
+        <v>80</v>
       </c>
       <c r="D33" t="n">
-        <v>3203937.581275163</v>
+        <v>1907125.147166258</v>
       </c>
       <c r="E33" t="n">
-        <v>608748140.4422809</v>
+        <v>152570011.7733006</v>
       </c>
       <c r="F33" t="n">
-        <v>1.246305360377922</v>
+        <v>2.922741166837872</v>
       </c>
       <c r="G33" t="n">
-        <v>2406865.473687933</v>
+        <v>1435534.515662068</v>
       </c>
       <c r="H33" t="n">
-        <v>457304440.0007072</v>
+        <v>114842761.2529654</v>
       </c>
       <c r="I33" t="n">
-        <v>457304440.0007072</v>
+        <v>8601528599.47703</v>
       </c>
       <c r="J33" t="n">
-        <v>0</v>
+        <v>-0.3302227925025578</v>
       </c>
     </row>
     <row r="34">
@@ -1569,32 +1569,32 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>B461</t>
+          <t>B462</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="D34" t="n">
         <v>1907125.147166258</v>
       </c>
       <c r="E34" t="n">
-        <v>152570011.7733006</v>
+        <v>171641263.2449632</v>
       </c>
       <c r="F34" t="n">
-        <v>4.362502110167918</v>
+        <v>2.623618271687993</v>
       </c>
       <c r="G34" t="n">
-        <v>1432672.626814906</v>
+        <v>1435534.515662068</v>
       </c>
       <c r="H34" t="n">
-        <v>114613810.1451925</v>
+        <v>129198106.4095861</v>
       </c>
       <c r="I34" t="n">
-        <v>8584380548.699557</v>
+        <v>2799583479.748453</v>
       </c>
       <c r="J34" t="n">
-        <v>-0.8306890205300059</v>
+        <v>0.3395529677816287</v>
       </c>
     </row>
     <row r="35">
@@ -1603,32 +1603,32 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>B462</t>
+          <t>B463</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="D35" t="n">
         <v>1907125.147166258</v>
       </c>
       <c r="E35" t="n">
-        <v>171641263.2449632</v>
+        <v>190712514.7166258</v>
       </c>
       <c r="F35" t="n">
-        <v>3.896658027792295</v>
+        <v>2.488394116576957</v>
       </c>
       <c r="G35" t="n">
-        <v>1432672.626814906</v>
+        <v>1435534.515662068</v>
       </c>
       <c r="H35" t="n">
-        <v>128940536.4133415</v>
+        <v>143553451.5662068</v>
       </c>
       <c r="I35" t="n">
-        <v>2794002216.010119</v>
+        <v>1231331150.888789</v>
       </c>
       <c r="J35" t="n">
-        <v>-0.4197088181238978</v>
+        <v>-0.6891582901811604</v>
       </c>
     </row>
     <row r="36">
@@ -1637,32 +1637,32 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>B463</t>
+          <t>B703</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="D36" t="n">
-        <v>1907125.147166258</v>
+        <v>2100973.964773551</v>
       </c>
       <c r="E36" t="n">
-        <v>190712514.7166258</v>
+        <v>273126615.4205617</v>
       </c>
       <c r="F36" t="n">
-        <v>3.730631705746964</v>
+        <v>3.08194565299555</v>
       </c>
       <c r="G36" t="n">
-        <v>1432672.626814906</v>
+        <v>1581448.730525751</v>
       </c>
       <c r="H36" t="n">
-        <v>143267262.6814906</v>
+        <v>205588334.9683477</v>
       </c>
       <c r="I36" t="n">
-        <v>1228876362.899058</v>
+        <v>8735143756.122335</v>
       </c>
       <c r="J36" t="n">
-        <v>-1.232574526988627</v>
+        <v>2.695567568467057</v>
       </c>
     </row>
     <row r="37">
@@ -1671,32 +1671,32 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>B703</t>
+          <t>B712</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>130</v>
+        <v>114.0912363814062</v>
       </c>
       <c r="D37" t="n">
-        <v>2100973.964773551</v>
+        <v>1907125.147166258</v>
       </c>
       <c r="E37" t="n">
-        <v>273126615.4205617</v>
+        <v>217586265.9742696</v>
       </c>
       <c r="F37" t="n">
-        <v>4.576585493413694</v>
+        <v>1.889656157541419</v>
       </c>
       <c r="G37" t="n">
-        <v>1578295.946364262</v>
+        <v>1435534.515662068</v>
       </c>
       <c r="H37" t="n">
-        <v>205178473.0273541</v>
+        <v>163781907.7600685</v>
       </c>
       <c r="I37" t="n">
-        <v>13547923760.93622</v>
+        <v>16227670556.04209</v>
       </c>
       <c r="J37" t="n">
-        <v>0.3110328188325694</v>
+        <v>-0.4231579231605213</v>
       </c>
     </row>
     <row r="38">
@@ -1705,32 +1705,32 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>B712</t>
+          <t>B722</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>114.0912363814062</v>
+        <v>32.27666887844529</v>
       </c>
       <c r="D38" t="n">
-        <v>1907125.147166258</v>
+        <v>2100973.964773551</v>
       </c>
       <c r="E38" t="n">
-        <v>217586265.9742696</v>
+        <v>67812440.98323029</v>
       </c>
       <c r="F38" t="n">
-        <v>2.835120319709717</v>
+        <v>12.48206279236391</v>
       </c>
       <c r="G38" t="n">
-        <v>1432672.626814906</v>
+        <v>1581448.730525751</v>
       </c>
       <c r="H38" t="n">
-        <v>163455391.3231096</v>
+        <v>51043897.02341732</v>
       </c>
       <c r="I38" t="n">
-        <v>16195318990.21552</v>
+        <v>397469700.4251648</v>
       </c>
       <c r="J38" t="n">
-        <v>-0.5126348695660322</v>
+        <v>0.1923850343935946</v>
       </c>
     </row>
     <row r="39">
@@ -1739,32 +1739,32 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>B721</t>
+          <t>B732</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>140</v>
+        <v>114.0266535528839</v>
       </c>
       <c r="D39" t="n">
-        <v>2100973.964773551</v>
+        <v>1853851.041269496</v>
       </c>
       <c r="E39" t="n">
-        <v>294136355.0682971</v>
+        <v>211388430.4214899</v>
       </c>
       <c r="F39" t="n">
-        <v>4.470813984061079</v>
+        <v>2.424017752474225</v>
       </c>
       <c r="G39" t="n">
-        <v>1578295.946364262</v>
+        <v>1395433.939189951</v>
       </c>
       <c r="H39" t="n">
-        <v>220961432.4909966</v>
+        <v>159116662.3399486</v>
       </c>
       <c r="I39" t="n">
-        <v>753624682.6129431</v>
+        <v>5491096158.939373</v>
       </c>
       <c r="J39" t="n">
-        <v>0.3677071642850549</v>
+        <v>0.3777079671711455</v>
       </c>
     </row>
     <row r="40">
@@ -1773,32 +1773,32 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>B722</t>
+          <t>B733</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>32.27666887844529</v>
+        <v>136.5032139948638</v>
       </c>
       <c r="D40" t="n">
-        <v>2100973.964773551</v>
+        <v>2112088.776021521</v>
       </c>
       <c r="E40" t="n">
-        <v>67812440.98323029</v>
+        <v>288306906.1694157</v>
       </c>
       <c r="F40" t="n">
-        <v>19.39214855553273</v>
+        <v>1.645469940597836</v>
       </c>
       <c r="G40" t="n">
-        <v>1578295.946364262</v>
+        <v>1589815.090334513</v>
       </c>
       <c r="H40" t="n">
-        <v>50942135.65299173</v>
+        <v>217014869.4881957</v>
       </c>
       <c r="I40" t="n">
-        <v>558441596.4248008</v>
+        <v>35902777856.87491</v>
       </c>
       <c r="J40" t="n">
-        <v>-0.8949876654191289</v>
+        <v>-0.5500089086283718</v>
       </c>
     </row>
     <row r="41">
@@ -1807,32 +1807,32 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>B732</t>
+          <t>B734</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>114.0266535528839</v>
+        <v>139.7808911299119</v>
       </c>
       <c r="D41" t="n">
-        <v>1853851.041269496</v>
+        <v>2311340.421146744</v>
       </c>
       <c r="E41" t="n">
-        <v>211388430.4214899</v>
+        <v>323081223.7724777</v>
       </c>
       <c r="F41" t="n">
-        <v>3.583800007014426</v>
+        <v>1.705966933028853</v>
       </c>
       <c r="G41" t="n">
-        <v>1392651.995054197</v>
+        <v>1739796.130805147</v>
       </c>
       <c r="H41" t="n">
-        <v>158799446.5597775</v>
+        <v>243190253.5483162</v>
       </c>
       <c r="I41" t="n">
-        <v>6765166915.820084</v>
+        <v>21902636341.22357</v>
       </c>
       <c r="J41" t="n">
-        <v>-0.456081748729347</v>
+        <v>-0.08805658987431857</v>
       </c>
     </row>
     <row r="42">
@@ -1841,32 +1841,32 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>B733</t>
+          <t>B735</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>136.5032139948638</v>
+        <v>117.7505572169622</v>
       </c>
       <c r="D42" t="n">
-        <v>2112088.776021521</v>
+        <v>2366481.28167164</v>
       </c>
       <c r="E42" t="n">
-        <v>288306906.1694157</v>
+        <v>278654489.5603465</v>
       </c>
       <c r="F42" t="n">
-        <v>2.61867102769283</v>
+        <v>1.747985551995309</v>
       </c>
       <c r="G42" t="n">
-        <v>1586645.626955932</v>
+        <v>1781301.854026516</v>
       </c>
       <c r="H42" t="n">
-        <v>216582227.5503806</v>
+        <v>209749285.8832301</v>
       </c>
       <c r="I42" t="n">
-        <v>35831201897.94832</v>
+        <v>22141012746.7139</v>
       </c>
       <c r="J42" t="n">
-        <v>-1.089976687695952</v>
+        <v>-0.5201939056659951</v>
       </c>
     </row>
     <row r="43">
@@ -1875,32 +1875,32 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>B734</t>
+          <t>B736</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>139.7808911299119</v>
+        <v>114.7201522807672</v>
       </c>
       <c r="D43" t="n">
-        <v>2311340.421146744</v>
+        <v>2797758.035958845</v>
       </c>
       <c r="E43" t="n">
-        <v>323081223.7724777</v>
+        <v>320959227.9299389</v>
       </c>
       <c r="F43" t="n">
-        <v>2.68105396851786</v>
+        <v>1.477731589399572</v>
       </c>
       <c r="G43" t="n">
-        <v>1736327.664468209</v>
+        <v>2105933.233095642</v>
       </c>
       <c r="H43" t="n">
-        <v>242705428.2328848</v>
+        <v>241592981.1938605</v>
       </c>
       <c r="I43" t="n">
-        <v>21858971134.99933</v>
+        <v>4266495305.40716</v>
       </c>
       <c r="J43" t="n">
-        <v>-0.6493189872782845</v>
+        <v>-1.914544047609871</v>
       </c>
     </row>
     <row r="44">
@@ -1909,32 +1909,32 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>B735</t>
+          <t>B737</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>117.7505572169622</v>
+        <v>138.6026311800802</v>
       </c>
       <c r="D44" t="n">
-        <v>2366481.28167164</v>
+        <v>2465474.348708929</v>
       </c>
       <c r="E44" t="n">
-        <v>278654489.5603465</v>
+        <v>341721231.8380522</v>
       </c>
       <c r="F44" t="n">
-        <v>2.700486994246298</v>
+        <v>1.436323561650747</v>
       </c>
       <c r="G44" t="n">
-        <v>1777750.641670527</v>
+        <v>1855816.085436255</v>
       </c>
       <c r="H44" t="n">
-        <v>209331128.6495167</v>
+        <v>257220992.4277814</v>
       </c>
       <c r="I44" t="n">
-        <v>22096872312.08599</v>
+        <v>192185680562.2291</v>
       </c>
       <c r="J44" t="n">
-        <v>-0.9787600482465307</v>
+        <v>-1.073763731338126</v>
       </c>
     </row>
     <row r="45">
@@ -1943,32 +1943,32 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>B736</t>
+          <t>B738</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>114.7201522807672</v>
+        <v>166.1301280616927</v>
       </c>
       <c r="D45" t="n">
-        <v>2797758.035958845</v>
+        <v>2896741.750226228</v>
       </c>
       <c r="E45" t="n">
-        <v>320959227.9299389</v>
+        <v>481236077.9267349</v>
       </c>
       <c r="F45" t="n">
-        <v>2.376611123076421</v>
+        <v>1.158904218673777</v>
       </c>
       <c r="G45" t="n">
-        <v>2101734.833985827</v>
+        <v>2180440.424472356</v>
       </c>
       <c r="H45" t="n">
-        <v>241111340.2086471</v>
+        <v>362236846.9484839</v>
       </c>
       <c r="I45" t="n">
-        <v>4257989598.858277</v>
+        <v>1588965285738.62</v>
       </c>
       <c r="J45" t="n">
-        <v>-1.945113458916124</v>
+        <v>0.4119103387843562</v>
       </c>
     </row>
     <row r="46">
@@ -1977,32 +1977,32 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>B737</t>
+          <t>B739</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>138.6026311800802</v>
+        <v>178.5701700968943</v>
       </c>
       <c r="D46" t="n">
-        <v>2465474.348708929</v>
+        <v>2957093.83964751</v>
       </c>
       <c r="E46" t="n">
-        <v>341721231.8380522</v>
+        <v>528048749.938334</v>
       </c>
       <c r="F46" t="n">
-        <v>2.218301133604561</v>
+        <v>1.085212054990146</v>
       </c>
       <c r="G46" t="n">
-        <v>1852116.32113289</v>
+        <v>2225868.752857259</v>
       </c>
       <c r="H46" t="n">
-        <v>256708195.360589</v>
+        <v>397473761.8110825</v>
       </c>
       <c r="I46" t="n">
-        <v>191802538220.6243</v>
+        <v>195705401564.8515</v>
       </c>
       <c r="J46" t="n">
-        <v>-1.103680459505332</v>
+        <v>0.14975135519457</v>
       </c>
     </row>
     <row r="47">
@@ -2011,32 +2011,32 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>B738</t>
+          <t>B744</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>166.1301280616927</v>
+        <v>335.0242252924581</v>
       </c>
       <c r="D47" t="n">
-        <v>2896741.750226228</v>
+        <v>4777422.14567662</v>
       </c>
       <c r="E47" t="n">
-        <v>481236077.9267349</v>
+        <v>1600552153.250343</v>
       </c>
       <c r="F47" t="n">
-        <v>1.924626598245413</v>
+        <v>1.544157495477784</v>
       </c>
       <c r="G47" t="n">
-        <v>2176093.487450211</v>
+        <v>3596069.401212322</v>
       </c>
       <c r="H47" t="n">
-        <v>361514689.7443188</v>
+        <v>1204770365.239072</v>
       </c>
       <c r="I47" t="n">
-        <v>1585797516534.766</v>
+        <v>55165222744.45591</v>
       </c>
       <c r="J47" t="n">
-        <v>0.7265913743825997</v>
+        <v>-1.099696200748784</v>
       </c>
     </row>
     <row r="48">
@@ -2045,32 +2045,32 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>B739</t>
+          <t>B748</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>178.5701700968943</v>
+        <v>365.3586232234018</v>
       </c>
       <c r="D48" t="n">
-        <v>2957093.83964751</v>
+        <v>4853176.852122201</v>
       </c>
       <c r="E48" t="n">
-        <v>528048749.938334</v>
+        <v>1773150012.951051</v>
       </c>
       <c r="F48" t="n">
-        <v>1.824936982877567</v>
+        <v>1.241535095777449</v>
       </c>
       <c r="G48" t="n">
-        <v>2221431.249690634</v>
+        <v>3653091.6139329</v>
       </c>
       <c r="H48" t="n">
-        <v>396681356.1158129</v>
+        <v>1334688522.57548</v>
       </c>
       <c r="I48" t="n">
-        <v>195315242289.7125</v>
+        <v>55547846882.41961</v>
       </c>
       <c r="J48" t="n">
-        <v>0.661230989153156</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -2079,32 +2079,32 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>B744</t>
+          <t>B752</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>335.0242252924581</v>
+        <v>179.0970265826863</v>
       </c>
       <c r="D49" t="n">
-        <v>4777422.14567662</v>
+        <v>3279932.55416027</v>
       </c>
       <c r="E49" t="n">
-        <v>1600552153.250343</v>
+        <v>587426167.8418602</v>
       </c>
       <c r="F49" t="n">
-        <v>3.122706025070125</v>
+        <v>1.324212276281809</v>
       </c>
       <c r="G49" t="n">
-        <v>3588900.259125756</v>
+        <v>2468876.464419167</v>
       </c>
       <c r="H49" t="n">
-        <v>1202368528.965509</v>
+        <v>442168433.7774481</v>
       </c>
       <c r="I49" t="n">
-        <v>55055245078.29665</v>
+        <v>81086857502.55305</v>
       </c>
       <c r="J49" t="n">
-        <v>-1.478769653878538</v>
+        <v>-0.1898163249432536</v>
       </c>
     </row>
     <row r="50">
@@ -2113,32 +2113,32 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>B748</t>
+          <t>B753</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>365.3586232234018</v>
+        <v>228.7978272657155</v>
       </c>
       <c r="D50" t="n">
-        <v>4853176.852122201</v>
+        <v>3188105.689859158</v>
       </c>
       <c r="E50" t="n">
-        <v>1773150012.951051</v>
+        <v>729431654.9332407</v>
       </c>
       <c r="F50" t="n">
-        <v>2.444968439264291</v>
+        <v>1.163961944685927</v>
       </c>
       <c r="G50" t="n">
-        <v>3645808.792075597</v>
+        <v>2399756.389438701</v>
       </c>
       <c r="H50" t="n">
-        <v>1332027680.808514</v>
+        <v>549059047.8705932</v>
       </c>
       <c r="I50" t="n">
-        <v>55437106414.85004</v>
+        <v>24101455087.35828</v>
       </c>
       <c r="J50" t="n">
-        <v>0</v>
+        <v>2.015553782672774</v>
       </c>
     </row>
     <row r="51">
@@ -2147,32 +2147,32 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>B752</t>
+          <t>B762</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>179.0970265826863</v>
+        <v>193.8227458894083</v>
       </c>
       <c r="D51" t="n">
-        <v>3279932.55416027</v>
+        <v>4131668.673472243</v>
       </c>
       <c r="E51" t="n">
-        <v>587426167.8418602</v>
+        <v>800811367.3976392</v>
       </c>
       <c r="F51" t="n">
-        <v>2.293996476969463</v>
+        <v>1.383383760653715</v>
       </c>
       <c r="G51" t="n">
-        <v>2463954.499853735</v>
+        <v>3109996.738736336</v>
       </c>
       <c r="H51" t="n">
-        <v>441286924.5588341</v>
+        <v>602788107.6089813</v>
       </c>
       <c r="I51" t="n">
-        <v>80925202334.66533</v>
+        <v>17346000352.13657</v>
       </c>
       <c r="J51" t="n">
-        <v>-0.7356576123492866</v>
+        <v>-0.124758191718537</v>
       </c>
     </row>
     <row r="52">
@@ -2181,32 +2181,32 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>B753</t>
+          <t>B763</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>228.7978272657155</v>
+        <v>223.0260557846611</v>
       </c>
       <c r="D52" t="n">
-        <v>3188105.689859158</v>
+        <v>4394802.833309786</v>
       </c>
       <c r="E52" t="n">
-        <v>729431654.9332407</v>
+        <v>980155541.8643353</v>
       </c>
       <c r="F52" t="n">
-        <v>2.02571150843473</v>
+        <v>1.174247232680542</v>
       </c>
       <c r="G52" t="n">
-        <v>2394972.223003195</v>
+        <v>3308063.535379337</v>
       </c>
       <c r="H52" t="n">
-        <v>547964440.9848719</v>
+        <v>737784362.5807153</v>
       </c>
       <c r="I52" t="n">
-        <v>24053406304.99718</v>
+        <v>135710185718.0529</v>
       </c>
       <c r="J52" t="n">
-        <v>1.48815789571841</v>
+        <v>-0.1893430030811168</v>
       </c>
     </row>
     <row r="53">
@@ -2215,32 +2215,32 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>B762</t>
+          <t>B764</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>193.8227458894083</v>
+        <v>239.0919791752058</v>
       </c>
       <c r="D53" t="n">
-        <v>4131668.673472243</v>
+        <v>4676487.462829613</v>
       </c>
       <c r="E53" t="n">
-        <v>800811367.3976392</v>
+        <v>1118110643.075969</v>
       </c>
       <c r="F53" t="n">
-        <v>2.645244752305779</v>
+        <v>1.224601924257454</v>
       </c>
       <c r="G53" t="n">
-        <v>3103796.633560045</v>
+        <v>3520093.673416178</v>
       </c>
       <c r="H53" t="n">
-        <v>601586386.1989095</v>
+        <v>841626163.2591947</v>
       </c>
       <c r="I53" t="n">
-        <v>17311419278.39084</v>
+        <v>25406801830.26596</v>
       </c>
       <c r="J53" t="n">
-        <v>-0.8572520265977058</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
@@ -2249,32 +2249,32 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>B763</t>
+          <t>B772</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>223.0260557846611</v>
+        <v>283.4055860622861</v>
       </c>
       <c r="D54" t="n">
-        <v>4394802.833309786</v>
+        <v>4711405.94823829</v>
       </c>
       <c r="E54" t="n">
-        <v>980155541.8643353</v>
+        <v>1335238763.937814</v>
       </c>
       <c r="F54" t="n">
-        <v>2.207241243771939</v>
+        <v>1.242461676533537</v>
       </c>
       <c r="G54" t="n">
-        <v>3301468.563238775</v>
+        <v>3546377.575714504</v>
       </c>
       <c r="H54" t="n">
-        <v>736313511.9561962</v>
+        <v>1005063215.243519</v>
       </c>
       <c r="I54" t="n">
-        <v>135439633207.6706</v>
+        <v>295670248955.9517</v>
       </c>
       <c r="J54" t="n">
-        <v>-0.6798838772308782</v>
+        <v>-0.505904260809742</v>
       </c>
     </row>
     <row r="55">
@@ -2283,32 +2283,32 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>B764</t>
+          <t>B773</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>239.0919791752058</v>
+        <v>350</v>
       </c>
       <c r="D55" t="n">
-        <v>4676487.462829613</v>
+        <v>4838623.285985882</v>
       </c>
       <c r="E55" t="n">
-        <v>1118110643.075969</v>
+        <v>1693518150.095059</v>
       </c>
       <c r="F55" t="n">
-        <v>2.335688945862603</v>
+        <v>1.249185074303995</v>
       </c>
       <c r="G55" t="n">
-        <v>3513075.996923552</v>
+        <v>3642136.828639602</v>
       </c>
       <c r="H55" t="n">
-        <v>839948293.0973613</v>
+        <v>1274747890.023861</v>
       </c>
       <c r="I55" t="n">
-        <v>25356150702.05777</v>
+        <v>52411052553.07043</v>
       </c>
       <c r="J55" t="n">
-        <v>0</v>
+        <v>0.2553647868288557</v>
       </c>
     </row>
     <row r="56">
@@ -2317,32 +2317,32 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>B772</t>
+          <t>B77L</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>283.4055860622861</v>
+        <v>350</v>
       </c>
       <c r="D56" t="n">
-        <v>4711405.94823829</v>
+        <v>4838623.285985882</v>
       </c>
       <c r="E56" t="n">
-        <v>1335238763.937814</v>
+        <v>1693518150.095059</v>
       </c>
       <c r="F56" t="n">
-        <v>2.461448190938961</v>
+        <v>0.9757883476193243</v>
       </c>
       <c r="G56" t="n">
-        <v>3539307.499501755</v>
+        <v>3642136.828639602</v>
       </c>
       <c r="H56" t="n">
-        <v>1003059516.15094</v>
+        <v>1274747890.023861</v>
       </c>
       <c r="I56" t="n">
-        <v>295080799257.1164</v>
+        <v>60754106082.89317</v>
       </c>
       <c r="J56" t="n">
-        <v>-0.6857256757042275</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
@@ -2351,32 +2351,32 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>B773</t>
+          <t>B77W</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>350</v>
+        <v>317.4522639539198</v>
       </c>
       <c r="D57" t="n">
         <v>4838623.285985882</v>
       </c>
       <c r="E57" t="n">
-        <v>1693518150.095059</v>
+        <v>1536031916.556373</v>
       </c>
       <c r="F57" t="n">
-        <v>2.358051517262374</v>
+        <v>1.251541412066441</v>
       </c>
       <c r="G57" t="n">
-        <v>3634875.846297485</v>
+        <v>3642136.828639602</v>
       </c>
       <c r="H57" t="n">
-        <v>1272206546.20412</v>
+        <v>1156204581.881591</v>
       </c>
       <c r="I57" t="n">
-        <v>52306565614.4889</v>
+        <v>833362741764.8564</v>
       </c>
       <c r="J57" t="n">
-        <v>0.1328022093787508</v>
+        <v>-0.2003866629378316</v>
       </c>
     </row>
     <row r="58">
@@ -2385,32 +2385,32 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>B77L</t>
+          <t>B788</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>350</v>
+        <v>241.91300690316</v>
       </c>
       <c r="D58" t="n">
-        <v>4838623.285985882</v>
+        <v>4708923.555571395</v>
       </c>
       <c r="E58" t="n">
-        <v>1693518150.095059</v>
+        <v>1139149856.605396</v>
       </c>
       <c r="F58" t="n">
-        <v>1.961725890743383</v>
+        <v>0.9949389212208551</v>
       </c>
       <c r="G58" t="n">
-        <v>3634875.846297485</v>
+        <v>3544509.024843551</v>
       </c>
       <c r="H58" t="n">
-        <v>1272206546.20412</v>
+        <v>857462836.1952912</v>
       </c>
       <c r="I58" t="n">
-        <v>60632986390.73604</v>
+        <v>308206341899.0812</v>
       </c>
       <c r="J58" t="n">
-        <v>0</v>
+        <v>-0.4374306655313249</v>
       </c>
     </row>
     <row r="59">
@@ -2419,32 +2419,32 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>B77W</t>
+          <t>B789</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>317.4522639539198</v>
+        <v>273.4925758295888</v>
       </c>
       <c r="D59" t="n">
-        <v>4838623.285985882</v>
+        <v>4776565.096988944</v>
       </c>
       <c r="E59" t="n">
-        <v>1536031916.556373</v>
+        <v>1306355091.993216</v>
       </c>
       <c r="F59" t="n">
-        <v>2.527768814084611</v>
+        <v>0.8812055291279901</v>
       </c>
       <c r="G59" t="n">
-        <v>3634875.846297485</v>
+        <v>3595424.282052423</v>
       </c>
       <c r="H59" t="n">
-        <v>1153899566.598557</v>
+        <v>983321848.098767</v>
       </c>
       <c r="I59" t="n">
-        <v>831701345601.7712</v>
+        <v>595653212492.6771</v>
       </c>
       <c r="J59" t="n">
-        <v>0.4776092282624212</v>
+        <v>0.7240994360207816</v>
       </c>
     </row>
     <row r="60">
@@ -2453,32 +2453,32 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>B788</t>
+          <t>B78X</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>241.91300690316</v>
+        <v>311.2551813304133</v>
       </c>
       <c r="D60" t="n">
-        <v>4708923.555571395</v>
+        <v>4703115.032635386</v>
       </c>
       <c r="E60" t="n">
-        <v>1139149856.605396</v>
+        <v>1463868922.30072</v>
       </c>
       <c r="F60" t="n">
-        <v>1.915855325393217</v>
+        <v>0.8828858610008796</v>
       </c>
       <c r="G60" t="n">
-        <v>3537442.673783238</v>
+        <v>3540136.823484849</v>
       </c>
       <c r="H60" t="n">
-        <v>855753393.9624574</v>
+        <v>1101885928.92825</v>
       </c>
       <c r="I60" t="n">
-        <v>307591900182.1582</v>
+        <v>124496634194.9239</v>
       </c>
       <c r="J60" t="n">
-        <v>0.4890111181139369</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61">
@@ -2487,32 +2487,32 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>B789</t>
+          <t>BCS1</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>273.4925758295888</v>
+        <v>110</v>
       </c>
       <c r="D61" t="n">
-        <v>4776565.096988944</v>
+        <v>2654083.763084724</v>
       </c>
       <c r="E61" t="n">
-        <v>1306355091.993216</v>
+        <v>291949213.9393196</v>
       </c>
       <c r="F61" t="n">
-        <v>1.723861029760471</v>
+        <v>1.559350380561198</v>
       </c>
       <c r="G61" t="n">
-        <v>3588256.426078666</v>
+        <v>1997786.487702498</v>
       </c>
       <c r="H61" t="n">
-        <v>981361492.7053291</v>
+        <v>219756513.6472748</v>
       </c>
       <c r="I61" t="n">
-        <v>594465715245.4773</v>
+        <v>14700678736.23966</v>
       </c>
       <c r="J61" t="n">
-        <v>0.8456938716404536</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
@@ -2521,29 +2521,29 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>B78X</t>
+          <t>BCS3</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>311.2551813304133</v>
+        <v>140</v>
       </c>
       <c r="D62" t="n">
-        <v>4703115.032635386</v>
+        <v>2876842.467941348</v>
       </c>
       <c r="E62" t="n">
-        <v>1463868922.30072</v>
+        <v>402757945.5117888</v>
       </c>
       <c r="F62" t="n">
-        <v>1.630034360830604</v>
+        <v>1.260115242506681</v>
       </c>
       <c r="G62" t="n">
-        <v>3533079.188867205</v>
+        <v>2165461.802540128</v>
       </c>
       <c r="H62" t="n">
-        <v>1099689203.585572</v>
+        <v>303164652.355618</v>
       </c>
       <c r="I62" t="n">
-        <v>124248437077.3873</v>
+        <v>93906693290.05441</v>
       </c>
       <c r="J62" t="n">
         <v>0</v>
@@ -2555,29 +2555,29 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>BCS1</t>
+          <t>C919</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>110</v>
+        <v>150</v>
       </c>
       <c r="D63" t="n">
-        <v>2654083.763084724</v>
+        <v>2876842.467941348</v>
       </c>
       <c r="E63" t="n">
-        <v>291949213.9393196</v>
+        <v>431526370.1912023</v>
       </c>
       <c r="F63" t="n">
-        <v>2.465267946452722</v>
+        <v>1.186044863978063</v>
       </c>
       <c r="G63" t="n">
-        <v>1993803.690489483</v>
+        <v>2165461.802540128</v>
       </c>
       <c r="H63" t="n">
-        <v>219318405.9538431</v>
+        <v>324819270.3810193</v>
       </c>
       <c r="I63" t="n">
-        <v>14671371389.00284</v>
+        <v>4830969390.167755</v>
       </c>
       <c r="J63" t="n">
         <v>0</v>
@@ -2589,32 +2589,32 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>BCS3</t>
+          <t>CRJ2</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>140</v>
+        <v>49.99590676873404</v>
       </c>
       <c r="D64" t="n">
-        <v>2876842.467941348</v>
+        <v>1698679.465539658</v>
       </c>
       <c r="E64" t="n">
-        <v>402757945.5117888</v>
+        <v>84927020.18908368</v>
       </c>
       <c r="F64" t="n">
-        <v>2.089083076234863</v>
+        <v>2.426303926504643</v>
       </c>
       <c r="G64" t="n">
-        <v>2161144.726974176</v>
+        <v>1278632.924248254</v>
       </c>
       <c r="H64" t="n">
-        <v>302560261.7763847</v>
+        <v>63926412.47214945</v>
       </c>
       <c r="I64" t="n">
-        <v>93719480432.91408</v>
+        <v>28877362820.42909</v>
       </c>
       <c r="J64" t="n">
-        <v>0</v>
+        <v>-1.37249742165644</v>
       </c>
     </row>
     <row r="65">
@@ -2623,32 +2623,32 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>C919</t>
+          <t>CRJ7</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>150</v>
+        <v>65.78763158003113</v>
       </c>
       <c r="D65" t="n">
-        <v>2876842.467941348</v>
+        <v>2038513.358160724</v>
       </c>
       <c r="E65" t="n">
-        <v>431526370.1912023</v>
+        <v>134108965.7776498</v>
       </c>
       <c r="F65" t="n">
-        <v>1.95954532000242</v>
+        <v>2.315458107421362</v>
       </c>
       <c r="G65" t="n">
-        <v>2161144.726974176</v>
+        <v>1534433.275459714</v>
       </c>
       <c r="H65" t="n">
-        <v>324171709.0461265</v>
+        <v>100946731.0100842</v>
       </c>
       <c r="I65" t="n">
-        <v>4821338345.237898</v>
+        <v>26504550907.88561</v>
       </c>
       <c r="J65" t="n">
-        <v>0</v>
+        <v>-0.1116831792069889</v>
       </c>
     </row>
     <row r="66">
@@ -2657,32 +2657,32 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>CRJ2</t>
+          <t>CRJ9</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>49.99590676873404</v>
+        <v>76.38671489837947</v>
       </c>
       <c r="D66" t="n">
-        <v>1698679.465539658</v>
+        <v>2070367.994738347</v>
       </c>
       <c r="E66" t="n">
-        <v>84927020.18908368</v>
+        <v>158148609.7488077</v>
       </c>
       <c r="F66" t="n">
-        <v>3.541539822162323</v>
+        <v>2.012412678660564</v>
       </c>
       <c r="G66" t="n">
-        <v>1276083.835204698</v>
+        <v>1558410.952204733</v>
       </c>
       <c r="H66" t="n">
-        <v>63798968.45398264</v>
+        <v>119041893.100575</v>
       </c>
       <c r="I66" t="n">
-        <v>28819792764.3353</v>
+        <v>49395339585.50361</v>
       </c>
       <c r="J66" t="n">
-        <v>-1.479183307205579</v>
+        <v>0.01005374338884722</v>
       </c>
     </row>
     <row r="67">
@@ -2691,32 +2691,32 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>CRJ7</t>
+          <t>CRJX</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>65.78763158003113</v>
+        <v>100</v>
       </c>
       <c r="D67" t="n">
-        <v>2038513.358160724</v>
+        <v>2070367.994738347</v>
       </c>
       <c r="E67" t="n">
-        <v>134108965.7776498</v>
+        <v>207036799.4738347</v>
       </c>
       <c r="F67" t="n">
-        <v>3.515124994178294</v>
+        <v>1.556991741800394</v>
       </c>
       <c r="G67" t="n">
-        <v>1531374.221546457</v>
+        <v>1558410.952204733</v>
       </c>
       <c r="H67" t="n">
-        <v>100745483.0982553</v>
+        <v>155841095.2204733</v>
       </c>
       <c r="I67" t="n">
-        <v>26451711301.58236</v>
+        <v>6448381807.709344</v>
       </c>
       <c r="J67" t="n">
-        <v>0.06247312108029204</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68">
@@ -2725,32 +2725,32 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>CRJ9</t>
+          <t>CVLT</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>76.38671489837947</v>
+        <v>8.991285951408372</v>
       </c>
       <c r="D68" t="n">
-        <v>2070367.994738347</v>
+        <v>1262967.042595795</v>
       </c>
       <c r="E68" t="n">
-        <v>158148609.7488077</v>
+        <v>11355697.82718335</v>
       </c>
       <c r="F68" t="n">
-        <v>3.084978462279732</v>
+        <v>10.28864736013324</v>
       </c>
       <c r="G68" t="n">
-        <v>1555304.096274242</v>
+        <v>950662.7210510238</v>
       </c>
       <c r="H68" t="n">
-        <v>118804570.5823822</v>
+        <v>8547680.368313728</v>
       </c>
       <c r="I68" t="n">
-        <v>49296864787.49686</v>
+        <v>21860357.98181826</v>
       </c>
       <c r="J68" t="n">
-        <v>0.5422450444784533</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69">
@@ -2759,32 +2759,32 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>CRJX</t>
+          <t>D228</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>100</v>
+        <v>19</v>
       </c>
       <c r="D69" t="n">
-        <v>2070367.994738347</v>
+        <v>758575.0104772012</v>
       </c>
       <c r="E69" t="n">
-        <v>207036799.4738347</v>
+        <v>14412925.19906682</v>
       </c>
       <c r="F69" t="n">
-        <v>2.35879533342805</v>
+        <v>2.211827734792698</v>
       </c>
       <c r="G69" t="n">
-        <v>1555304.096274242</v>
+        <v>570995.884500182</v>
       </c>
       <c r="H69" t="n">
-        <v>155530409.6274242</v>
+        <v>10848921.80550346</v>
       </c>
       <c r="I69" t="n">
-        <v>6435526281.230265</v>
+        <v>1515907198.7075</v>
       </c>
       <c r="J69" t="n">
-        <v>0</v>
+        <v>0.8416986725011051</v>
       </c>
     </row>
     <row r="70">
@@ -2793,32 +2793,32 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>D328</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>8.991285951408372</v>
+        <v>30</v>
       </c>
       <c r="D70" t="n">
-        <v>1262967.042595795</v>
+        <v>975824.3201168067</v>
       </c>
       <c r="E70" t="n">
-        <v>11355697.82718335</v>
+        <v>29274729.6035042</v>
       </c>
       <c r="F70" t="n">
-        <v>16.1191084521</v>
+        <v>2.569399862184858</v>
       </c>
       <c r="G70" t="n">
-        <v>948767.4750579075</v>
+        <v>734524.1579094057</v>
       </c>
       <c r="H70" t="n">
-        <v>8530639.669641359</v>
+        <v>22035724.73728217</v>
       </c>
       <c r="I70" t="n">
-        <v>68807572.7087936</v>
+        <v>2311091551.744297</v>
       </c>
       <c r="J70" t="n">
-        <v>1.362271848243459</v>
+        <v>-0.5719368943839582</v>
       </c>
     </row>
     <row r="71">
@@ -2827,32 +2827,32 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>D228</t>
+          <t>DH8A</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>19</v>
+        <v>36.29959255529862</v>
       </c>
       <c r="D71" t="n">
-        <v>758575.0104772012</v>
+        <v>1101395.512311833</v>
       </c>
       <c r="E71" t="n">
-        <v>14412925.19906682</v>
+        <v>39980208.33915395</v>
       </c>
       <c r="F71" t="n">
-        <v>3.706261078993328</v>
+        <v>2.118769808888522</v>
       </c>
       <c r="G71" t="n">
-        <v>569857.5442263692</v>
+        <v>829044.321327439</v>
       </c>
       <c r="H71" t="n">
-        <v>10827293.34030101</v>
+        <v>30093971.07447013</v>
       </c>
       <c r="I71" t="n">
-        <v>1512885078.474248</v>
+        <v>3929084634.577616</v>
       </c>
       <c r="J71" t="n">
-        <v>0.05867192930219328</v>
+        <v>0.9510423547929142</v>
       </c>
     </row>
     <row r="72">
@@ -2861,32 +2861,32 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>D328</t>
+          <t>DH8B</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="D72" t="n">
-        <v>975824.3201168067</v>
+        <v>1011409.017644414</v>
       </c>
       <c r="E72" t="n">
-        <v>29274729.6035042</v>
+        <v>37422133.65284332</v>
       </c>
       <c r="F72" t="n">
-        <v>3.754906724273647</v>
+        <v>2.374455858833616</v>
       </c>
       <c r="G72" t="n">
-        <v>733059.8068453545</v>
+        <v>761309.5325379024</v>
       </c>
       <c r="H72" t="n">
-        <v>21991794.20536063</v>
+        <v>28168452.70390239</v>
       </c>
       <c r="I72" t="n">
-        <v>2306484147.976191</v>
+        <v>1852972098.445735</v>
       </c>
       <c r="J72" t="n">
-        <v>-0.8513581929928902</v>
+        <v>0.4298525439995274</v>
       </c>
     </row>
     <row r="73">
@@ -2895,32 +2895,32 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>DH8A</t>
+          <t>DH8C</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>36.29959255529862</v>
+        <v>50</v>
       </c>
       <c r="D73" t="n">
-        <v>1101395.512311833</v>
+        <v>1042789.688643109</v>
       </c>
       <c r="E73" t="n">
-        <v>39980208.33915395</v>
+        <v>52139484.43215544</v>
       </c>
       <c r="F73" t="n">
-        <v>3.469101887257184</v>
+        <v>1.800774401633875</v>
       </c>
       <c r="G73" t="n">
-        <v>827391.5343891077</v>
+        <v>784930.4450984639</v>
       </c>
       <c r="H73" t="n">
-        <v>30033975.58202798</v>
+        <v>39246522.25492319</v>
       </c>
       <c r="I73" t="n">
-        <v>3921251591.643035</v>
+        <v>6292838420.812389</v>
       </c>
       <c r="J73" t="n">
-        <v>0.2238993874414584</v>
+        <v>0.5537224434725666</v>
       </c>
     </row>
     <row r="74">
@@ -2929,32 +2929,32 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>DH8B</t>
+          <t>DH8D</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>37</v>
+        <v>75.40687030072012</v>
       </c>
       <c r="D74" t="n">
-        <v>1011409.017644414</v>
+        <v>1446839.618250487</v>
       </c>
       <c r="E74" t="n">
-        <v>37422133.65284332</v>
+        <v>109101647.4393578</v>
       </c>
       <c r="F74" t="n">
-        <v>3.614570302941415</v>
+        <v>1.662943479721646</v>
       </c>
       <c r="G74" t="n">
-        <v>759791.7820159628</v>
+        <v>1089067.60194109</v>
       </c>
       <c r="H74" t="n">
-        <v>28112295.93459062</v>
+        <v>82123179.40828799</v>
       </c>
       <c r="I74" t="n">
-        <v>1849278003.929173</v>
+        <v>38217217850.79016</v>
       </c>
       <c r="J74" t="n">
-        <v>0.1503936380649345</v>
+        <v>-1.299301372651262</v>
       </c>
     </row>
     <row r="75">
@@ -2963,32 +2963,32 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>DH8C</t>
+          <t>DHC6</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>50</v>
+        <v>15.9328331054753</v>
       </c>
       <c r="D75" t="n">
-        <v>1042789.688643109</v>
+        <v>610417.8060183238</v>
       </c>
       <c r="E75" t="n">
-        <v>52139484.43215544</v>
+        <v>9725685.027900351</v>
       </c>
       <c r="F75" t="n">
-        <v>2.771002035709643</v>
+        <v>3.208873931952691</v>
       </c>
       <c r="G75" t="n">
-        <v>783365.6038061671</v>
+        <v>459474.7391465366</v>
       </c>
       <c r="H75" t="n">
-        <v>39168280.19030835</v>
+        <v>7320734.335003569</v>
       </c>
       <c r="I75" t="n">
-        <v>6280292986.413545</v>
+        <v>1204156694.827935</v>
       </c>
       <c r="J75" t="n">
-        <v>0.0748611213578271</v>
+        <v>2.360621738565051</v>
       </c>
     </row>
     <row r="76">
@@ -2997,32 +2997,32 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>DH8D</t>
+          <t>DHC7</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>75.40687030072012</v>
+        <v>50</v>
       </c>
       <c r="D76" t="n">
-        <v>1446839.618250487</v>
+        <v>610417.8060183238</v>
       </c>
       <c r="E76" t="n">
-        <v>109101647.4393578</v>
+        <v>30520890.30091619</v>
       </c>
       <c r="F76" t="n">
-        <v>2.577767465700282</v>
+        <v>3.384179807511537</v>
       </c>
       <c r="G76" t="n">
-        <v>1086896.431279712</v>
+        <v>459474.7391465366</v>
       </c>
       <c r="H76" t="n">
-        <v>81959458.22382474</v>
+        <v>22973736.95732684</v>
       </c>
       <c r="I76" t="n">
-        <v>38141027812.62428</v>
+        <v>321993542.3690056</v>
       </c>
       <c r="J76" t="n">
-        <v>-1.082854317458158</v>
+        <v>0.8905869708967964</v>
       </c>
     </row>
     <row r="77">
@@ -3031,32 +3031,32 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>DHC6</t>
+          <t>E110</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>15.9328331054753</v>
+        <v>20</v>
       </c>
       <c r="D77" t="n">
-        <v>610417.8060183238</v>
+        <v>1191751.053870659</v>
       </c>
       <c r="E77" t="n">
-        <v>9725685.027900351</v>
+        <v>23835021.07741318</v>
       </c>
       <c r="F77" t="n">
-        <v>4.909470398253264</v>
+        <v>1.89954363108434</v>
       </c>
       <c r="G77" t="n">
-        <v>458558.7279902952</v>
+        <v>897056.8997267976</v>
       </c>
       <c r="H77" t="n">
-        <v>7306139.68212842</v>
+        <v>17941137.99453595</v>
       </c>
       <c r="I77" t="n">
-        <v>2464450805.780659</v>
+        <v>1210937705.580302</v>
       </c>
       <c r="J77" t="n">
-        <v>1.586668934222617</v>
+        <v>1.18188475643242</v>
       </c>
     </row>
     <row r="78">
@@ -3065,32 +3065,32 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>DHC7</t>
+          <t>E120</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>50</v>
+        <v>29.9928591596618</v>
       </c>
       <c r="D78" t="n">
-        <v>610417.8060183238</v>
+        <v>1080595.846682759</v>
       </c>
       <c r="E78" t="n">
-        <v>30520890.30091619</v>
+        <v>32410159.03807151</v>
       </c>
       <c r="F78" t="n">
-        <v>4.309490820554568</v>
+        <v>2.273818170296539</v>
       </c>
       <c r="G78" t="n">
-        <v>458558.7279902952</v>
+        <v>813387.9612982444</v>
       </c>
       <c r="H78" t="n">
-        <v>22927936.39951476</v>
+        <v>24395830.5653827</v>
       </c>
       <c r="I78" t="n">
-        <v>365064641.1078074</v>
+        <v>2675978987.266396</v>
       </c>
       <c r="J78" t="n">
-        <v>-0.1132770736645061</v>
+        <v>0.04060053816857773</v>
       </c>
     </row>
     <row r="79">
@@ -3099,32 +3099,32 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>E110</t>
+          <t>E135</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>20</v>
+        <v>32.75343729440979</v>
       </c>
       <c r="D79" t="n">
-        <v>1191751.053870659</v>
+        <v>1705781.400628938</v>
       </c>
       <c r="E79" t="n">
-        <v>23835021.07741318</v>
+        <v>55870204.14347041</v>
       </c>
       <c r="F79" t="n">
-        <v>2.879017270647067</v>
+        <v>3.55838836547066</v>
       </c>
       <c r="G79" t="n">
-        <v>895268.5225693081</v>
+        <v>1283978.705023995</v>
       </c>
       <c r="H79" t="n">
-        <v>17905370.45138616</v>
+        <v>42054716.00236087</v>
       </c>
       <c r="I79" t="n">
-        <v>1712948174.717424</v>
+        <v>15256884581.25966</v>
       </c>
       <c r="J79" t="n">
-        <v>0.2181844312240844</v>
+        <v>-0.3669084370679702</v>
       </c>
     </row>
     <row r="80">
@@ -3133,32 +3133,32 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>E120</t>
+          <t>E145</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>29.9928591596618</v>
+        <v>49.14959220312173</v>
       </c>
       <c r="D80" t="n">
-        <v>1080595.846682759</v>
+        <v>1861120.109332631</v>
       </c>
       <c r="E80" t="n">
-        <v>32410159.03807151</v>
+        <v>91473294.41472815</v>
       </c>
       <c r="F80" t="n">
-        <v>3.324148363962107</v>
+        <v>2.355038326002673</v>
       </c>
       <c r="G80" t="n">
-        <v>811766.3869581933</v>
+        <v>1400905.52458477</v>
       </c>
       <c r="H80" t="n">
-        <v>24347194.91458463</v>
+        <v>68853935.24844179</v>
       </c>
       <c r="I80" t="n">
-        <v>2670644142.067383</v>
+        <v>31343331725.25679</v>
       </c>
       <c r="J80" t="n">
-        <v>-0.6038846400979285</v>
+        <v>-0.5313596997289746</v>
       </c>
     </row>
     <row r="81">
@@ -3167,32 +3167,32 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>E135</t>
+          <t>E170</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>32.75343729440979</v>
+        <v>70.21270508384954</v>
       </c>
       <c r="D81" t="n">
-        <v>1705781.400628938</v>
+        <v>2127350.84120212</v>
       </c>
       <c r="E81" t="n">
-        <v>55870204.14347041</v>
+        <v>149367057.2232037</v>
       </c>
       <c r="F81" t="n">
-        <v>5.17483371490656</v>
+        <v>2.113679823793869</v>
       </c>
       <c r="G81" t="n">
-        <v>1281418.958604936</v>
+        <v>1601303.178245045</v>
       </c>
       <c r="H81" t="n">
-        <v>41970875.50853463</v>
+        <v>112431827.8039503</v>
       </c>
       <c r="I81" t="n">
-        <v>15226468379.24629</v>
+        <v>15180378022.92099</v>
       </c>
       <c r="J81" t="n">
-        <v>-0.3011245124417429</v>
+        <v>-1.112813954315406</v>
       </c>
     </row>
     <row r="82">
@@ -3201,32 +3201,32 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>E145</t>
+          <t>E190</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>49.14959220312173</v>
+        <v>101.4191587862864</v>
       </c>
       <c r="D82" t="n">
-        <v>1861120.109332631</v>
+        <v>2364307.208889224</v>
       </c>
       <c r="E82" t="n">
-        <v>91473294.41472815</v>
+        <v>239786048.2378977</v>
       </c>
       <c r="F82" t="n">
-        <v>3.541798155793244</v>
+        <v>1.664294268071398</v>
       </c>
       <c r="G82" t="n">
-        <v>1398112.67226879</v>
+        <v>1779665.382228451</v>
       </c>
       <c r="H82" t="n">
-        <v>68716667.6960278</v>
+        <v>180492165.9866842</v>
       </c>
       <c r="I82" t="n">
-        <v>31280845501.12303</v>
+        <v>88667569676.46544</v>
       </c>
       <c r="J82" t="n">
-        <v>-0.6353970442201748</v>
+        <v>-1.358635352365281</v>
       </c>
     </row>
     <row r="83">
@@ -3235,32 +3235,32 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>E170</t>
+          <t>E195</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>70.21270508384954</v>
+        <v>115</v>
       </c>
       <c r="D83" t="n">
-        <v>2127350.84120212</v>
+        <v>2364307.208889224</v>
       </c>
       <c r="E83" t="n">
-        <v>149367057.2232037</v>
+        <v>271895329.0222607</v>
       </c>
       <c r="F83" t="n">
-        <v>3.203146668382609</v>
+        <v>1.538340835265424</v>
       </c>
       <c r="G83" t="n">
-        <v>1598110.812156494</v>
+        <v>1779665.382228451</v>
       </c>
       <c r="H83" t="n">
-        <v>112207683.1452552</v>
+        <v>204661518.9562718</v>
       </c>
       <c r="I83" t="n">
-        <v>15150114344.76801</v>
+        <v>55562262324.43901</v>
       </c>
       <c r="J83" t="n">
-        <v>-0.9574599407340857</v>
+        <v>-0.1441280878007292</v>
       </c>
     </row>
     <row r="84">
@@ -3269,32 +3269,32 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>E190</t>
+          <t>E75L</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>101.4191587862864</v>
+        <v>75.54287538625948</v>
       </c>
       <c r="D84" t="n">
-        <v>2364307.208889224</v>
+        <v>2177886.2061572</v>
       </c>
       <c r="E84" t="n">
-        <v>239786048.2378977</v>
+        <v>164523786.2771868</v>
       </c>
       <c r="F84" t="n">
-        <v>2.57682580348053</v>
+        <v>1.929169690711981</v>
       </c>
       <c r="G84" t="n">
-        <v>1776117.432350888</v>
+        <v>1639342.244932614</v>
       </c>
       <c r="H84" t="n">
-        <v>180132335.8946859</v>
+        <v>123840626.9243754</v>
       </c>
       <c r="I84" t="n">
-        <v>88490801562.57233</v>
+        <v>78198659803.48123</v>
       </c>
       <c r="J84" t="n">
-        <v>-0.9607649993827438</v>
+        <v>1.510505963981229</v>
       </c>
     </row>
     <row r="85">
@@ -3303,32 +3303,32 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>E195</t>
+          <t>E75S</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>115</v>
+        <v>80</v>
       </c>
       <c r="D85" t="n">
-        <v>2364307.208889224</v>
+        <v>2177886.2061572</v>
       </c>
       <c r="E85" t="n">
-        <v>271895329.0222607</v>
+        <v>174230896.492576</v>
       </c>
       <c r="F85" t="n">
-        <v>2.430980755920789</v>
+        <v>1.886327114619066</v>
       </c>
       <c r="G85" t="n">
-        <v>1776117.432350888</v>
+        <v>1639342.244932614</v>
       </c>
       <c r="H85" t="n">
-        <v>204253504.7203521</v>
+        <v>131147379.5946091</v>
       </c>
       <c r="I85" t="n">
-        <v>55451493118.17157</v>
+        <v>10479748254.35207</v>
       </c>
       <c r="J85" t="n">
-        <v>0.6103180901499708</v>
+        <v>0.1184410844905116</v>
       </c>
     </row>
     <row r="86">
@@ -3337,32 +3337,32 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>E75L</t>
+          <t>F100</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>75.54287538625948</v>
+        <v>100</v>
       </c>
       <c r="D86" t="n">
-        <v>2177886.2061572</v>
+        <v>2364307.208889224</v>
       </c>
       <c r="E86" t="n">
-        <v>164523786.2771868</v>
+        <v>236430720.8889224</v>
       </c>
       <c r="F86" t="n">
-        <v>2.908758600696512</v>
+        <v>1.886505995483197</v>
       </c>
       <c r="G86" t="n">
-        <v>1636074.043968954</v>
+        <v>1779665.382228451</v>
       </c>
       <c r="H86" t="n">
-        <v>123593737.6262403</v>
+        <v>177966538.222845</v>
       </c>
       <c r="I86" t="n">
-        <v>78042762561.0862</v>
+        <v>12422286390.56007</v>
       </c>
       <c r="J86" t="n">
-        <v>1.056517426982202</v>
+        <v>-0.3148547609773683</v>
       </c>
     </row>
     <row r="87">
@@ -3371,32 +3371,32 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>E75S</t>
+          <t>F27</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="D87" t="n">
-        <v>2177886.2061572</v>
+        <v>1011409.017644414</v>
       </c>
       <c r="E87" t="n">
-        <v>174230896.492576</v>
+        <v>60684541.05866484</v>
       </c>
       <c r="F87" t="n">
-        <v>2.890363309770574</v>
+        <v>2.176923010599811</v>
       </c>
       <c r="G87" t="n">
-        <v>1636074.043968954</v>
+        <v>761309.5325379024</v>
       </c>
       <c r="H87" t="n">
-        <v>130885923.5175163</v>
+        <v>45678571.95227414</v>
       </c>
       <c r="I87" t="n">
-        <v>10458855775.40226</v>
+        <v>241319258.6746674</v>
       </c>
       <c r="J87" t="n">
-        <v>0.6827660856379408</v>
+        <v>0.1413669374168149</v>
       </c>
     </row>
     <row r="88">
@@ -3405,32 +3405,32 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>F100</t>
+          <t>F28</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="D88" t="n">
-        <v>2364307.208889224</v>
+        <v>1698679.465539658</v>
       </c>
       <c r="E88" t="n">
-        <v>236430720.8889224</v>
+        <v>135894357.2431726</v>
       </c>
       <c r="F88" t="n">
-        <v>2.924146685301195</v>
+        <v>2.803339255488408</v>
       </c>
       <c r="G88" t="n">
-        <v>1776117.432350888</v>
+        <v>1278632.924248254</v>
       </c>
       <c r="H88" t="n">
-        <v>177611743.2350888</v>
+        <v>102290633.9398603</v>
       </c>
       <c r="I88" t="n">
-        <v>12397521257.7893</v>
+        <v>205088087.774049</v>
       </c>
       <c r="J88" t="n">
-        <v>-0.8529076488946334</v>
+        <v>-0.2488637257542743</v>
       </c>
     </row>
     <row r="89">
@@ -3439,32 +3439,32 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>F27</t>
+          <t>F50</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="D89" t="n">
-        <v>1011409.017644414</v>
+        <v>975824.3201168067</v>
       </c>
       <c r="E89" t="n">
-        <v>60684541.05866484</v>
+        <v>43912094.4052563</v>
       </c>
       <c r="F89" t="n">
-        <v>3.217792055524643</v>
+        <v>2.313212370015794</v>
       </c>
       <c r="G89" t="n">
-        <v>759791.7820159628</v>
+        <v>734524.1579094057</v>
       </c>
       <c r="H89" t="n">
-        <v>45587506.92095777</v>
+        <v>33053587.10592326</v>
       </c>
       <c r="I89" t="n">
-        <v>1077340802.936898</v>
+        <v>2422151166.485693</v>
       </c>
       <c r="J89" t="n">
-        <v>0.5129301111905863</v>
+        <v>0.3345341155600038</v>
       </c>
     </row>
     <row r="90">
@@ -3473,32 +3473,32 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>F28</t>
+          <t>F70</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="D90" t="n">
-        <v>1698679.465539658</v>
+        <v>2127350.84120212</v>
       </c>
       <c r="E90" t="n">
-        <v>135894357.2431726</v>
+        <v>159551313.090159</v>
       </c>
       <c r="F90" t="n">
-        <v>3.86749133195302</v>
+        <v>2.353526411073462</v>
       </c>
       <c r="G90" t="n">
-        <v>1276083.835204698</v>
+        <v>1601303.178245045</v>
       </c>
       <c r="H90" t="n">
-        <v>102086706.8163758</v>
+        <v>120097738.3683784</v>
       </c>
       <c r="I90" t="n">
-        <v>767785135.6967998</v>
+        <v>2794857159.108887</v>
       </c>
       <c r="J90" t="n">
-        <v>-0.1599694485222073</v>
+        <v>0.1409770581272369</v>
       </c>
     </row>
     <row r="91">
@@ -3507,32 +3507,32 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>F50</t>
+          <t>IL62</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>45</v>
+        <v>160</v>
       </c>
       <c r="D91" t="n">
-        <v>975824.3201168067</v>
+        <v>4394802.833309786</v>
       </c>
       <c r="E91" t="n">
-        <v>43912094.4052563</v>
+        <v>703168453.3295658</v>
       </c>
       <c r="F91" t="n">
-        <v>3.71212240591614</v>
+        <v>1.653622329073557</v>
       </c>
       <c r="G91" t="n">
-        <v>733059.8068453545</v>
+        <v>3308063.535379337</v>
       </c>
       <c r="H91" t="n">
-        <v>32987691.30804095</v>
+        <v>529290165.6606938</v>
       </c>
       <c r="I91" t="n">
-        <v>2417322353.709772</v>
+        <v>4040984617.197445</v>
       </c>
       <c r="J91" t="n">
-        <v>-0.3130880546953848</v>
+        <v>-0.3283954657832898</v>
       </c>
     </row>
     <row r="92">
@@ -3541,32 +3541,32 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>F70</t>
+          <t>IL96</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>75</v>
+        <v>260</v>
       </c>
       <c r="D92" t="n">
-        <v>2127350.84120212</v>
+        <v>4659848.415635562</v>
       </c>
       <c r="E92" t="n">
-        <v>159551313.090159</v>
+        <v>1211560588.065246</v>
       </c>
       <c r="F92" t="n">
-        <v>3.526860461996824</v>
+        <v>1.621291185719461</v>
       </c>
       <c r="G92" t="n">
-        <v>1598110.812156494</v>
+        <v>3507569.101239946</v>
       </c>
       <c r="H92" t="n">
-        <v>119858310.911737</v>
+        <v>911967966.3223861</v>
       </c>
       <c r="I92" t="n">
-        <v>2789285317.787206</v>
+        <v>14041572423.34831</v>
       </c>
       <c r="J92" t="n">
-        <v>-0.2527483308750961</v>
+        <v>-1.145268098720747</v>
       </c>
     </row>
     <row r="93">
@@ -3575,32 +3575,32 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>IL18</t>
+          <t>JS31</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>120</v>
+        <v>15.99851012011292</v>
       </c>
       <c r="D93" t="n">
-        <v>1118751.395250489</v>
+        <v>1030232.433108681</v>
       </c>
       <c r="E93" t="n">
-        <v>134250167.4300586</v>
+        <v>16482184.00715778</v>
       </c>
       <c r="F93" t="n">
-        <v>7.278567356101347</v>
+        <v>2.704362102058114</v>
       </c>
       <c r="G93" t="n">
-        <v>840429.6396426423</v>
+        <v>775478.3261494559</v>
       </c>
       <c r="H93" t="n">
-        <v>100851556.757117</v>
+        <v>12406497.84883029</v>
       </c>
       <c r="I93" t="n">
-        <v>1032159108.812671</v>
+        <v>333735032.4178561</v>
       </c>
       <c r="J93" t="n">
-        <v>1.050473855829789</v>
+        <v>-0.0831167848204427</v>
       </c>
     </row>
     <row r="94">
@@ -3609,32 +3609,32 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>IL62</t>
+          <t>JS32</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>160</v>
+        <v>15</v>
       </c>
       <c r="D94" t="n">
-        <v>4394802.833309786</v>
+        <v>1080595.846682759</v>
       </c>
       <c r="E94" t="n">
-        <v>703168453.3295658</v>
+        <v>16208937.70024139</v>
       </c>
       <c r="F94" t="n">
-        <v>3.179203748622764</v>
+        <v>2.903794056576392</v>
       </c>
       <c r="G94" t="n">
-        <v>3301468.563238775</v>
+        <v>813387.9612982444</v>
       </c>
       <c r="H94" t="n">
-        <v>528234970.118204</v>
+        <v>12200819.41947367</v>
       </c>
       <c r="I94" t="n">
-        <v>4703212075.132324</v>
+        <v>664874541.9905297</v>
       </c>
       <c r="J94" t="n">
-        <v>-1.159687813637907</v>
+        <v>0.2098790855225464</v>
       </c>
     </row>
     <row r="95">
@@ -3643,32 +3643,32 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>IL96</t>
+          <t>JS41</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>260</v>
+        <v>29</v>
       </c>
       <c r="D95" t="n">
-        <v>4659848.415635562</v>
+        <v>1080595.846682759</v>
       </c>
       <c r="E95" t="n">
-        <v>1211560588.065246</v>
+        <v>31337279.55380002</v>
       </c>
       <c r="F95" t="n">
-        <v>3.247267516220309</v>
+        <v>2.106414806033488</v>
       </c>
       <c r="G95" t="n">
-        <v>3500576.393797548</v>
+        <v>813387.9612982444</v>
       </c>
       <c r="H95" t="n">
-        <v>910149862.3873627</v>
+        <v>23588250.87764909</v>
       </c>
       <c r="I95" t="n">
-        <v>14013579073.77952</v>
+        <v>914924925.9557829</v>
       </c>
       <c r="J95" t="n">
-        <v>-1.34326025434018</v>
+        <v>-0.4325826643443635</v>
       </c>
     </row>
     <row r="96">
@@ -3677,32 +3677,32 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>JS31</t>
+          <t>MD82</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>15.99851012011292</v>
+        <v>150</v>
       </c>
       <c r="D96" t="n">
-        <v>1030232.433108681</v>
+        <v>1853851.041269496</v>
       </c>
       <c r="E96" t="n">
-        <v>16482184.00715778</v>
+        <v>278077656.1904244</v>
       </c>
       <c r="F96" t="n">
-        <v>4.114288318781506</v>
+        <v>2.043090480942521</v>
       </c>
       <c r="G96" t="n">
-        <v>773932.3286491453</v>
+        <v>1395433.939189951</v>
       </c>
       <c r="H96" t="n">
-        <v>12381764.1921759</v>
+        <v>209315090.8784927</v>
       </c>
       <c r="I96" t="n">
-        <v>333069696.5748211</v>
+        <v>9370266597.866537</v>
       </c>
       <c r="J96" t="n">
-        <v>-0.8462764209424475</v>
+        <v>-0.3112607672735425</v>
       </c>
     </row>
     <row r="97">
@@ -3711,32 +3711,32 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>JS32</t>
+          <t>MD83</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>15</v>
+        <v>150</v>
       </c>
       <c r="D97" t="n">
-        <v>1080595.846682759</v>
+        <v>2112088.776021521</v>
       </c>
       <c r="E97" t="n">
-        <v>16208937.70024139</v>
+        <v>316813316.4032282</v>
       </c>
       <c r="F97" t="n">
-        <v>4.517150656870017</v>
+        <v>1.855077351120051</v>
       </c>
       <c r="G97" t="n">
-        <v>811766.3869581933</v>
+        <v>1589815.090334513</v>
       </c>
       <c r="H97" t="n">
-        <v>12176495.8043729</v>
+        <v>238472263.5501769</v>
       </c>
       <c r="I97" t="n">
-        <v>663549044.751888</v>
+        <v>13421281541.08939</v>
       </c>
       <c r="J97" t="n">
-        <v>-0.4151248914293396</v>
+        <v>-0.1528028849805292</v>
       </c>
     </row>
     <row r="98">
@@ -3745,32 +3745,32 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>JS41</t>
+          <t>MD87</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>29</v>
+        <v>142.374093976337</v>
       </c>
       <c r="D98" t="n">
-        <v>1080595.846682759</v>
+        <v>2452369.46993664</v>
       </c>
       <c r="E98" t="n">
-        <v>31337279.55380002</v>
+        <v>349153881.3774588</v>
       </c>
       <c r="F98" t="n">
-        <v>3.144878631589028</v>
+        <v>1.670513388775463</v>
       </c>
       <c r="G98" t="n">
-        <v>811766.3869581933</v>
+        <v>1845951.758583273</v>
       </c>
       <c r="H98" t="n">
-        <v>23541225.22178761</v>
+        <v>262815709.1523194</v>
       </c>
       <c r="I98" t="n">
-        <v>913100927.0111279</v>
+        <v>2441349872.644446</v>
       </c>
       <c r="J98" t="n">
-        <v>-0.8459317633419543</v>
+        <v>-0.5400954328639965</v>
       </c>
     </row>
     <row r="99">
@@ -3779,32 +3779,32 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>MD82</t>
+          <t>MD88</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="D99" t="n">
-        <v>1853851.041269496</v>
+        <v>2452369.46993664</v>
       </c>
       <c r="E99" t="n">
-        <v>278077656.1904244</v>
+        <v>343331725.7911296</v>
       </c>
       <c r="F99" t="n">
-        <v>3.007562546433515</v>
+        <v>1.780474223446541</v>
       </c>
       <c r="G99" t="n">
-        <v>1392651.995054197</v>
+        <v>1845951.758583273</v>
       </c>
       <c r="H99" t="n">
-        <v>208897799.2581295</v>
+        <v>258433246.2016582</v>
       </c>
       <c r="I99" t="n">
-        <v>9351585987.140154</v>
+        <v>2469140147.760809</v>
       </c>
       <c r="J99" t="n">
-        <v>-0.9886873322871458</v>
+        <v>-0.338533271288491</v>
       </c>
     </row>
     <row r="100">
@@ -3813,32 +3813,32 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>MD83</t>
+          <t>SB20</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>150</v>
+        <v>42.8605841591612</v>
       </c>
       <c r="D100" t="n">
-        <v>2112088.776021521</v>
+        <v>1855278.529205146</v>
       </c>
       <c r="E100" t="n">
-        <v>316813316.4032282</v>
+        <v>79518321.53968199</v>
       </c>
       <c r="F100" t="n">
-        <v>2.833239294834605</v>
+        <v>2.011201253621685</v>
       </c>
       <c r="G100" t="n">
-        <v>1586645.626955932</v>
+        <v>1396508.440360135</v>
       </c>
       <c r="H100" t="n">
-        <v>237996844.0433899</v>
+        <v>59855167.53703452</v>
       </c>
       <c r="I100" t="n">
-        <v>13394524806.55044</v>
+        <v>2127819043.435884</v>
       </c>
       <c r="J100" t="n">
-        <v>-0.7832100164088397</v>
+        <v>0.3133047223977287</v>
       </c>
     </row>
     <row r="101">
@@ -3847,32 +3847,32 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>MD87</t>
+          <t>SF34</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>142.374093976337</v>
+        <v>32.97576216384803</v>
       </c>
       <c r="D101" t="n">
-        <v>2452369.46993664</v>
+        <v>1132015.500158164</v>
       </c>
       <c r="E101" t="n">
-        <v>349153881.3774588</v>
+        <v>37329073.89900509</v>
       </c>
       <c r="F101" t="n">
-        <v>2.635311880495173</v>
+        <v>1.97942671109101</v>
       </c>
       <c r="G101" t="n">
-        <v>1842271.65985165</v>
+        <v>852092.6511593193</v>
       </c>
       <c r="H101" t="n">
-        <v>262291758.4296611</v>
+        <v>28098404.60619244</v>
       </c>
       <c r="I101" t="n">
-        <v>2436482785.231143</v>
+        <v>4987612455.372992</v>
       </c>
       <c r="J101" t="n">
-        <v>-1.108074009410709</v>
+        <v>0.5156587315590514</v>
       </c>
     </row>
     <row r="102">
@@ -3881,32 +3881,32 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>MD88</t>
+          <t>SH33</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>140</v>
+        <v>27</v>
       </c>
       <c r="D102" t="n">
-        <v>2452369.46993664</v>
+        <v>1010764.767290413</v>
       </c>
       <c r="E102" t="n">
-        <v>343331725.7911296</v>
+        <v>27290648.71684115</v>
       </c>
       <c r="F102" t="n">
-        <v>2.83286732126529</v>
+        <v>3.550313974429316</v>
       </c>
       <c r="G102" t="n">
-        <v>1842271.65985165</v>
+        <v>760824.5913051416</v>
       </c>
       <c r="H102" t="n">
-        <v>257918032.379231</v>
+        <v>20542263.96523882</v>
       </c>
       <c r="I102" t="n">
-        <v>2464217657.514939</v>
+        <v>283303895.3340147</v>
       </c>
       <c r="J102" t="n">
-        <v>-0.9427829562611728</v>
+        <v>0.06206509921321894</v>
       </c>
     </row>
     <row r="103">
@@ -3915,32 +3915,32 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>SB20</t>
+          <t>SH36</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>42.8605841591612</v>
+        <v>30</v>
       </c>
       <c r="D103" t="n">
-        <v>1855278.529205146</v>
+        <v>577444.0586482342</v>
       </c>
       <c r="E103" t="n">
-        <v>79518321.53968199</v>
+        <v>17323321.75944703</v>
       </c>
       <c r="F103" t="n">
-        <v>3.252811386444076</v>
+        <v>6.027772899553292</v>
       </c>
       <c r="G103" t="n">
-        <v>1393724.354093431</v>
+        <v>434654.6834040918</v>
       </c>
       <c r="H103" t="n">
-        <v>59735839.97329409</v>
+        <v>13039640.50212276</v>
       </c>
       <c r="I103" t="n">
-        <v>2123577012.664245</v>
+        <v>376133517.8402697</v>
       </c>
       <c r="J103" t="n">
-        <v>-0.06186018843593995</v>
+        <v>0.4232629378679352</v>
       </c>
     </row>
     <row r="104">
@@ -3949,32 +3949,32 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>SF34</t>
+          <t>SU95</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>32.97576216384803</v>
+        <v>92.99652532012097</v>
       </c>
       <c r="D104" t="n">
-        <v>1132015.500158164</v>
+        <v>1650956.253056576</v>
       </c>
       <c r="E104" t="n">
-        <v>37329073.89900509</v>
+        <v>153533194.9897879</v>
       </c>
       <c r="F104" t="n">
-        <v>3.053006137678274</v>
+        <v>2.345739057351345</v>
       </c>
       <c r="G104" t="n">
-        <v>850393.9149544452</v>
+        <v>1242710.625798394</v>
       </c>
       <c r="H104" t="n">
-        <v>28042387.4851214</v>
+        <v>115567770.1776437</v>
       </c>
       <c r="I104" t="n">
-        <v>4977669126.038681</v>
+        <v>22768660647.00279</v>
       </c>
       <c r="J104" t="n">
-        <v>-0.1716250573194323</v>
+        <v>-0.8145318666927864</v>
       </c>
     </row>
     <row r="105">
@@ -3983,32 +3983,32 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>SH33</t>
+          <t>T134</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>27</v>
+        <v>80</v>
       </c>
       <c r="D105" t="n">
-        <v>1010764.767290413</v>
+        <v>1698679.465539658</v>
       </c>
       <c r="E105" t="n">
-        <v>27290648.71684115</v>
+        <v>135894357.2431726</v>
       </c>
       <c r="F105" t="n">
-        <v>4.909569655201927</v>
+        <v>4.370135818413353</v>
       </c>
       <c r="G105" t="n">
-        <v>759307.8075644883</v>
+        <v>1278632.924248254</v>
       </c>
       <c r="H105" t="n">
-        <v>20501310.80424118</v>
+        <v>102290633.9398603</v>
       </c>
       <c r="I105" t="n">
-        <v>308883525.0879642</v>
+        <v>2901919457.761273</v>
       </c>
       <c r="J105" t="n">
-        <v>-0.8137266066635098</v>
+        <v>1.193788355979296</v>
       </c>
     </row>
     <row r="106">
@@ -4017,32 +4017,32 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>SH36</t>
+          <t>T154</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>30</v>
+        <v>130</v>
       </c>
       <c r="D106" t="n">
-        <v>577444.0586482342</v>
+        <v>2311340.421146744</v>
       </c>
       <c r="E106" t="n">
-        <v>17323321.75944703</v>
+        <v>300474254.7490768</v>
       </c>
       <c r="F106" t="n">
-        <v>7.131681777174038</v>
+        <v>3.271437003499027</v>
       </c>
       <c r="G106" t="n">
-        <v>433788.1536360999</v>
+        <v>1739796.130805147</v>
       </c>
       <c r="H106" t="n">
-        <v>13013644.609083</v>
+        <v>226173497.0046691</v>
       </c>
       <c r="I106" t="n">
-        <v>375383656.1629596</v>
+        <v>7390973521.991333</v>
       </c>
       <c r="J106" t="n">
-        <v>-0.4168112116987083</v>
+        <v>-0.4807855632499191</v>
       </c>
     </row>
     <row r="107">
@@ -4051,32 +4051,32 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>SU95</t>
+          <t>T204</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>92.99652532012097</v>
+        <v>150</v>
       </c>
       <c r="D107" t="n">
-        <v>1650956.253056576</v>
+        <v>2250616.116283897</v>
       </c>
       <c r="E107" t="n">
-        <v>153533194.9897879</v>
+        <v>337592417.4425846</v>
       </c>
       <c r="F107" t="n">
-        <v>3.447713941369326</v>
+        <v>2.111058972320168</v>
       </c>
       <c r="G107" t="n">
-        <v>1240233.151630118</v>
+        <v>1694087.627773907</v>
       </c>
       <c r="H107" t="n">
-        <v>115337373.6884236</v>
+        <v>254113144.166086</v>
       </c>
       <c r="I107" t="n">
-        <v>22723268930.3568</v>
+        <v>9727626370.751316</v>
       </c>
       <c r="J107" t="n">
-        <v>0.2880746431442765</v>
+        <v>-1.258017787492887</v>
       </c>
     </row>
     <row r="108">
@@ -4085,168 +4085,32 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>T134</t>
+          <t>YK42</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="D108" t="n">
-        <v>1698679.465539658</v>
+        <v>2038513.358160724</v>
       </c>
       <c r="E108" t="n">
-        <v>135894357.2431726</v>
+        <v>203851335.8160724</v>
       </c>
       <c r="F108" t="n">
-        <v>5.611024283500194</v>
+        <v>3.04765368496966</v>
       </c>
       <c r="G108" t="n">
-        <v>1276083.835204698</v>
+        <v>1534433.275459714</v>
       </c>
       <c r="H108" t="n">
-        <v>102086706.8163758</v>
+        <v>153443327.5459715</v>
       </c>
       <c r="I108" t="n">
-        <v>3469947414.02542</v>
+        <v>3951715746.50779</v>
       </c>
       <c r="J108" t="n">
-        <v>-0.3123618427215484</v>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="1" t="n">
-        <v>107</v>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>T154</t>
-        </is>
-      </c>
-      <c r="C109" t="n">
-        <v>130</v>
-      </c>
-      <c r="D109" t="n">
-        <v>2311340.421146744</v>
-      </c>
-      <c r="E109" t="n">
-        <v>300474254.7490768</v>
-      </c>
-      <c r="F109" t="n">
-        <v>5.172048134994319</v>
-      </c>
-      <c r="G109" t="n">
-        <v>1736327.664468209</v>
-      </c>
-      <c r="H109" t="n">
-        <v>225722596.3808672</v>
-      </c>
-      <c r="I109" t="n">
-        <v>7659839315.62436</v>
-      </c>
-      <c r="J109" t="n">
-        <v>-1.261066719610108</v>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="1" t="n">
-        <v>108</v>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>T204</t>
-        </is>
-      </c>
-      <c r="C110" t="n">
-        <v>150</v>
-      </c>
-      <c r="D110" t="n">
-        <v>2250616.116283897</v>
-      </c>
-      <c r="E110" t="n">
-        <v>337592417.4425846</v>
-      </c>
-      <c r="F110" t="n">
-        <v>3.172128027122035</v>
-      </c>
-      <c r="G110" t="n">
-        <v>1690710.286139035</v>
-      </c>
-      <c r="H110" t="n">
-        <v>253606542.9208553</v>
-      </c>
-      <c r="I110" t="n">
-        <v>9708233325.780207</v>
-      </c>
-      <c r="J110" t="n">
-        <v>-1.418653563394773</v>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="1" t="n">
-        <v>109</v>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>YK40</t>
-        </is>
-      </c>
-      <c r="C111" t="n">
-        <v>30</v>
-      </c>
-      <c r="D111" t="n">
-        <v>1698679.465539658</v>
-      </c>
-      <c r="E111" t="n">
-        <v>50960383.96618973</v>
-      </c>
-      <c r="F111" t="n">
-        <v>8.849915034327175</v>
-      </c>
-      <c r="G111" t="n">
-        <v>1276083.835204698</v>
-      </c>
-      <c r="H111" t="n">
-        <v>38282515.05614093</v>
-      </c>
-      <c r="I111" t="n">
-        <v>1236050097.722882</v>
-      </c>
-      <c r="J111" t="n">
-        <v>0.2619580223274577</v>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="1" t="n">
-        <v>110</v>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>YK42</t>
-        </is>
-      </c>
-      <c r="C112" t="n">
-        <v>100</v>
-      </c>
-      <c r="D112" t="n">
-        <v>2038513.358160724</v>
-      </c>
-      <c r="E112" t="n">
-        <v>203851335.8160724</v>
-      </c>
-      <c r="F112" t="n">
-        <v>4.70663475903901</v>
-      </c>
-      <c r="G112" t="n">
-        <v>1531374.221546457</v>
-      </c>
-      <c r="H112" t="n">
-        <v>153137422.1546457</v>
-      </c>
-      <c r="I112" t="n">
-        <v>3943837586.074378</v>
-      </c>
-      <c r="J112" t="n">
-        <v>-0.8252581062329447</v>
+        <v>-0.2020529799342099</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
- calibration notebook rerun - review of the segment names
</commit_message>
<xml_diff>
--- a/aeromaps/utils/calibration_notebooks/fleet_calibrated_inputs_processed_here/aircraft_type_key_parameters.xlsx
+++ b/aeromaps/utils/calibration_notebooks/fleet_calibrated_inputs_processed_here/aircraft_type_key_parameters.xlsx
@@ -497,13 +497,13 @@
         <v>1.178449744963836</v>
       </c>
       <c r="G2" t="n">
-        <v>2028725.720176643</v>
+        <v>2124883.488884532</v>
       </c>
       <c r="H2" t="n">
-        <v>284021600.8247299</v>
+        <v>297483688.4438344</v>
       </c>
       <c r="I2" t="n">
-        <v>6418102795.956368</v>
+        <v>6722308750.491856</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -531,13 +531,13 @@
         <v>0.8524547275953843</v>
       </c>
       <c r="G3" t="n">
-        <v>2193508.839569498</v>
+        <v>2297477.017010296</v>
       </c>
       <c r="H3" t="n">
-        <v>401166631.841258</v>
+        <v>420181172.7495064</v>
       </c>
       <c r="I3" t="n">
-        <v>812872522552.1776</v>
+        <v>851401145339.9662</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -565,13 +565,13 @@
         <v>0.8330292323059032</v>
       </c>
       <c r="G4" t="n">
-        <v>2472087.789021186</v>
+        <v>2589260.082682253</v>
       </c>
       <c r="H4" t="n">
-        <v>490558143.4194629</v>
+        <v>513809673.1967819</v>
       </c>
       <c r="I4" t="n">
-        <v>758898209770.7921</v>
+        <v>794868552041.4155</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -599,13 +599,13 @@
         <v>1.229639562991454</v>
       </c>
       <c r="G5" t="n">
-        <v>2610879.897151033</v>
+        <v>2734630.67468466</v>
       </c>
       <c r="H5" t="n">
-        <v>699950740.2284578</v>
+        <v>733127083.7412435</v>
       </c>
       <c r="I5" t="n">
-        <v>13419563573.9791</v>
+        <v>14055625549.96427</v>
       </c>
       <c r="J5" t="n">
         <v>-0.6243207238688866</v>
@@ -633,13 +633,13 @@
         <v>1.174570952133184</v>
       </c>
       <c r="G6" t="n">
-        <v>2696823.183226326</v>
+        <v>2824647.510250766</v>
       </c>
       <c r="H6" t="n">
-        <v>622921828.9654467</v>
+        <v>652447147.5223285</v>
       </c>
       <c r="I6" t="n">
-        <v>10661705947.4627</v>
+        <v>11167050679.05036</v>
       </c>
       <c r="J6" t="n">
         <v>-0.4315208434238162</v>
@@ -667,13 +667,13 @@
         <v>1.680027915024445</v>
       </c>
       <c r="G7" t="n">
-        <v>2321023.902299946</v>
+        <v>2431036.052953514</v>
       </c>
       <c r="H7" t="n">
-        <v>220819430.7793765</v>
+        <v>231285854.8700822</v>
       </c>
       <c r="I7" t="n">
-        <v>4892370777.182905</v>
+        <v>5124259914.756726</v>
       </c>
       <c r="J7" t="n">
         <v>-2.693006512525284</v>
@@ -701,13 +701,13 @@
         <v>1.343098767003529</v>
       </c>
       <c r="G8" t="n">
-        <v>2028725.720176643</v>
+        <v>2124883.488884532</v>
       </c>
       <c r="H8" t="n">
-        <v>265148333.4699696</v>
+        <v>277715863.8509949</v>
       </c>
       <c r="I8" t="n">
-        <v>233917999697.0553</v>
+        <v>245005271223.1062</v>
       </c>
       <c r="J8" t="n">
         <v>-1.054220956300929</v>
@@ -735,13 +735,13 @@
         <v>1.129040999847672</v>
       </c>
       <c r="G9" t="n">
-        <v>2198997.78175266</v>
+        <v>2303226.12468929</v>
       </c>
       <c r="H9" t="n">
-        <v>346503363.2922248</v>
+        <v>362926968.4807361</v>
       </c>
       <c r="I9" t="n">
-        <v>1186571190299.336</v>
+        <v>1242812424359.461</v>
       </c>
       <c r="J9" t="n">
         <v>-0.4964523917793309</v>
@@ -769,13 +769,13 @@
         <v>1.213652392088143</v>
       </c>
       <c r="G10" t="n">
-        <v>2302027.524011897</v>
+        <v>2411139.282201593</v>
       </c>
       <c r="H10" t="n">
-        <v>428523133.2485166</v>
+        <v>448834320.671774</v>
       </c>
       <c r="I10" t="n">
-        <v>636240443739.0677</v>
+        <v>666397039489.3988</v>
       </c>
       <c r="J10" t="n">
         <v>-0.1662883240459748</v>
@@ -803,13 +803,13 @@
         <v>1.158197581335016</v>
       </c>
       <c r="G11" t="n">
-        <v>3561889.969115667</v>
+        <v>3730716.828462308</v>
       </c>
       <c r="H11" t="n">
-        <v>935736793.0379031</v>
+        <v>980088950.2672037</v>
       </c>
       <c r="I11" t="n">
-        <v>367117917895.2161</v>
+        <v>384518614049.6555</v>
       </c>
       <c r="J11" t="n">
         <v>-1.42681980614188</v>
@@ -837,13 +837,13 @@
         <v>1.148368652583524</v>
       </c>
       <c r="G12" t="n">
-        <v>3669242.924534954</v>
+        <v>3843158.111275807</v>
       </c>
       <c r="H12" t="n">
-        <v>1058626968.059853</v>
+        <v>1108803887.556772</v>
       </c>
       <c r="I12" t="n">
-        <v>646414447679.1494</v>
+        <v>677053272006.7463</v>
       </c>
       <c r="J12" t="n">
         <v>-0.5285890937797832</v>
@@ -871,13 +871,13 @@
         <v>1.206911147835214</v>
       </c>
       <c r="G13" t="n">
-        <v>3636907.153840894</v>
+        <v>3809289.68610388</v>
       </c>
       <c r="H13" t="n">
-        <v>891042252.6910192</v>
+        <v>933275973.0954509</v>
       </c>
       <c r="I13" t="n">
-        <v>6035920787.119107</v>
+        <v>6322012036.031949</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -905,13 +905,13 @@
         <v>1.081850374244981</v>
       </c>
       <c r="G14" t="n">
-        <v>3636907.153840894</v>
+        <v>3809289.68610388</v>
       </c>
       <c r="H14" t="n">
-        <v>994045806.6722177</v>
+        <v>1041161701.054782</v>
       </c>
       <c r="I14" t="n">
-        <v>137347323845.6507</v>
+        <v>143857327671.0312</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -939,13 +939,13 @@
         <v>1.225404189833046</v>
       </c>
       <c r="G15" t="n">
-        <v>3686703.543913495</v>
+        <v>3861446.331045568</v>
       </c>
       <c r="H15" t="n">
-        <v>1023367235.889536</v>
+        <v>1071872910.655335</v>
       </c>
       <c r="I15" t="n">
-        <v>4587177498.721916</v>
+        <v>4804601051.130829</v>
       </c>
       <c r="J15" t="n">
         <v>-0.8585427768451319</v>
@@ -973,13 +973,13 @@
         <v>1.260179397395529</v>
       </c>
       <c r="G16" t="n">
-        <v>3723185.529826646</v>
+        <v>3899657.494209519</v>
       </c>
       <c r="H16" t="n">
-        <v>1032011459.517374</v>
+        <v>1080926854.162009</v>
       </c>
       <c r="I16" t="n">
-        <v>54597111321.17908</v>
+        <v>57184911313.22714</v>
       </c>
       <c r="J16" t="n">
         <v>-1.363064396189034</v>
@@ -1007,13 +1007,13 @@
         <v>2.076914867607091</v>
       </c>
       <c r="G17" t="n">
-        <v>3897545.180924576</v>
+        <v>4082281.463561768</v>
       </c>
       <c r="H17" t="n">
-        <v>796888173.0667516</v>
+        <v>834659167.8689139</v>
       </c>
       <c r="I17" t="n">
-        <v>12616739097.03875</v>
+        <v>13214748708.62646</v>
       </c>
       <c r="J17" t="n">
         <v>-1.85691811720076</v>
@@ -1041,13 +1041,13 @@
         <v>1.428662850478296</v>
       </c>
       <c r="G18" t="n">
-        <v>3698210.336613057</v>
+        <v>3873498.523993163</v>
       </c>
       <c r="H18" t="n">
-        <v>1119619973.237859</v>
+        <v>1172687846.019579</v>
       </c>
       <c r="I18" t="n">
-        <v>47337013478.27247</v>
+        <v>49580698540.3269</v>
       </c>
       <c r="J18" t="n">
         <v>-2.019125475237955</v>
@@ -1075,13 +1075,13 @@
         <v>1.097180837791816</v>
       </c>
       <c r="G19" t="n">
-        <v>3725253.635452399</v>
+        <v>3901823.624137151</v>
       </c>
       <c r="H19" t="n">
-        <v>1102092082.567823</v>
+        <v>1154329166.42612</v>
       </c>
       <c r="I19" t="n">
-        <v>569197174995.5222</v>
+        <v>596176046391.5223</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1109,13 +1109,13 @@
         <v>0.9984880328710761</v>
       </c>
       <c r="G20" t="n">
-        <v>3729868.941361081</v>
+        <v>3906657.686831765</v>
       </c>
       <c r="H20" t="n">
-        <v>1264387900.124974</v>
+        <v>1324317499.305431</v>
       </c>
       <c r="I20" t="n">
-        <v>113391153463.4148</v>
+        <v>118765680044.2216</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1143,13 +1143,13 @@
         <v>1.412066518413993</v>
       </c>
       <c r="G21" t="n">
-        <v>3750151.345093933</v>
+        <v>3927901.438206434</v>
       </c>
       <c r="H21" t="n">
-        <v>1771666477.279503</v>
+        <v>1855640123.226541</v>
       </c>
       <c r="I21" t="n">
-        <v>361145039018.8002</v>
+        <v>378262631991.8649</v>
       </c>
       <c r="J21" t="n">
         <v>-1.786346028204582</v>
@@ -1177,13 +1177,13 @@
         <v>2.729543634431751</v>
       </c>
       <c r="G22" t="n">
-        <v>1298434.800743027</v>
+        <v>1359978.15872897</v>
       </c>
       <c r="H22" t="n">
-        <v>103874784.0594421</v>
+        <v>108798252.6983176</v>
       </c>
       <c r="I22" t="n">
-        <v>15231625291.97161</v>
+        <v>15953575572.04354</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1211,13 +1211,13 @@
         <v>2.41333855030665</v>
       </c>
       <c r="G23" t="n">
-        <v>745899.5545392873</v>
+        <v>781253.7850946437</v>
       </c>
       <c r="H23" t="n">
-        <v>30947623.24495404</v>
+        <v>32414482.15468782</v>
       </c>
       <c r="I23" t="n">
-        <v>1242178218.956549</v>
+        <v>1301055121.183628</v>
       </c>
       <c r="J23" t="n">
         <v>-0.1490941480697875</v>
@@ -1245,13 +1245,13 @@
         <v>4.028249795385581</v>
       </c>
       <c r="G24" t="n">
-        <v>466590.5124576276</v>
+        <v>488706.0217805386</v>
       </c>
       <c r="H24" t="n">
-        <v>19596801.52322036</v>
+        <v>20525652.91478262</v>
       </c>
       <c r="I24" t="n">
-        <v>1492412804.325547</v>
+        <v>1563150353.43225</v>
       </c>
       <c r="J24" t="n">
         <v>-0.2286593211176034</v>
@@ -1279,13 +1279,13 @@
         <v>3.759699809026542</v>
       </c>
       <c r="G25" t="n">
-        <v>466590.5124576276</v>
+        <v>488706.0217805386</v>
       </c>
       <c r="H25" t="n">
-        <v>20996573.06059324</v>
+        <v>21991770.98012424</v>
       </c>
       <c r="I25" t="n">
-        <v>1396762904.246571</v>
+        <v>1462966828.685704</v>
       </c>
       <c r="J25" t="n">
         <v>-1.917517451853091</v>
@@ -1313,13 +1313,13 @@
         <v>1.587888411702909</v>
       </c>
       <c r="G26" t="n">
-        <v>855150.000009898</v>
+        <v>895682.4954052556</v>
       </c>
       <c r="H26" t="n">
-        <v>55657681.23685402</v>
+        <v>58295750.24044749</v>
       </c>
       <c r="I26" t="n">
-        <v>1143349524.596758</v>
+        <v>1197542133.309225</v>
       </c>
       <c r="J26" t="n">
         <v>-0.6379947226602307</v>
@@ -1347,13 +1347,13 @@
         <v>1.476402419913499</v>
       </c>
       <c r="G27" t="n">
-        <v>855150.000009898</v>
+        <v>895682.4954052556</v>
       </c>
       <c r="H27" t="n">
-        <v>59860500.00069284</v>
+        <v>62697774.67836787</v>
       </c>
       <c r="I27" t="n">
-        <v>13472663742.45835</v>
+        <v>14111242566.17124</v>
       </c>
       <c r="J27" t="n">
         <v>-0.8649438723091367</v>
@@ -1381,13 +1381,13 @@
         <v>1.476402419913499</v>
       </c>
       <c r="G28" t="n">
-        <v>855150.000009898</v>
+        <v>895682.4954052556</v>
       </c>
       <c r="H28" t="n">
-        <v>59860500.00069284</v>
+        <v>62697774.67836787</v>
       </c>
       <c r="I28" t="n">
-        <v>32527722981.66713</v>
+        <v>34069475635.54146</v>
       </c>
       <c r="J28" t="n">
         <v>-0.6152740745620315</v>
@@ -1415,13 +1415,13 @@
         <v>2.967918644423394</v>
       </c>
       <c r="G29" t="n">
-        <v>910949.4013199486</v>
+        <v>954126.6829827881</v>
       </c>
       <c r="H29" t="n">
-        <v>15560011.76054947</v>
+        <v>16297526.93920688</v>
       </c>
       <c r="I29" t="n">
-        <v>5359628449.145752</v>
+        <v>5613664718.14337</v>
       </c>
       <c r="J29" t="n">
         <v>1.057632377297526</v>
@@ -1449,13 +1449,13 @@
         <v>0.8763039646656254</v>
       </c>
       <c r="G30" t="n">
-        <v>2200961.756570229</v>
+        <v>2305283.18820504</v>
       </c>
       <c r="H30" t="n">
-        <v>378400467.9402116</v>
+        <v>396335935.6642486</v>
       </c>
       <c r="I30" t="n">
-        <v>526573732066.5878</v>
+        <v>551532332744.8994</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1483,13 +1483,13 @@
         <v>0.7851654512067765</v>
       </c>
       <c r="G31" t="n">
-        <v>2449022.396120199</v>
+        <v>2565101.43370743</v>
       </c>
       <c r="H31" t="n">
-        <v>436059736.0420694</v>
+        <v>456728144.2079134</v>
       </c>
       <c r="I31" t="n">
-        <v>99423094009.90126</v>
+        <v>104135560945.6457</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1517,13 +1517,13 @@
         <v>0.7358017415760942</v>
       </c>
       <c r="G32" t="n">
-        <v>2449022.396120199</v>
+        <v>2565101.43370743</v>
       </c>
       <c r="H32" t="n">
-        <v>465314255.2628377</v>
+        <v>487369272.4044116</v>
       </c>
       <c r="I32" t="n">
-        <v>465314255.2628377</v>
+        <v>487369272.4044116</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1551,13 +1551,13 @@
         <v>2.922741166837872</v>
       </c>
       <c r="G33" t="n">
-        <v>1457766.288866123</v>
+        <v>1526861.65855599</v>
       </c>
       <c r="H33" t="n">
-        <v>116621303.1092898</v>
+        <v>122148932.6844791</v>
       </c>
       <c r="I33" t="n">
-        <v>8461305507.313281</v>
+        <v>8862355412.604656</v>
       </c>
       <c r="J33" t="n">
         <v>-0.2964742868686928</v>
@@ -1585,13 +1585,13 @@
         <v>2.623618271687993</v>
       </c>
       <c r="G34" t="n">
-        <v>1457766.288866123</v>
+        <v>1526861.65855599</v>
       </c>
       <c r="H34" t="n">
-        <v>131198965.997951</v>
+        <v>137417549.2700391</v>
       </c>
       <c r="I34" t="n">
-        <v>2842939946.84035</v>
+        <v>2977689932.577649</v>
       </c>
       <c r="J34" t="n">
         <v>0.4428404390783032</v>
@@ -1619,13 +1619,13 @@
         <v>2.488394116576957</v>
       </c>
       <c r="G35" t="n">
-        <v>1457766.288866123</v>
+        <v>1526861.65855599</v>
       </c>
       <c r="H35" t="n">
-        <v>145776628.8866123</v>
+        <v>152686165.855599</v>
       </c>
       <c r="I35" t="n">
-        <v>1250400476.346995</v>
+        <v>1309667098.049972</v>
       </c>
       <c r="J35" t="n">
         <v>-0.6045605979355976</v>
@@ -1653,13 +1653,13 @@
         <v>1.889656157541419</v>
       </c>
       <c r="G36" t="n">
-        <v>1457766.288866123</v>
+        <v>1526861.65855599</v>
       </c>
       <c r="H36" t="n">
-        <v>166318358.2518701</v>
+        <v>174201534.4080173</v>
       </c>
       <c r="I36" t="n">
-        <v>16074499101.50867</v>
+        <v>16836400008.72615</v>
       </c>
       <c r="J36" t="n">
         <v>-0.2585451858503126</v>
@@ -1687,13 +1687,13 @@
         <v>12.48206279236391</v>
       </c>
       <c r="G37" t="n">
-        <v>1605940.241616081</v>
+        <v>1682058.77689968</v>
       </c>
       <c r="H37" t="n">
-        <v>51834401.41721267</v>
+        <v>54291254.17607365</v>
       </c>
       <c r="I37" t="n">
-        <v>269085725.8101796</v>
+        <v>281839881.153957</v>
       </c>
       <c r="J37" t="n">
         <v>0.0752079882855939</v>
@@ -1721,13 +1721,13 @@
         <v>2.424017752474225</v>
       </c>
       <c r="G38" t="n">
-        <v>1417044.684538699</v>
+        <v>1484209.927069736</v>
       </c>
       <c r="H38" t="n">
-        <v>161580863.3128499</v>
+        <v>169239491.1537319</v>
       </c>
       <c r="I38" t="n">
-        <v>4825492441.080703</v>
+        <v>5054211671.795984</v>
       </c>
       <c r="J38" t="n">
         <v>0.4353941581541733</v>
@@ -1755,13 +1755,13 @@
         <v>1.645469940597836</v>
       </c>
       <c r="G39" t="n">
-        <v>1614436.169200317</v>
+        <v>1690957.395410284</v>
       </c>
       <c r="H39" t="n">
-        <v>220375725.8853991</v>
+        <v>230821119.2018875</v>
       </c>
       <c r="I39" t="n">
-        <v>35035370185.31226</v>
+        <v>36695980581.96124</v>
       </c>
       <c r="J39" t="n">
         <v>-0.4956950334836177</v>
@@ -1789,13 +1789,13 @@
         <v>1.705966933028853</v>
       </c>
       <c r="G40" t="n">
-        <v>1766739.929494315</v>
+        <v>1850480.06637813</v>
       </c>
       <c r="H40" t="n">
-        <v>246956481.7395131</v>
+        <v>258661752.6964734</v>
       </c>
       <c r="I40" t="n">
-        <v>21343345186.8785</v>
+        <v>22354979450.45643</v>
       </c>
       <c r="J40" t="n">
         <v>-0.02443755020506672</v>
@@ -1823,13 +1823,13 @@
         <v>1.747985551995309</v>
       </c>
       <c r="G41" t="n">
-        <v>1808888.441736263</v>
+        <v>1894626.338519917</v>
       </c>
       <c r="H41" t="n">
-        <v>212997621.9577674</v>
+        <v>223093307.078653</v>
       </c>
       <c r="I41" t="n">
-        <v>21999330820.9717</v>
+        <v>23042057565.04193</v>
       </c>
       <c r="J41" t="n">
         <v>-0.4467128126006354</v>
@@ -1857,13 +1857,13 @@
         <v>1.477731589399572</v>
       </c>
       <c r="G42" t="n">
-        <v>2138547.30786031</v>
+        <v>2239910.412470728</v>
       </c>
       <c r="H42" t="n">
-        <v>245334472.8173595</v>
+        <v>256962863.613918</v>
       </c>
       <c r="I42" t="n">
-        <v>4332569478.456374</v>
+        <v>4537925091.42903</v>
       </c>
       <c r="J42" t="n">
         <v>-1.86319444881112</v>
@@ -1891,13 +1891,13 @@
         <v>1.436323561650747</v>
       </c>
       <c r="G43" t="n">
-        <v>1884556.656888712</v>
+        <v>1973881.084201755</v>
       </c>
       <c r="H43" t="n">
-        <v>261204511.2527112</v>
+        <v>273585111.9069527</v>
       </c>
       <c r="I43" t="n">
-        <v>185024955299.0512</v>
+        <v>193794788835.3878</v>
       </c>
       <c r="J43" t="n">
         <v>-1.056465935146006</v>
@@ -1925,13 +1925,13 @@
         <v>1.158904218673777</v>
       </c>
       <c r="G44" t="n">
-        <v>2214208.37395246</v>
+        <v>2319157.670240306</v>
       </c>
       <c r="H44" t="n">
-        <v>367846720.7199944</v>
+        <v>385281960.7522787</v>
       </c>
       <c r="I44" t="n">
-        <v>1551652636802.191</v>
+        <v>1625198042117.81</v>
       </c>
       <c r="J44" t="n">
         <v>0.4649960614078142</v>
@@ -1959,13 +1959,13 @@
         <v>1.085212054990146</v>
       </c>
       <c r="G45" t="n">
-        <v>2260340.239788168</v>
+        <v>2367476.099415245</v>
       </c>
       <c r="H45" t="n">
-        <v>403629341.0958279</v>
+        <v>422760609.772912</v>
       </c>
       <c r="I45" t="n">
-        <v>197690496205.9271</v>
+        <v>207060652467.4952</v>
       </c>
       <c r="J45" t="n">
         <v>0.1791196930766627</v>
@@ -1993,13 +1993,13 @@
         <v>1.544157495477784</v>
       </c>
       <c r="G46" t="n">
-        <v>3651760.851666177</v>
+        <v>3824847.421160877</v>
       </c>
       <c r="H46" t="n">
-        <v>1223428350.282788</v>
+        <v>1281416544.136279</v>
       </c>
       <c r="I46" t="n">
-        <v>56019553105.3252</v>
+        <v>58674774152.23545</v>
       </c>
       <c r="J46" t="n">
         <v>-1.030542493092959</v>
@@ -2027,13 +2027,13 @@
         <v>1.241535095777449</v>
       </c>
       <c r="G47" t="n">
-        <v>3709666.153498835</v>
+        <v>3885497.324969647</v>
       </c>
       <c r="H47" t="n">
-        <v>1355358518.460788</v>
+        <v>1419599953.189121</v>
       </c>
       <c r="I47" t="n">
-        <v>47821364173.6073</v>
+        <v>50088006544.12009</v>
       </c>
       <c r="J47" t="n">
         <v>0</v>
@@ -2061,13 +2061,13 @@
         <v>1.324212276281809</v>
       </c>
       <c r="G48" t="n">
-        <v>2507111.352558015</v>
+        <v>2625943.697002884</v>
       </c>
       <c r="H48" t="n">
-        <v>449016188.5548375</v>
+        <v>470298708.1067632</v>
       </c>
       <c r="I48" t="n">
-        <v>77316597419.06854</v>
+        <v>80981258155.59061</v>
       </c>
       <c r="J48" t="n">
         <v>-0.1360243100705888</v>
@@ -2095,13 +2095,13 @@
         <v>1.163961944685927</v>
       </c>
       <c r="G49" t="n">
-        <v>2436920.831820901</v>
+        <v>2552426.278109258</v>
       </c>
       <c r="H49" t="n">
-        <v>557562191.5391824</v>
+        <v>583989586.6873152</v>
       </c>
       <c r="I49" t="n">
-        <v>24474708448.76752</v>
+        <v>25634763418.64521</v>
       </c>
       <c r="J49" t="n">
         <v>2.066449901832937</v>
@@ -2129,13 +2129,13 @@
         <v>1.383383760653715</v>
       </c>
       <c r="G50" t="n">
-        <v>3158160.500322415</v>
+        <v>3307851.345128164</v>
       </c>
       <c r="H50" t="n">
-        <v>612123340.1319579</v>
+        <v>641136830.7067136</v>
       </c>
       <c r="I50" t="n">
-        <v>11275096410.21249</v>
+        <v>11809514691.59454</v>
       </c>
       <c r="J50" t="n">
         <v>-0.04844023038190387</v>
@@ -2163,13 +2163,13 @@
         <v>1.174247232680542</v>
       </c>
       <c r="G51" t="n">
-        <v>3359294.709176114</v>
+        <v>3518518.935720877</v>
       </c>
       <c r="H51" t="n">
-        <v>749210249.2058291</v>
+        <v>784721400.4374709</v>
       </c>
       <c r="I51" t="n">
-        <v>136643466216.3939</v>
+        <v>143120108519.0982</v>
       </c>
       <c r="J51" t="n">
         <v>-0.1098505376682319</v>
@@ -2197,13 +2197,13 @@
         <v>1.224601924257454</v>
       </c>
       <c r="G52" t="n">
-        <v>3574608.506288952</v>
+        <v>3744038.20028379</v>
       </c>
       <c r="H52" t="n">
-        <v>854660222.5451517</v>
+        <v>895169503.4134271</v>
       </c>
       <c r="I52" t="n">
-        <v>25800270778.5694</v>
+        <v>27023154900.09105</v>
       </c>
       <c r="J52" t="n">
         <v>0</v>
@@ -2231,13 +2231,13 @@
         <v>1.242461676533537</v>
       </c>
       <c r="G53" t="n">
-        <v>3601299.46097678</v>
+        <v>3771994.255828743</v>
       </c>
       <c r="H53" t="n">
-        <v>1020628384.32392</v>
+        <v>1069004242.696722</v>
       </c>
       <c r="I53" t="n">
-        <v>300249222046.6429</v>
+        <v>314480468272.3628</v>
       </c>
       <c r="J53" t="n">
         <v>-0.4393742853662961</v>
@@ -2265,13 +2265,13 @@
         <v>1.249185074303995</v>
       </c>
       <c r="G54" t="n">
-        <v>3698541.714115383</v>
+        <v>3873845.608163427</v>
       </c>
       <c r="H54" t="n">
-        <v>1294489599.940384</v>
+        <v>1355845962.857199</v>
       </c>
       <c r="I54" t="n">
-        <v>53222729751.37748</v>
+        <v>55745386651.981</v>
       </c>
       <c r="J54" t="n">
         <v>0.322840932025079</v>
@@ -2299,13 +2299,13 @@
         <v>0.9757883476193243</v>
       </c>
       <c r="G55" t="n">
-        <v>3698541.714115383</v>
+        <v>3873845.608163427</v>
       </c>
       <c r="H55" t="n">
-        <v>1294489599.940384</v>
+        <v>1355845962.857199</v>
       </c>
       <c r="I55" t="n">
-        <v>58096153212.95697</v>
+        <v>60849801184.14905</v>
       </c>
       <c r="J55" t="n">
         <v>0</v>
@@ -2333,13 +2333,13 @@
         <v>1.251541412066441</v>
       </c>
       <c r="G56" t="n">
-        <v>3698541.714115383</v>
+        <v>3873845.608163427</v>
       </c>
       <c r="H56" t="n">
-        <v>1174110440.473939</v>
+        <v>1229761058.519429</v>
       </c>
       <c r="I56" t="n">
-        <v>839817992396.6256</v>
+        <v>879623779579.413</v>
       </c>
       <c r="J56" t="n">
         <v>-0.1746664338412045</v>
@@ -2367,13 +2367,13 @@
         <v>0.9949389212208551</v>
       </c>
       <c r="G57" t="n">
-        <v>3599401.972313855</v>
+        <v>3770006.829785835</v>
       </c>
       <c r="H57" t="n">
-        <v>870742154.1756097</v>
+        <v>912013688.2389414</v>
       </c>
       <c r="I57" t="n">
-        <v>311395779914.5441</v>
+        <v>326155351937.4335</v>
       </c>
       <c r="J57" t="n">
         <v>-0.429498513927575</v>
@@ -2401,13 +2401,13 @@
         <v>0.8812055291279901</v>
       </c>
       <c r="G58" t="n">
-        <v>3651105.741703064</v>
+        <v>3824161.260222423</v>
       </c>
       <c r="H58" t="n">
-        <v>998550313.9245722</v>
+        <v>1045879713.445957</v>
       </c>
       <c r="I58" t="n">
-        <v>604877948633.7627</v>
+        <v>633548021331.4971</v>
       </c>
       <c r="J58" t="n">
         <v>0.7135031330351608</v>
@@ -2435,13 +2435,13 @@
         <v>0.8828858610008796</v>
       </c>
       <c r="G59" t="n">
-        <v>3594962.059738217</v>
+        <v>3765356.473737092</v>
       </c>
       <c r="H59" t="n">
-        <v>1118950567.779775</v>
+        <v>1171986712.006684</v>
       </c>
       <c r="I59" t="n">
-        <v>126424683228.8499</v>
+        <v>132416974511.9857</v>
       </c>
       <c r="J59" t="n">
         <v>0</v>
@@ -2469,13 +2469,13 @@
         <v>1.559350380561198</v>
       </c>
       <c r="G60" t="n">
-        <v>2028725.720176643</v>
+        <v>2124883.488884532</v>
       </c>
       <c r="H60" t="n">
-        <v>223159829.2194307</v>
+        <v>233737183.7772985</v>
       </c>
       <c r="I60" t="n">
-        <v>14928344565.26991</v>
+        <v>15635919911.51924</v>
       </c>
       <c r="J60" t="n">
         <v>0</v>
@@ -2503,13 +2503,13 @@
         <v>1.260115242506681</v>
       </c>
       <c r="G61" t="n">
-        <v>2198997.78175266</v>
+        <v>2303226.12468929</v>
       </c>
       <c r="H61" t="n">
-        <v>307859689.4453725</v>
+        <v>322451657.4565007</v>
       </c>
       <c r="I61" t="n">
-        <v>95361003363.96048</v>
+        <v>99880934872.70358</v>
       </c>
       <c r="J61" t="n">
         <v>0</v>
@@ -2537,13 +2537,13 @@
         <v>1.186044863978063</v>
       </c>
       <c r="G62" t="n">
-        <v>2198997.78175266</v>
+        <v>2303226.12468929</v>
       </c>
       <c r="H62" t="n">
-        <v>329849667.2628991</v>
+        <v>345483918.7033936</v>
       </c>
       <c r="I62" t="n">
-        <v>4905785435.805227</v>
+        <v>5138310402.869585</v>
       </c>
       <c r="J62" t="n">
         <v>0</v>
@@ -2571,13 +2571,13 @@
         <v>2.426303926504643</v>
       </c>
       <c r="G63" t="n">
-        <v>1298434.800743027</v>
+        <v>1359978.15872897</v>
       </c>
       <c r="H63" t="n">
-        <v>64916425.24322812</v>
+        <v>67993341.23132817</v>
       </c>
       <c r="I63" t="n">
-        <v>28668639905.03608</v>
+        <v>30027479307.39659</v>
       </c>
       <c r="J63" t="n">
         <v>-1.339402047145975</v>
@@ -2605,13 +2605,13 @@
         <v>2.315458107421362</v>
       </c>
       <c r="G64" t="n">
-        <v>1558196.669655111</v>
+        <v>1632052.249772197</v>
       </c>
       <c r="H64" t="n">
-        <v>102510068.4325019</v>
+        <v>107368852.1273743</v>
       </c>
       <c r="I64" t="n">
-        <v>25751714036.1874</v>
+        <v>26972296659.79992</v>
       </c>
       <c r="J64" t="n">
         <v>-0.07908807757601682</v>
@@ -2639,13 +2639,13 @@
         <v>2.012412678660564</v>
       </c>
       <c r="G65" t="n">
-        <v>1582545.682836516</v>
+        <v>1657555.360205131</v>
       </c>
       <c r="H65" t="n">
-        <v>120885465.8884942</v>
+        <v>126615208.7282701</v>
       </c>
       <c r="I65" t="n">
-        <v>50160313172.0117</v>
+        <v>52537817308.88912</v>
       </c>
       <c r="J65" t="n">
         <v>0.0476991099844348</v>
@@ -2673,13 +2673,13 @@
         <v>1.556991741800394</v>
       </c>
       <c r="G66" t="n">
-        <v>1582545.682836516</v>
+        <v>1657555.360205131</v>
       </c>
       <c r="H66" t="n">
-        <v>158254568.2836516</v>
+        <v>165755536.0205131</v>
       </c>
       <c r="I66" t="n">
-        <v>6548246325.293603</v>
+        <v>6858620837.396226</v>
       </c>
       <c r="J66" t="n">
         <v>0</v>
@@ -2707,13 +2707,13 @@
         <v>10.28864736013324</v>
       </c>
       <c r="G67" t="n">
-        <v>965385.4029352755</v>
+        <v>1011142.848294296</v>
       </c>
       <c r="H67" t="n">
-        <v>8680056.211106654</v>
+        <v>9091474.486735553</v>
       </c>
       <c r="I67" t="n">
-        <v>22198904.01850975</v>
+        <v>23251090.15532997</v>
       </c>
       <c r="J67" t="n">
         <v>0</v>
@@ -2741,13 +2741,13 @@
         <v>2.211827734792698</v>
       </c>
       <c r="G68" t="n">
-        <v>579838.7586116429</v>
+        <v>607322.0209787179</v>
       </c>
       <c r="H68" t="n">
-        <v>11016936.41362121</v>
+        <v>11539118.39859564</v>
       </c>
       <c r="I68" t="n">
-        <v>1264246406.659165</v>
+        <v>1324169299.316497</v>
       </c>
       <c r="J68" t="n">
         <v>0.8500069992404432</v>
@@ -2775,13 +2775,13 @@
         <v>2.569399862184858</v>
       </c>
       <c r="G69" t="n">
-        <v>745899.5545392873</v>
+        <v>781253.7850946437</v>
       </c>
       <c r="H69" t="n">
-        <v>22376986.63617862</v>
+        <v>23437613.55283931</v>
       </c>
       <c r="I69" t="n">
-        <v>1973680997.430003</v>
+        <v>2067229750.20941</v>
       </c>
       <c r="J69" t="n">
         <v>-0.6941248011433353</v>
@@ -2809,13 +2809,13 @@
         <v>2.118769808888522</v>
       </c>
       <c r="G70" t="n">
-        <v>841883.528693596</v>
+        <v>881787.2183969294</v>
       </c>
       <c r="H70" t="n">
-        <v>30560029.07059461</v>
+        <v>32008516.74827868</v>
       </c>
       <c r="I70" t="n">
-        <v>3926814752.89656</v>
+        <v>4112938357.981468</v>
       </c>
       <c r="J70" t="n">
         <v>1.033802837172117</v>
@@ -2843,13 +2843,13 @@
         <v>2.374455858833616</v>
       </c>
       <c r="G71" t="n">
-        <v>773099.7477370552</v>
+        <v>809743.2160934155</v>
       </c>
       <c r="H71" t="n">
-        <v>28604690.66627104</v>
+        <v>29960498.99545638</v>
       </c>
       <c r="I71" t="n">
-        <v>1708280234.448134</v>
+        <v>1789249492.164263</v>
       </c>
       <c r="J71" t="n">
         <v>0.4404970943555943</v>
@@ -2877,13 +2877,13 @@
         <v>1.800774401633875</v>
       </c>
       <c r="G72" t="n">
-        <v>797086.4716140219</v>
+        <v>834866.8653929182</v>
       </c>
       <c r="H72" t="n">
-        <v>39854323.58070108</v>
+        <v>41743343.2696459</v>
       </c>
       <c r="I72" t="n">
-        <v>5675689353.641687</v>
+        <v>5944706312.759151</v>
       </c>
       <c r="J72" t="n">
         <v>0.5606894324126999</v>
@@ -2911,13 +2911,13 @@
         <v>1.662943479721646</v>
       </c>
       <c r="G73" t="n">
-        <v>1105933.726486393</v>
+        <v>1158352.897013039</v>
       </c>
       <c r="H73" t="n">
-        <v>83395001.07435144</v>
+        <v>87347766.66752559</v>
       </c>
       <c r="I73" t="n">
-        <v>38668335589.62057</v>
+        <v>40501141687.0471</v>
       </c>
       <c r="J73" t="n">
         <v>-1.260124888013365</v>
@@ -2945,13 +2945,13 @@
         <v>3.208873931952691</v>
       </c>
       <c r="G74" t="n">
-        <v>466590.5124576276</v>
+        <v>488706.0217805386</v>
       </c>
       <c r="H74" t="n">
-        <v>7434108.763585576</v>
+        <v>7786471.482670101</v>
       </c>
       <c r="I74" t="n">
-        <v>1009921833.979157</v>
+        <v>1057790222.08061</v>
       </c>
       <c r="J74" t="n">
         <v>2.49562259711823</v>
@@ -2979,13 +2979,13 @@
         <v>3.384179807511537</v>
       </c>
       <c r="G75" t="n">
-        <v>466590.5124576276</v>
+        <v>488706.0217805386</v>
       </c>
       <c r="H75" t="n">
-        <v>23329525.62288138</v>
+        <v>24435301.08902694</v>
       </c>
       <c r="I75" t="n">
-        <v>219507485.9004568</v>
+        <v>229911726.2809793</v>
       </c>
       <c r="J75" t="n">
         <v>0.7395250710411861</v>
@@ -3013,13 +3013,13 @@
         <v>1.89954363108434</v>
       </c>
       <c r="G76" t="n">
-        <v>910949.4013199486</v>
+        <v>954126.6829827881</v>
       </c>
       <c r="H76" t="n">
-        <v>18218988.02639897</v>
+        <v>19082533.65965576</v>
       </c>
       <c r="I76" t="n">
-        <v>1203755732.744985</v>
+        <v>1260811481.670971</v>
       </c>
       <c r="J76" t="n">
         <v>1.325854459725506</v>
@@ -3047,13 +3047,13 @@
         <v>2.273818170296539</v>
       </c>
       <c r="G77" t="n">
-        <v>825984.7024320868</v>
+        <v>865134.8177891315</v>
       </c>
       <c r="H77" t="n">
-        <v>24773642.84808076</v>
+        <v>25947866.74406912</v>
       </c>
       <c r="I77" t="n">
-        <v>2700137237.580015</v>
+        <v>2828118644.523567</v>
       </c>
       <c r="J77" t="n">
         <v>0.13557282597508</v>
@@ -3081,13 +3081,13 @@
         <v>3.55838836547066</v>
       </c>
       <c r="G78" t="n">
-        <v>1303863.370322874</v>
+        <v>1365664.032257243</v>
       </c>
       <c r="H78" t="n">
-        <v>42706007.14034805</v>
+        <v>44730191.24576841</v>
       </c>
       <c r="I78" t="n">
-        <v>15024513012.62612</v>
+        <v>15736646561.70489</v>
       </c>
       <c r="J78" t="n">
         <v>-0.3341193962242646</v>
@@ -3115,13 +3115,13 @@
         <v>2.355038326002673</v>
       </c>
       <c r="G79" t="n">
-        <v>1422601.007043102</v>
+        <v>1490029.608769978</v>
       </c>
       <c r="H79" t="n">
-        <v>69920259.36391877</v>
+        <v>73234347.64162143</v>
       </c>
       <c r="I79" t="n">
-        <v>31081470066.68366</v>
+        <v>32554673063.0518</v>
       </c>
       <c r="J79" t="n">
         <v>-0.4842784633623248</v>
@@ -3149,13 +3149,13 @@
         <v>2.113679823793869</v>
       </c>
       <c r="G80" t="n">
-        <v>1626102.170328671</v>
+        <v>1703176.342965594</v>
       </c>
       <c r="H80" t="n">
-        <v>114173032.1214947</v>
+        <v>119584618.2744327</v>
       </c>
       <c r="I80" t="n">
-        <v>15415472837.90128</v>
+        <v>16146137144.5285</v>
       </c>
       <c r="J80" t="n">
         <v>-1.06814992589538</v>
@@ -3183,13 +3183,13 @@
         <v>1.664294268071398</v>
       </c>
       <c r="G81" t="n">
-        <v>1807226.626298269</v>
+        <v>1892885.756167829</v>
       </c>
       <c r="H81" t="n">
-        <v>183287404.1753487</v>
+        <v>191974881.0690847</v>
       </c>
       <c r="I81" t="n">
-        <v>90040742719.74315</v>
+        <v>94308503919.11206</v>
       </c>
       <c r="J81" t="n">
         <v>-1.326873824072968</v>
@@ -3217,13 +3217,13 @@
         <v>1.538340835265424</v>
       </c>
       <c r="G82" t="n">
-        <v>1807226.626298269</v>
+        <v>1892885.756167829</v>
       </c>
       <c r="H82" t="n">
-        <v>207831062.0243008</v>
+        <v>217681861.9593002</v>
       </c>
       <c r="I82" t="n">
-        <v>56422741540.52489</v>
+        <v>59097072958.00522</v>
       </c>
       <c r="J82" t="n">
         <v>-0.1166760577335978</v>
@@ -3251,13 +3251,13 @@
         <v>1.929169690711981</v>
       </c>
       <c r="G83" t="n">
-        <v>1664730.338771904</v>
+        <v>1743635.413659354</v>
       </c>
       <c r="H83" t="n">
-        <v>125758516.5335715</v>
+        <v>131719232.7731376</v>
       </c>
       <c r="I83" t="n">
-        <v>79299275412.06366</v>
+        <v>83057911341.96773</v>
       </c>
       <c r="J83" t="n">
         <v>1.5106373641421</v>
@@ -3285,13 +3285,13 @@
         <v>1.886327114619066</v>
       </c>
       <c r="G84" t="n">
-        <v>1664730.338771904</v>
+        <v>1743635.413659354</v>
       </c>
       <c r="H84" t="n">
-        <v>133178427.1017523</v>
+        <v>139490833.0927483</v>
       </c>
       <c r="I84" t="n">
-        <v>10642045561.6508</v>
+        <v>11146458428.07166</v>
       </c>
       <c r="J84" t="n">
         <v>0.1540710305347492</v>
@@ -3319,13 +3319,13 @@
         <v>1.886505995483197</v>
       </c>
       <c r="G85" t="n">
-        <v>1807226.626298269</v>
+        <v>1892885.756167829</v>
       </c>
       <c r="H85" t="n">
-        <v>180722662.6298268</v>
+        <v>189288575.6167828</v>
       </c>
       <c r="I85" t="n">
-        <v>12354802697.22079</v>
+        <v>12940397018.01814</v>
       </c>
       <c r="J85" t="n">
         <v>-0.242195679044257</v>
@@ -3353,13 +3353,13 @@
         <v>2.176923010599811</v>
       </c>
       <c r="G86" t="n">
-        <v>773099.7477370552</v>
+        <v>809743.2160934155</v>
       </c>
       <c r="H86" t="n">
-        <v>46385984.86422332</v>
+        <v>48584592.96560494</v>
       </c>
       <c r="I86" t="n">
-        <v>183488370.3082953</v>
+        <v>192185372.6172897</v>
       </c>
       <c r="J86" t="n">
         <v>0.1217130551185047</v>
@@ -3387,13 +3387,13 @@
         <v>2.803339255488408</v>
       </c>
       <c r="G87" t="n">
-        <v>1298434.800743027</v>
+        <v>1359978.15872897</v>
       </c>
       <c r="H87" t="n">
-        <v>103874784.0594421</v>
+        <v>108798252.6983176</v>
       </c>
       <c r="I87" t="n">
-        <v>70329136.63445766</v>
+        <v>73662604.92278442</v>
       </c>
       <c r="J87" t="n">
         <v>-0.3300007082497931</v>
@@ -3421,13 +3421,13 @@
         <v>2.313212370015794</v>
       </c>
       <c r="G88" t="n">
-        <v>745899.5545392873</v>
+        <v>781253.7850946437</v>
       </c>
       <c r="H88" t="n">
-        <v>33565479.95426793</v>
+        <v>35156420.32925897</v>
       </c>
       <c r="I88" t="n">
-        <v>2261900972.518727</v>
+        <v>2369110807.930419</v>
       </c>
       <c r="J88" t="n">
         <v>0.3942829371039798</v>
@@ -3455,13 +3455,13 @@
         <v>2.353526411073462</v>
       </c>
       <c r="G89" t="n">
-        <v>1626102.170328671</v>
+        <v>1703176.342965594</v>
       </c>
       <c r="H89" t="n">
-        <v>121957662.7746504</v>
+        <v>127738225.7224196</v>
       </c>
       <c r="I89" t="n">
-        <v>2838140430.824845</v>
+        <v>2972662928.564954</v>
       </c>
       <c r="J89" t="n">
         <v>0.2229042444227899</v>
@@ -3489,13 +3489,13 @@
         <v>1.653622329073557</v>
       </c>
       <c r="G90" t="n">
-        <v>3359294.709176114</v>
+        <v>3518518.935720877</v>
       </c>
       <c r="H90" t="n">
-        <v>537487153.4681783</v>
+        <v>562963029.7153403</v>
       </c>
       <c r="I90" t="n">
-        <v>2204250916.509902</v>
+        <v>2308728248.115604</v>
       </c>
       <c r="J90" t="n">
         <v>-0.4019223458759687</v>
@@ -3523,13 +3523,13 @@
         <v>1.621291185719461</v>
       </c>
       <c r="G91" t="n">
-        <v>3561889.969115667</v>
+        <v>3730716.828462308</v>
       </c>
       <c r="H91" t="n">
-        <v>926091391.9700736</v>
+        <v>969986375.4002001</v>
       </c>
       <c r="I91" t="n">
-        <v>12770760930.66539</v>
+        <v>13376070886.35903</v>
       </c>
       <c r="J91" t="n">
         <v>-1.111236709763408</v>
@@ -3557,13 +3557,13 @@
         <v>2.704362102058114</v>
       </c>
       <c r="G92" t="n">
-        <v>787487.9700023335</v>
+        <v>824813.4129277262</v>
       </c>
       <c r="H92" t="n">
-        <v>12598634.2575495</v>
+        <v>13195785.7339291</v>
       </c>
       <c r="I92" t="n">
-        <v>330287785.7561088</v>
+        <v>345942803.1859718</v>
       </c>
       <c r="J92" t="n">
         <v>0.008433295864435024</v>
@@ -3591,13 +3591,13 @@
         <v>2.903794056576392</v>
       </c>
       <c r="G93" t="n">
-        <v>825984.7024320868</v>
+        <v>865134.8177891315</v>
       </c>
       <c r="H93" t="n">
-        <v>12389770.53648131</v>
+        <v>12977022.26683698</v>
       </c>
       <c r="I93" t="n">
-        <v>666174472.0476688</v>
+        <v>697749884.2215148</v>
       </c>
       <c r="J93" t="n">
         <v>0.2987928189149225</v>
@@ -3625,13 +3625,13 @@
         <v>2.106414806033488</v>
       </c>
       <c r="G94" t="n">
-        <v>825984.7024320868</v>
+        <v>865134.8177891315</v>
       </c>
       <c r="H94" t="n">
-        <v>23953556.37053053</v>
+        <v>25088909.71588482</v>
       </c>
       <c r="I94" t="n">
-        <v>911170571.7706938</v>
+        <v>954358336.4953076</v>
       </c>
       <c r="J94" t="n">
         <v>-0.3451456876604662</v>
@@ -3659,13 +3659,13 @@
         <v>2.043090480942521</v>
       </c>
       <c r="G95" t="n">
-        <v>1417044.684538699</v>
+        <v>1484209.927069736</v>
       </c>
       <c r="H95" t="n">
-        <v>212556702.6808049</v>
+        <v>222631489.0604604</v>
       </c>
       <c r="I95" t="n">
-        <v>9515381633.132143</v>
+        <v>9966392756.590641</v>
       </c>
       <c r="J95" t="n">
         <v>-0.2228894695439083</v>
@@ -3693,13 +3693,13 @@
         <v>1.855077351120051</v>
       </c>
       <c r="G96" t="n">
-        <v>1614436.169200317</v>
+        <v>1690957.395410284</v>
       </c>
       <c r="H96" t="n">
-        <v>242165425.3800476</v>
+        <v>253643609.3115426</v>
       </c>
       <c r="I96" t="n">
-        <v>13629133657.54766</v>
+        <v>14275128859.80559</v>
       </c>
       <c r="J96" t="n">
         <v>-0.05633405688587591</v>
@@ -3727,13 +3727,13 @@
         <v>1.670513388775463</v>
       </c>
       <c r="G97" t="n">
-        <v>1874539.563609697</v>
+        <v>1963389.199614546</v>
       </c>
       <c r="H97" t="n">
-        <v>266885871.9917287</v>
+        <v>279535758.4180463</v>
       </c>
       <c r="I97" t="n">
-        <v>2289197019.916382</v>
+        <v>2397700636.437171</v>
       </c>
       <c r="J97" t="n">
         <v>-0.4896919372250297</v>
@@ -3761,13 +3761,13 @@
         <v>1.780474223446541</v>
       </c>
       <c r="G98" t="n">
-        <v>1874539.563609697</v>
+        <v>1963389.199614546</v>
       </c>
       <c r="H98" t="n">
-        <v>262435538.9053576</v>
+        <v>274874487.9460363</v>
       </c>
       <c r="I98" t="n">
-        <v>2507379119.49931</v>
+        <v>2626224155.591627</v>
       </c>
       <c r="J98" t="n">
         <v>-0.2499201623741735</v>
@@ -3795,13 +3795,13 @@
         <v>2.011201253621685</v>
       </c>
       <c r="G99" t="n">
-        <v>1418135.826246649</v>
+        <v>1485352.786834463</v>
       </c>
       <c r="H99" t="n">
-        <v>60782129.92996614</v>
+        <v>63663088.12616313</v>
       </c>
       <c r="I99" t="n">
-        <v>1650775275.057275</v>
+        <v>1729018906.273149</v>
       </c>
       <c r="J99" t="n">
         <v>0.3145632119546559</v>
@@ -3829,13 +3829,13 @@
         <v>1.97942671109101</v>
       </c>
       <c r="G100" t="n">
-        <v>865288.8023927008</v>
+        <v>906301.8578779731</v>
       </c>
       <c r="H100" t="n">
-        <v>28533557.7507426</v>
+        <v>29885994.51403764</v>
       </c>
       <c r="I100" t="n">
-        <v>4999289683.260242</v>
+        <v>5236246575.108992</v>
       </c>
       <c r="J100" t="n">
         <v>0.6206152799119374</v>
@@ -3863,13 +3863,13 @@
         <v>3.550313974429316</v>
       </c>
       <c r="G101" t="n">
-        <v>772607.2963376029</v>
+        <v>809227.4234274246</v>
       </c>
       <c r="H101" t="n">
-        <v>20860397.00111528</v>
+        <v>21849140.43254047</v>
       </c>
       <c r="I101" t="n">
-        <v>201925220.5526807</v>
+        <v>211496094.7527197</v>
       </c>
       <c r="J101" t="n">
         <v>0.01747954020451694</v>
@@ -3897,13 +3897,13 @@
         <v>6.027772899553292</v>
       </c>
       <c r="G102" t="n">
-        <v>441386.0745605513</v>
+        <v>462306.9411155339</v>
       </c>
       <c r="H102" t="n">
-        <v>13241582.23681654</v>
+        <v>13869208.23346602</v>
       </c>
       <c r="I102" t="n">
-        <v>346454213.9089898</v>
+        <v>362875489.5095346</v>
       </c>
       <c r="J102" t="n">
         <v>0.4867669899500718</v>
@@ -3931,13 +3931,13 @@
         <v>2.345739057351345</v>
       </c>
       <c r="G103" t="n">
-        <v>1261956.182411344</v>
+        <v>1321770.522763492</v>
       </c>
       <c r="H103" t="n">
-        <v>117357540.0704998</v>
+        <v>122920065.8875646</v>
       </c>
       <c r="I103" t="n">
-        <v>22909887562.38569</v>
+        <v>23995772976.78061</v>
       </c>
       <c r="J103" t="n">
         <v>-0.8185617128641272</v>
@@ -3965,13 +3965,13 @@
         <v>4.370135818413353</v>
       </c>
       <c r="G104" t="n">
-        <v>1298434.800743027</v>
+        <v>1359978.15872897</v>
       </c>
       <c r="H104" t="n">
-        <v>103874784.0594421</v>
+        <v>108798252.6983176</v>
       </c>
       <c r="I104" t="n">
-        <v>1247352785.630842</v>
+        <v>1306474952.548206</v>
       </c>
       <c r="J104" t="n">
         <v>0.8031375102129624</v>
@@ -3999,13 +3999,13 @@
         <v>3.271437003499027</v>
       </c>
       <c r="G105" t="n">
-        <v>1766739.929494315</v>
+        <v>1850480.06637813</v>
       </c>
       <c r="H105" t="n">
-        <v>229676190.834261</v>
+        <v>240562408.6291569</v>
       </c>
       <c r="I105" t="n">
-        <v>2693837169.144162</v>
+        <v>2821519964.738987</v>
       </c>
       <c r="J105" t="n">
         <v>-0.7984587759301017</v>
@@ -4033,13 +4033,13 @@
         <v>2.111058972320168</v>
       </c>
       <c r="G106" t="n">
-        <v>1720323.5500158</v>
+        <v>1801863.638150904</v>
       </c>
       <c r="H106" t="n">
-        <v>258048532.5023701</v>
+        <v>270279545.7226356</v>
       </c>
       <c r="I106" t="n">
-        <v>8955576354.601547</v>
+        <v>9380053764.823683</v>
       </c>
       <c r="J106" t="n">
         <v>-1.17482502842645</v>
@@ -4067,13 +4067,13 @@
         <v>3.04765368496966</v>
       </c>
       <c r="G107" t="n">
-        <v>1558196.669655111</v>
+        <v>1632052.249772197</v>
       </c>
       <c r="H107" t="n">
-        <v>155819666.9655111</v>
+        <v>163205224.9772197</v>
       </c>
       <c r="I107" t="n">
-        <v>3785481243.660276</v>
+        <v>3964905907.258588</v>
       </c>
       <c r="J107" t="n">
         <v>-0.06387731674032879</v>

</xml_diff>

<commit_message>
Update to the graphs and segmentation flexibility
</commit_message>
<xml_diff>
--- a/aeromaps/utils/calibration_notebooks/fleet_calibrated_inputs_processed_here/aircraft_type_key_parameters.xlsx
+++ b/aeromaps/utils/calibration_notebooks/fleet_calibrated_inputs_processed_here/aircraft_type_key_parameters.xlsx
@@ -497,13 +497,13 @@
         <v>1.178449744963836</v>
       </c>
       <c r="G2" t="n">
-        <v>2124883.488884532</v>
+        <v>1883429.961753126</v>
       </c>
       <c r="H2" t="n">
-        <v>297483688.4438344</v>
+        <v>263680194.6454376</v>
       </c>
       <c r="I2" t="n">
-        <v>6722308750.491856</v>
+        <v>5958443264.801326</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -531,13 +531,13 @@
         <v>0.8524547275953843</v>
       </c>
       <c r="G3" t="n">
-        <v>2297477.017010296</v>
+        <v>2036411.442280038</v>
       </c>
       <c r="H3" t="n">
-        <v>420181172.7495064</v>
+        <v>372435389.6393757</v>
       </c>
       <c r="I3" t="n">
-        <v>851401145339.9662</v>
+        <v>754655224624.1106</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -565,13 +565,13 @@
         <v>0.8330292323059032</v>
       </c>
       <c r="G4" t="n">
-        <v>2589260.082682253</v>
+        <v>2295038.784011247</v>
       </c>
       <c r="H4" t="n">
-        <v>513809673.1967819</v>
+        <v>455424750.6744066</v>
       </c>
       <c r="I4" t="n">
-        <v>794868552041.4155</v>
+        <v>704546510150.552</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -599,13 +599,13 @@
         <v>1.229639562991454</v>
       </c>
       <c r="G5" t="n">
-        <v>2734630.67468466</v>
+        <v>2423890.709289678</v>
       </c>
       <c r="H5" t="n">
-        <v>733127083.7412435</v>
+        <v>649820812.5358466</v>
       </c>
       <c r="I5" t="n">
-        <v>14055625549.96427</v>
+        <v>12458464866.64664</v>
       </c>
       <c r="J5" t="n">
         <v>-0.6243207238688866</v>
@@ -633,13 +633,13 @@
         <v>1.174570952133184</v>
       </c>
       <c r="G6" t="n">
-        <v>2824647.510250766</v>
+        <v>2503678.804050775</v>
       </c>
       <c r="H6" t="n">
-        <v>652447147.5223285</v>
+        <v>578308651.995315</v>
       </c>
       <c r="I6" t="n">
-        <v>11167050679.05036</v>
+        <v>9898122858.67028</v>
       </c>
       <c r="J6" t="n">
         <v>-0.4315208434238162</v>
@@ -667,13 +667,13 @@
         <v>1.680027915024445</v>
       </c>
       <c r="G7" t="n">
-        <v>2431036.052953514</v>
+        <v>2154793.975380886</v>
       </c>
       <c r="H7" t="n">
-        <v>231285854.8700822</v>
+        <v>205004514.8690359</v>
       </c>
       <c r="I7" t="n">
-        <v>5124259914.756726</v>
+        <v>4541982986.714145</v>
       </c>
       <c r="J7" t="n">
         <v>-2.693006512525284</v>
@@ -701,13 +701,13 @@
         <v>1.343098767003529</v>
       </c>
       <c r="G8" t="n">
-        <v>2124883.488884532</v>
+        <v>1883429.961753126</v>
       </c>
       <c r="H8" t="n">
-        <v>277715863.8509949</v>
+        <v>246158616.0216709</v>
       </c>
       <c r="I8" t="n">
-        <v>245005271223.1062</v>
+        <v>217164974467.0423</v>
       </c>
       <c r="J8" t="n">
         <v>-1.054220956300929</v>
@@ -735,13 +735,13 @@
         <v>1.129040999847672</v>
       </c>
       <c r="G9" t="n">
-        <v>2303226.12468929</v>
+        <v>2041507.270692563</v>
       </c>
       <c r="H9" t="n">
-        <v>362926968.4807361</v>
+        <v>321687061.874476</v>
       </c>
       <c r="I9" t="n">
-        <v>1242812424359.461</v>
+        <v>1101589884397.115</v>
       </c>
       <c r="J9" t="n">
         <v>-0.4964523917793309</v>
@@ -769,13 +769,13 @@
         <v>1.213652392088143</v>
       </c>
       <c r="G10" t="n">
-        <v>2411139.282201593</v>
+        <v>2137158.102933135</v>
       </c>
       <c r="H10" t="n">
-        <v>448834320.671774</v>
+        <v>397832639.6898587</v>
       </c>
       <c r="I10" t="n">
-        <v>666397039489.3988</v>
+        <v>590673397936.1815</v>
       </c>
       <c r="J10" t="n">
         <v>-0.1662883240459748</v>
@@ -803,13 +803,13 @@
         <v>1.158197581335016</v>
       </c>
       <c r="G11" t="n">
-        <v>3730716.828462308</v>
+        <v>3306790.179461147</v>
       </c>
       <c r="H11" t="n">
-        <v>980088950.2672037</v>
+        <v>868720051.6040766</v>
       </c>
       <c r="I11" t="n">
-        <v>384518614049.6555</v>
+        <v>340825218107.8819</v>
       </c>
       <c r="J11" t="n">
         <v>-1.42681980614188</v>
@@ -837,13 +837,13 @@
         <v>1.148368652583524</v>
       </c>
       <c r="G12" t="n">
-        <v>3843158.111275807</v>
+        <v>3406454.599697229</v>
       </c>
       <c r="H12" t="n">
-        <v>1108803887.556772</v>
+        <v>982808927.8575276</v>
       </c>
       <c r="I12" t="n">
-        <v>677053272006.7463</v>
+        <v>600118747625.9738</v>
       </c>
       <c r="J12" t="n">
         <v>-0.5285890937797832</v>
@@ -871,13 +871,13 @@
         <v>1.206911147835214</v>
       </c>
       <c r="G13" t="n">
-        <v>3809289.68610388</v>
+        <v>3376434.691754095</v>
       </c>
       <c r="H13" t="n">
-        <v>933275973.0954509</v>
+        <v>827226499.4797533</v>
       </c>
       <c r="I13" t="n">
-        <v>6322012036.031949</v>
+        <v>5603632834.229952</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -905,13 +905,13 @@
         <v>1.081850374244981</v>
       </c>
       <c r="G14" t="n">
-        <v>3809289.68610388</v>
+        <v>3376434.691754095</v>
       </c>
       <c r="H14" t="n">
-        <v>1041161701.054782</v>
+        <v>922853019.0263941</v>
       </c>
       <c r="I14" t="n">
-        <v>143857327671.0312</v>
+        <v>127510615321.1211</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -939,13 +939,13 @@
         <v>1.225404189833046</v>
       </c>
       <c r="G15" t="n">
-        <v>3861446.331045568</v>
+        <v>3422664.703094275</v>
       </c>
       <c r="H15" t="n">
-        <v>1071872910.655335</v>
+        <v>950074470.2852235</v>
       </c>
       <c r="I15" t="n">
-        <v>4804601051.130829</v>
+        <v>4258647413.520424</v>
       </c>
       <c r="J15" t="n">
         <v>-0.8585427768451319</v>
@@ -973,13 +973,13 @@
         <v>1.260179397395529</v>
       </c>
       <c r="G16" t="n">
-        <v>3899657.494209519</v>
+        <v>3456533.877546848</v>
       </c>
       <c r="H16" t="n">
-        <v>1080926854.162009</v>
+        <v>958099601.339088</v>
       </c>
       <c r="I16" t="n">
-        <v>57184911313.22714</v>
+        <v>50686908666.25677</v>
       </c>
       <c r="J16" t="n">
         <v>-1.363064396189034</v>
@@ -1007,13 +1007,13 @@
         <v>2.076914867607091</v>
       </c>
       <c r="G17" t="n">
-        <v>4082281.463561768</v>
+        <v>3618406.026025387</v>
       </c>
       <c r="H17" t="n">
-        <v>834659167.8689139</v>
+        <v>739815661.8184677</v>
       </c>
       <c r="I17" t="n">
-        <v>13214748708.62646</v>
+        <v>11713138054.42158</v>
       </c>
       <c r="J17" t="n">
         <v>-1.85691811720076</v>
@@ -1041,13 +1041,13 @@
         <v>1.428662850478296</v>
       </c>
       <c r="G18" t="n">
-        <v>3873498.523993163</v>
+        <v>3433347.388249048</v>
       </c>
       <c r="H18" t="n">
-        <v>1172687846.019579</v>
+        <v>1039433661.436405</v>
       </c>
       <c r="I18" t="n">
-        <v>49580698540.3269</v>
+        <v>43946773384.98328</v>
       </c>
       <c r="J18" t="n">
         <v>-2.019125475237955</v>
@@ -1075,13 +1075,13 @@
         <v>1.097180837791816</v>
       </c>
       <c r="G19" t="n">
-        <v>3901823.624137151</v>
+        <v>3458453.867055964</v>
       </c>
       <c r="H19" t="n">
-        <v>1154329166.42612</v>
+        <v>1023161104.665447</v>
       </c>
       <c r="I19" t="n">
-        <v>596176046391.5223</v>
+        <v>528431715963.2897</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1109,13 +1109,13 @@
         <v>0.9984880328710761</v>
       </c>
       <c r="G20" t="n">
-        <v>3906657.686831765</v>
+        <v>3462738.628344598</v>
       </c>
       <c r="H20" t="n">
-        <v>1324317499.305431</v>
+        <v>1173833421.979856</v>
       </c>
       <c r="I20" t="n">
-        <v>118765680044.2216</v>
+        <v>105270167231.9445</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1143,13 +1143,13 @@
         <v>1.412066518413993</v>
       </c>
       <c r="G21" t="n">
-        <v>3927901.438206434</v>
+        <v>3481568.422094884</v>
       </c>
       <c r="H21" t="n">
-        <v>1855640123.226541</v>
+        <v>1644781101.928008</v>
       </c>
       <c r="I21" t="n">
-        <v>378262631991.8649</v>
+        <v>335280112171.7357</v>
       </c>
       <c r="J21" t="n">
         <v>-1.786346028204582</v>
@@ -1177,13 +1177,13 @@
         <v>2.729543634431751</v>
       </c>
       <c r="G22" t="n">
-        <v>1359978.15872897</v>
+        <v>1205441.910052501</v>
       </c>
       <c r="H22" t="n">
-        <v>108798252.6983176</v>
+        <v>96435352.80420002</v>
       </c>
       <c r="I22" t="n">
-        <v>15953575572.04354</v>
+        <v>14140748133.56149</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1211,13 +1211,13 @@
         <v>2.41333855030665</v>
       </c>
       <c r="G23" t="n">
-        <v>781253.7850946437</v>
+        <v>692478.8084982146</v>
       </c>
       <c r="H23" t="n">
-        <v>32414482.15468782</v>
+        <v>28731178.53482865</v>
       </c>
       <c r="I23" t="n">
-        <v>1301055121.183628</v>
+        <v>1153214380.905169</v>
       </c>
       <c r="J23" t="n">
         <v>-0.1490941480697875</v>
@@ -1245,13 +1245,13 @@
         <v>4.028249795385581</v>
       </c>
       <c r="G24" t="n">
-        <v>488706.0217805386</v>
+        <v>433173.6628034291</v>
       </c>
       <c r="H24" t="n">
-        <v>20525652.91478262</v>
+        <v>18193293.83774402</v>
       </c>
       <c r="I24" t="n">
-        <v>1563150353.43225</v>
+        <v>1385527359.867058</v>
       </c>
       <c r="J24" t="n">
         <v>-0.2286593211176034</v>
@@ -1279,13 +1279,13 @@
         <v>3.759699809026542</v>
       </c>
       <c r="G25" t="n">
-        <v>488706.0217805386</v>
+        <v>433173.6628034291</v>
       </c>
       <c r="H25" t="n">
-        <v>21991770.98012424</v>
+        <v>19492814.82615431</v>
       </c>
       <c r="I25" t="n">
-        <v>1462966828.685704</v>
+        <v>1296727831.248793</v>
       </c>
       <c r="J25" t="n">
         <v>-1.917517451853091</v>
@@ -1313,13 +1313,13 @@
         <v>1.587888411702909</v>
       </c>
       <c r="G26" t="n">
-        <v>895682.4954052556</v>
+        <v>793904.8220237433</v>
       </c>
       <c r="H26" t="n">
-        <v>58295750.24044749</v>
+        <v>51671521.38933215</v>
       </c>
       <c r="I26" t="n">
-        <v>1197542133.309225</v>
+        <v>1061463720.780465</v>
       </c>
       <c r="J26" t="n">
         <v>-0.6379947226602307</v>
@@ -1347,13 +1347,13 @@
         <v>1.476402419913499</v>
       </c>
       <c r="G27" t="n">
-        <v>895682.4954052556</v>
+        <v>793904.8220237433</v>
       </c>
       <c r="H27" t="n">
-        <v>62697774.67836787</v>
+        <v>55573337.54166202</v>
       </c>
       <c r="I27" t="n">
-        <v>14111242566.17124</v>
+        <v>12507762042.3532</v>
       </c>
       <c r="J27" t="n">
         <v>-0.8649438723091367</v>
@@ -1381,13 +1381,13 @@
         <v>1.476402419913499</v>
       </c>
       <c r="G28" t="n">
-        <v>895682.4954052556</v>
+        <v>793904.8220237433</v>
       </c>
       <c r="H28" t="n">
-        <v>62697774.67836787</v>
+        <v>55573337.54166202</v>
       </c>
       <c r="I28" t="n">
-        <v>34069475635.54146</v>
+        <v>30198112757.17613</v>
       </c>
       <c r="J28" t="n">
         <v>-0.6152740745620315</v>
@@ -1415,13 +1415,13 @@
         <v>2.967918644423394</v>
       </c>
       <c r="G29" t="n">
-        <v>954126.6829827881</v>
+        <v>845707.9136048395</v>
       </c>
       <c r="H29" t="n">
-        <v>16297526.93920688</v>
+        <v>14445615.81863228</v>
       </c>
       <c r="I29" t="n">
-        <v>5613664718.14337</v>
+        <v>4975776027.577851</v>
       </c>
       <c r="J29" t="n">
         <v>1.057632377297526</v>
@@ -1449,13 +1449,13 @@
         <v>0.8763039646656254</v>
       </c>
       <c r="G30" t="n">
-        <v>2305283.18820504</v>
+        <v>2043330.587160999</v>
       </c>
       <c r="H30" t="n">
-        <v>396335935.6642486</v>
+        <v>351299720.6926244</v>
       </c>
       <c r="I30" t="n">
-        <v>551532332744.8994</v>
+        <v>488860930870.4484</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1483,13 +1483,13 @@
         <v>0.7851654512067765</v>
       </c>
       <c r="G31" t="n">
-        <v>2565101.43370743</v>
+        <v>2273625.316612833</v>
       </c>
       <c r="H31" t="n">
-        <v>456728144.2079134</v>
+        <v>404829476.8522395</v>
       </c>
       <c r="I31" t="n">
-        <v>104135560945.6457</v>
+        <v>92302489334.11327</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1517,13 +1517,13 @@
         <v>0.7358017415760942</v>
       </c>
       <c r="G32" t="n">
-        <v>2565101.43370743</v>
+        <v>2273625.316612833</v>
       </c>
       <c r="H32" t="n">
-        <v>487369272.4044116</v>
+        <v>431988810.1564381</v>
       </c>
       <c r="I32" t="n">
-        <v>487369272.4044116</v>
+        <v>431988810.1564381</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1551,13 +1551,13 @@
         <v>2.922741166837872</v>
       </c>
       <c r="G33" t="n">
-        <v>1526861.65855599</v>
+        <v>1353362.200901686</v>
       </c>
       <c r="H33" t="n">
-        <v>122148932.6844791</v>
+        <v>108268976.0721348</v>
       </c>
       <c r="I33" t="n">
-        <v>8862355412.604656</v>
+        <v>7855313386.884544</v>
       </c>
       <c r="J33" t="n">
         <v>-0.2964742868686928</v>
@@ -1585,13 +1585,13 @@
         <v>2.623618271687993</v>
       </c>
       <c r="G34" t="n">
-        <v>1526861.65855599</v>
+        <v>1353362.200901686</v>
       </c>
       <c r="H34" t="n">
-        <v>137417549.2700391</v>
+        <v>121802598.0811517</v>
       </c>
       <c r="I34" t="n">
-        <v>2977689932.577649</v>
+        <v>2639330798.683686</v>
       </c>
       <c r="J34" t="n">
         <v>0.4428404390783032</v>
@@ -1619,13 +1619,13 @@
         <v>2.488394116576957</v>
       </c>
       <c r="G35" t="n">
-        <v>1526861.65855599</v>
+        <v>1353362.200901686</v>
       </c>
       <c r="H35" t="n">
-        <v>152686165.855599</v>
+        <v>135336220.0901686</v>
       </c>
       <c r="I35" t="n">
-        <v>1309667098.049972</v>
+        <v>1160847766.615418</v>
       </c>
       <c r="J35" t="n">
         <v>-0.6045605979355976</v>
@@ -1653,13 +1653,13 @@
         <v>1.889656157541419</v>
       </c>
       <c r="G36" t="n">
-        <v>1526861.65855599</v>
+        <v>1353362.200901686</v>
       </c>
       <c r="H36" t="n">
-        <v>174201534.4080173</v>
+        <v>154406766.7727343</v>
       </c>
       <c r="I36" t="n">
-        <v>16836400008.72615</v>
+        <v>14923255976.32737</v>
       </c>
       <c r="J36" t="n">
         <v>-0.2585451858503126</v>
@@ -1687,13 +1687,13 @@
         <v>12.48206279236391</v>
       </c>
       <c r="G37" t="n">
-        <v>1682058.77689968</v>
+        <v>1490924.050384406</v>
       </c>
       <c r="H37" t="n">
-        <v>54291254.17607365</v>
+        <v>48122061.89716796</v>
       </c>
       <c r="I37" t="n">
-        <v>281839881.153957</v>
+        <v>249814015.3844211</v>
       </c>
       <c r="J37" t="n">
         <v>0.0752079882855939</v>
@@ -1721,13 +1721,13 @@
         <v>2.424017752474225</v>
       </c>
       <c r="G38" t="n">
-        <v>1484209.927069736</v>
+        <v>1315557.046208696</v>
       </c>
       <c r="H38" t="n">
-        <v>169239491.1537319</v>
+        <v>150008567.5370942</v>
       </c>
       <c r="I38" t="n">
-        <v>5054211671.795984</v>
+        <v>4479894425.035085</v>
       </c>
       <c r="J38" t="n">
         <v>0.4353941581541733</v>
@@ -1755,13 +1755,13 @@
         <v>1.645469940597836</v>
       </c>
       <c r="G39" t="n">
-        <v>1690957.395410284</v>
+        <v>1498811.506241988</v>
       </c>
       <c r="H39" t="n">
-        <v>230821119.2018875</v>
+        <v>204592587.7745143</v>
       </c>
       <c r="I39" t="n">
-        <v>36695980581.96124</v>
+        <v>32526164218.18902</v>
       </c>
       <c r="J39" t="n">
         <v>-0.4956950334836177</v>
@@ -1789,13 +1789,13 @@
         <v>1.705966933028853</v>
       </c>
       <c r="G40" t="n">
-        <v>1850480.06637813</v>
+        <v>1640207.389664024</v>
       </c>
       <c r="H40" t="n">
-        <v>258661752.6964734</v>
+        <v>229269650.5651039</v>
       </c>
       <c r="I40" t="n">
-        <v>22354979450.45643</v>
+        <v>19814751402.42527</v>
       </c>
       <c r="J40" t="n">
         <v>-0.02443755020506672</v>
@@ -1823,13 +1823,13 @@
         <v>1.747985551995309</v>
       </c>
       <c r="G41" t="n">
-        <v>1894626.338519917</v>
+        <v>1679337.258236347</v>
       </c>
       <c r="H41" t="n">
-        <v>223093307.078653</v>
+        <v>197742897.9125353</v>
       </c>
       <c r="I41" t="n">
-        <v>23042057565.04193</v>
+        <v>20423755855.53743</v>
       </c>
       <c r="J41" t="n">
         <v>-0.4467128126006354</v>
@@ -1857,13 +1857,13 @@
         <v>1.477731589399572</v>
       </c>
       <c r="G42" t="n">
-        <v>2239910.412470728</v>
+        <v>1985386.212730566</v>
       </c>
       <c r="H42" t="n">
-        <v>256962863.613918</v>
+        <v>227763808.6605862</v>
       </c>
       <c r="I42" t="n">
-        <v>4537925091.42903</v>
+        <v>4022274221.668242</v>
       </c>
       <c r="J42" t="n">
         <v>-1.86319444881112</v>
@@ -1891,13 +1891,13 @@
         <v>1.436323561650747</v>
       </c>
       <c r="G43" t="n">
-        <v>1973881.084201755</v>
+        <v>1749586.174663599</v>
       </c>
       <c r="H43" t="n">
-        <v>273585111.9069527</v>
+        <v>242497247.2846662</v>
       </c>
       <c r="I43" t="n">
-        <v>193794788835.3878</v>
+        <v>171773611886.7381</v>
       </c>
       <c r="J43" t="n">
         <v>-1.056465935146006</v>
@@ -1925,13 +1925,13 @@
         <v>1.158904218673777</v>
       </c>
       <c r="G44" t="n">
-        <v>2319157.670240306</v>
+        <v>2055628.492107657</v>
       </c>
       <c r="H44" t="n">
-        <v>385281960.7522787</v>
+        <v>341501824.6411092</v>
       </c>
       <c r="I44" t="n">
-        <v>1625198042117.81</v>
+        <v>1440524481610.077</v>
       </c>
       <c r="J44" t="n">
         <v>0.4649960614078142</v>
@@ -1959,13 +1959,13 @@
         <v>1.085212054990146</v>
       </c>
       <c r="G45" t="n">
-        <v>2367476.099415245</v>
+        <v>2098456.429587043</v>
       </c>
       <c r="H45" t="n">
-        <v>422760609.772912</v>
+        <v>374721721.5722797</v>
       </c>
       <c r="I45" t="n">
-        <v>207060652467.4952</v>
+        <v>183532056603.3275</v>
       </c>
       <c r="J45" t="n">
         <v>0.1791196930766627</v>
@@ -1993,13 +1993,13 @@
         <v>1.544157495477784</v>
       </c>
       <c r="G46" t="n">
-        <v>3824847.421160877</v>
+        <v>3390224.579292233</v>
       </c>
       <c r="H46" t="n">
-        <v>1281416544.136279</v>
+        <v>1135807363.24483</v>
       </c>
       <c r="I46" t="n">
-        <v>58674774152.23545</v>
+        <v>52007476275.99611</v>
       </c>
       <c r="J46" t="n">
         <v>-1.030542493092959</v>
@@ -2027,13 +2027,13 @@
         <v>1.241535095777449</v>
       </c>
       <c r="G47" t="n">
-        <v>3885497.324969647</v>
+        <v>3443982.748438179</v>
       </c>
       <c r="H47" t="n">
-        <v>1419599953.189121</v>
+        <v>1258288795.374521</v>
       </c>
       <c r="I47" t="n">
-        <v>50088006544.12009</v>
+        <v>44396435260.1776</v>
       </c>
       <c r="J47" t="n">
         <v>0</v>
@@ -2061,13 +2061,13 @@
         <v>1.324212276281809</v>
       </c>
       <c r="G48" t="n">
-        <v>2625943.697002884</v>
+        <v>2327553.987163935</v>
       </c>
       <c r="H48" t="n">
-        <v>470298708.1067632</v>
+        <v>416857998.3117368</v>
       </c>
       <c r="I48" t="n">
-        <v>80981258155.59061</v>
+        <v>71779242837.8139</v>
       </c>
       <c r="J48" t="n">
         <v>-0.1360243100705888</v>
@@ -2095,13 +2095,13 @@
         <v>1.163961944685927</v>
       </c>
       <c r="G49" t="n">
-        <v>2552426.278109258</v>
+        <v>2262390.456937767</v>
       </c>
       <c r="H49" t="n">
-        <v>583989586.6873152</v>
+        <v>517630020.9740506</v>
       </c>
       <c r="I49" t="n">
-        <v>25634763418.64521</v>
+        <v>22721848862.62864</v>
       </c>
       <c r="J49" t="n">
         <v>2.066449901832937</v>
@@ -2129,13 +2129,13 @@
         <v>1.383383760653715</v>
       </c>
       <c r="G50" t="n">
-        <v>3307851.345128164</v>
+        <v>2931975.501259267</v>
       </c>
       <c r="H50" t="n">
-        <v>641136830.7067136</v>
+        <v>568283542.5345454</v>
       </c>
       <c r="I50" t="n">
-        <v>11809514691.59454</v>
+        <v>10467582773.48615</v>
       </c>
       <c r="J50" t="n">
         <v>-0.04844023038190387</v>
@@ -2163,13 +2163,13 @@
         <v>1.174247232680542</v>
       </c>
       <c r="G51" t="n">
-        <v>3518518.935720877</v>
+        <v>3118704.634488565</v>
       </c>
       <c r="H51" t="n">
-        <v>784721400.4374709</v>
+        <v>695552393.7873281</v>
       </c>
       <c r="I51" t="n">
-        <v>143120108519.0982</v>
+        <v>126857167427.9109</v>
       </c>
       <c r="J51" t="n">
         <v>-0.1098505376682319</v>
@@ -2197,13 +2197,13 @@
         <v>1.224601924257454</v>
       </c>
       <c r="G52" t="n">
-        <v>3744038.20028379</v>
+        <v>3318597.824892758</v>
       </c>
       <c r="H52" t="n">
-        <v>895169503.4134271</v>
+        <v>793450122.0401427</v>
       </c>
       <c r="I52" t="n">
-        <v>27023154900.09105</v>
+        <v>23952475449.20475</v>
       </c>
       <c r="J52" t="n">
         <v>0</v>
@@ -2231,13 +2231,13 @@
         <v>1.242461676533537</v>
       </c>
       <c r="G53" t="n">
-        <v>3771994.255828743</v>
+        <v>3343377.194162289</v>
       </c>
       <c r="H53" t="n">
-        <v>1069004242.696722</v>
+        <v>947531773.1388456</v>
       </c>
       <c r="I53" t="n">
-        <v>314480468272.3628</v>
+        <v>278745606254.9826</v>
       </c>
       <c r="J53" t="n">
         <v>-0.4393742853662961</v>
@@ -2265,13 +2265,13 @@
         <v>1.249185074303995</v>
       </c>
       <c r="G54" t="n">
-        <v>3873845.608163427</v>
+        <v>3433655.032752356</v>
       </c>
       <c r="H54" t="n">
-        <v>1355845962.857199</v>
+        <v>1201779261.463325</v>
       </c>
       <c r="I54" t="n">
-        <v>55745386651.981</v>
+        <v>49410959235.68504</v>
       </c>
       <c r="J54" t="n">
         <v>0.322840932025079</v>
@@ -2299,13 +2299,13 @@
         <v>0.9757883476193243</v>
       </c>
       <c r="G55" t="n">
-        <v>3873845.608163427</v>
+        <v>3433655.032752356</v>
       </c>
       <c r="H55" t="n">
-        <v>1355845962.857199</v>
+        <v>1201779261.463325</v>
       </c>
       <c r="I55" t="n">
-        <v>60849801184.14905</v>
+        <v>53935351898.80474</v>
       </c>
       <c r="J55" t="n">
         <v>0</v>
@@ -2333,13 +2333,13 @@
         <v>1.251541412066441</v>
       </c>
       <c r="G56" t="n">
-        <v>3873845.608163427</v>
+        <v>3433655.032752356</v>
       </c>
       <c r="H56" t="n">
-        <v>1229761058.519429</v>
+        <v>1090021563.784006</v>
       </c>
       <c r="I56" t="n">
-        <v>879623779579.413</v>
+        <v>779670880872.6694</v>
       </c>
       <c r="J56" t="n">
         <v>-0.1746664338412045</v>
@@ -2367,13 +2367,13 @@
         <v>0.9949389212208551</v>
       </c>
       <c r="G57" t="n">
-        <v>3770006.829785835</v>
+        <v>3341615.602161804</v>
       </c>
       <c r="H57" t="n">
-        <v>912013688.2389414</v>
+        <v>808380278.2334759</v>
       </c>
       <c r="I57" t="n">
-        <v>326155351937.4335</v>
+        <v>289093856316.5987</v>
       </c>
       <c r="J57" t="n">
         <v>-0.429498513927575</v>
@@ -2401,13 +2401,13 @@
         <v>0.8812055291279901</v>
       </c>
       <c r="G58" t="n">
-        <v>3824161.260222423</v>
+        <v>3389616.387795227</v>
       </c>
       <c r="H58" t="n">
-        <v>1045879713.445957</v>
+        <v>927034916.9723028</v>
       </c>
       <c r="I58" t="n">
-        <v>633548021331.4971</v>
+        <v>561557060341.0116</v>
       </c>
       <c r="J58" t="n">
         <v>0.7135031330351608</v>
@@ -2435,13 +2435,13 @@
         <v>0.8828858610008796</v>
       </c>
       <c r="G59" t="n">
-        <v>3765356.473737092</v>
+        <v>3337493.672672098</v>
       </c>
       <c r="H59" t="n">
-        <v>1171986712.006684</v>
+        <v>1038812198.276661</v>
       </c>
       <c r="I59" t="n">
-        <v>132416974511.9857</v>
+        <v>117370245731.2126</v>
       </c>
       <c r="J59" t="n">
         <v>0</v>
@@ -2469,13 +2469,13 @@
         <v>1.559350380561198</v>
       </c>
       <c r="G60" t="n">
-        <v>2124883.488884532</v>
+        <v>1883429.961753126</v>
       </c>
       <c r="H60" t="n">
-        <v>233737183.7772985</v>
+        <v>207177295.7928438</v>
       </c>
       <c r="I60" t="n">
-        <v>15635919911.51924</v>
+        <v>13859188136.65737</v>
       </c>
       <c r="J60" t="n">
         <v>0</v>
@@ -2503,13 +2503,13 @@
         <v>1.260115242506681</v>
       </c>
       <c r="G61" t="n">
-        <v>2303226.12468929</v>
+        <v>2041507.270692563</v>
       </c>
       <c r="H61" t="n">
-        <v>322451657.4565007</v>
+        <v>285811017.8969588</v>
       </c>
       <c r="I61" t="n">
-        <v>99880934872.70358</v>
+        <v>88531322461.31596</v>
       </c>
       <c r="J61" t="n">
         <v>0</v>
@@ -2537,13 +2537,13 @@
         <v>1.186044863978063</v>
       </c>
       <c r="G62" t="n">
-        <v>2303226.12468929</v>
+        <v>2041507.270692563</v>
       </c>
       <c r="H62" t="n">
-        <v>345483918.7033936</v>
+        <v>306226090.6038845</v>
       </c>
       <c r="I62" t="n">
-        <v>5138310402.869585</v>
+        <v>4554436897.917957</v>
       </c>
       <c r="J62" t="n">
         <v>0</v>
@@ -2571,13 +2571,13 @@
         <v>2.426303926504643</v>
       </c>
       <c r="G63" t="n">
-        <v>1359978.15872897</v>
+        <v>1205441.910052501</v>
       </c>
       <c r="H63" t="n">
-        <v>67993341.23132817</v>
+        <v>60267161.35010949</v>
       </c>
       <c r="I63" t="n">
-        <v>30027479307.39659</v>
+        <v>26615414209.44514</v>
       </c>
       <c r="J63" t="n">
         <v>-1.339402047145975</v>
@@ -2605,13 +2605,13 @@
         <v>2.315458107421362</v>
       </c>
       <c r="G64" t="n">
-        <v>1632052.249772197</v>
+        <v>1446599.835919092</v>
       </c>
       <c r="H64" t="n">
-        <v>107368852.1273743</v>
+        <v>95168377.04917876</v>
       </c>
       <c r="I64" t="n">
-        <v>26972296659.79992</v>
+        <v>23907396302.95159</v>
       </c>
       <c r="J64" t="n">
         <v>-0.07908807757601682</v>
@@ -2639,13 +2639,13 @@
         <v>2.012412678660564</v>
       </c>
       <c r="G65" t="n">
-        <v>1657555.360205131</v>
+        <v>1469204.991711659</v>
       </c>
       <c r="H65" t="n">
-        <v>126615208.7282701</v>
+        <v>112227742.8291545</v>
       </c>
       <c r="I65" t="n">
-        <v>52537817308.88912</v>
+        <v>46567870550.21955</v>
       </c>
       <c r="J65" t="n">
         <v>0.0476991099844348</v>
@@ -2673,13 +2673,13 @@
         <v>1.556991741800394</v>
       </c>
       <c r="G66" t="n">
-        <v>1657555.360205131</v>
+        <v>1469204.991711659</v>
       </c>
       <c r="H66" t="n">
-        <v>165755536.0205131</v>
+        <v>146920499.1711659</v>
       </c>
       <c r="I66" t="n">
-        <v>6858620837.396226</v>
+        <v>6079266015.774632</v>
       </c>
       <c r="J66" t="n">
         <v>0</v>
@@ -2707,13 +2707,13 @@
         <v>10.28864736013324</v>
       </c>
       <c r="G67" t="n">
-        <v>1011142.848294296</v>
+        <v>896245.2511170888</v>
       </c>
       <c r="H67" t="n">
-        <v>9091474.486735553</v>
+        <v>8058397.335385551</v>
       </c>
       <c r="I67" t="n">
-        <v>23251090.15532997</v>
+        <v>20609035.77586757</v>
       </c>
       <c r="J67" t="n">
         <v>0</v>
@@ -2741,13 +2741,13 @@
         <v>2.211827734792698</v>
       </c>
       <c r="G68" t="n">
-        <v>607322.0209787179</v>
+        <v>538311.1576363404</v>
       </c>
       <c r="H68" t="n">
-        <v>11539118.39859564</v>
+        <v>10227911.99509046</v>
       </c>
       <c r="I68" t="n">
-        <v>1324169299.316497</v>
+        <v>1173702062.166034</v>
       </c>
       <c r="J68" t="n">
         <v>0.8500069992404432</v>
@@ -2775,13 +2775,13 @@
         <v>2.569399862184858</v>
       </c>
       <c r="G69" t="n">
-        <v>781253.7850946437</v>
+        <v>692478.8084982146</v>
       </c>
       <c r="H69" t="n">
-        <v>23437613.55283931</v>
+        <v>20774364.25494644</v>
       </c>
       <c r="I69" t="n">
-        <v>2067229750.20941</v>
+        <v>1832327499.243611</v>
       </c>
       <c r="J69" t="n">
         <v>-0.6941248011433353</v>
@@ -2809,13 +2809,13 @@
         <v>2.118769808888522</v>
       </c>
       <c r="G70" t="n">
-        <v>881787.2183969294</v>
+        <v>781588.4850663324</v>
       </c>
       <c r="H70" t="n">
-        <v>32008516.74827868</v>
+        <v>28371343.55382099</v>
       </c>
       <c r="I70" t="n">
-        <v>4112938357.981468</v>
+        <v>3645579334.014464</v>
       </c>
       <c r="J70" t="n">
         <v>1.033802837172117</v>
@@ -2843,13 +2843,13 @@
         <v>2.374455858833616</v>
       </c>
       <c r="G71" t="n">
-        <v>809743.2160934155</v>
+        <v>717730.9450116161</v>
       </c>
       <c r="H71" t="n">
-        <v>29960498.99545638</v>
+        <v>26556044.9654298</v>
       </c>
       <c r="I71" t="n">
-        <v>1789249492.164263</v>
+        <v>1585934532.515379</v>
       </c>
       <c r="J71" t="n">
         <v>0.4404970943555943</v>
@@ -2877,13 +2877,13 @@
         <v>1.800774401633875</v>
       </c>
       <c r="G72" t="n">
-        <v>834866.8653929182</v>
+        <v>739999.758377991</v>
       </c>
       <c r="H72" t="n">
-        <v>41743343.2696459</v>
+        <v>36999987.91889954</v>
       </c>
       <c r="I72" t="n">
-        <v>5944706312.759151</v>
+        <v>5269200895.881195</v>
       </c>
       <c r="J72" t="n">
         <v>0.5606894324126999</v>
@@ -2911,13 +2911,13 @@
         <v>1.662943479721646</v>
       </c>
       <c r="G73" t="n">
-        <v>1158352.897013039</v>
+        <v>1026727.613034055</v>
       </c>
       <c r="H73" t="n">
-        <v>87347766.66752559</v>
+        <v>77422315.95022692</v>
       </c>
       <c r="I73" t="n">
-        <v>40501141687.0471</v>
+        <v>35898939465.44674</v>
       </c>
       <c r="J73" t="n">
         <v>-1.260124888013365</v>
@@ -2945,13 +2945,13 @@
         <v>3.208873931952691</v>
       </c>
       <c r="G74" t="n">
-        <v>488706.0217805386</v>
+        <v>433173.6628034291</v>
       </c>
       <c r="H74" t="n">
-        <v>7786471.482670101</v>
+        <v>6901683.675134473</v>
       </c>
       <c r="I74" t="n">
-        <v>1057790222.08061</v>
+        <v>937592017.603736</v>
       </c>
       <c r="J74" t="n">
         <v>2.49562259711823</v>
@@ -2979,13 +2979,13 @@
         <v>3.384179807511537</v>
       </c>
       <c r="G75" t="n">
-        <v>488706.0217805386</v>
+        <v>433173.6628034291</v>
       </c>
       <c r="H75" t="n">
-        <v>24435301.08902694</v>
+        <v>21658683.14017146</v>
       </c>
       <c r="I75" t="n">
-        <v>229911726.2809793</v>
+        <v>203786530.4620996</v>
       </c>
       <c r="J75" t="n">
         <v>0.7395250710411861</v>
@@ -3013,13 +3013,13 @@
         <v>1.89954363108434</v>
       </c>
       <c r="G76" t="n">
-        <v>954126.6829827881</v>
+        <v>845707.9136048395</v>
       </c>
       <c r="H76" t="n">
-        <v>19082533.65965576</v>
+        <v>16914158.27209679</v>
       </c>
       <c r="I76" t="n">
-        <v>1260811481.670971</v>
+        <v>1117543683.276509</v>
       </c>
       <c r="J76" t="n">
         <v>1.325854459725506</v>
@@ -3047,13 +3047,13 @@
         <v>2.273818170296539</v>
       </c>
       <c r="G77" t="n">
-        <v>865134.8177891315</v>
+        <v>766828.3203778173</v>
       </c>
       <c r="H77" t="n">
-        <v>25947866.74406912</v>
+        <v>22999373.81273191</v>
       </c>
       <c r="I77" t="n">
-        <v>2828118644.523567</v>
+        <v>2506755508.408854</v>
       </c>
       <c r="J77" t="n">
         <v>0.13557282597508</v>
@@ -3081,13 +3081,13 @@
         <v>3.55838836547066</v>
       </c>
       <c r="G78" t="n">
-        <v>1365664.032257243</v>
+        <v>1210481.689700612</v>
       </c>
       <c r="H78" t="n">
-        <v>44730191.24576841</v>
+        <v>39647436.11964018</v>
       </c>
       <c r="I78" t="n">
-        <v>15736646561.70489</v>
+        <v>13948469074.60012</v>
       </c>
       <c r="J78" t="n">
         <v>-0.3341193962242646</v>
@@ -3115,13 +3115,13 @@
         <v>2.355038326002673</v>
       </c>
       <c r="G79" t="n">
-        <v>1490029.608769978</v>
+        <v>1320715.429216254</v>
       </c>
       <c r="H79" t="n">
-        <v>73234347.64162143</v>
+        <v>64912624.76234975</v>
       </c>
       <c r="I79" t="n">
-        <v>32554673063.0518</v>
+        <v>28855439351.27309</v>
       </c>
       <c r="J79" t="n">
         <v>-0.4842784633623248</v>
@@ -3149,13 +3149,13 @@
         <v>2.113679823793869</v>
       </c>
       <c r="G80" t="n">
-        <v>1703176.342965594</v>
+        <v>1509641.997441693</v>
       </c>
       <c r="H80" t="n">
-        <v>119584618.2744327</v>
+        <v>105996048.3485672</v>
       </c>
       <c r="I80" t="n">
-        <v>16146137144.5285</v>
+        <v>14311428661.22226</v>
       </c>
       <c r="J80" t="n">
         <v>-1.06814992589538</v>
@@ -3183,13 +3183,13 @@
         <v>1.664294268071398</v>
       </c>
       <c r="G81" t="n">
-        <v>1892885.756167829</v>
+        <v>1677794.460727697</v>
       </c>
       <c r="H81" t="n">
-        <v>191974881.0690847</v>
+        <v>170160502.823294</v>
       </c>
       <c r="I81" t="n">
-        <v>94308503919.11206</v>
+        <v>83592094747.09227</v>
       </c>
       <c r="J81" t="n">
         <v>-1.326873824072968</v>
@@ -3217,13 +3217,13 @@
         <v>1.538340835265424</v>
       </c>
       <c r="G82" t="n">
-        <v>1892885.756167829</v>
+        <v>1677794.460727697</v>
       </c>
       <c r="H82" t="n">
-        <v>217681861.9593002</v>
+        <v>192946362.9836851</v>
       </c>
       <c r="I82" t="n">
-        <v>59097072958.00522</v>
+        <v>52381788669.00966</v>
       </c>
       <c r="J82" t="n">
         <v>-0.1166760577335978</v>
@@ -3251,13 +3251,13 @@
         <v>1.929169690711981</v>
       </c>
       <c r="G83" t="n">
-        <v>1743635.413659354</v>
+        <v>1545503.64650054</v>
       </c>
       <c r="H83" t="n">
-        <v>131719232.7731376</v>
+        <v>116751789.3765999</v>
       </c>
       <c r="I83" t="n">
-        <v>83057911341.96773</v>
+        <v>73619922974.79684</v>
       </c>
       <c r="J83" t="n">
         <v>1.5106373641421</v>
@@ -3285,13 +3285,13 @@
         <v>1.886327114619066</v>
       </c>
       <c r="G84" t="n">
-        <v>1743635.413659354</v>
+        <v>1545503.64650054</v>
       </c>
       <c r="H84" t="n">
-        <v>139490833.0927483</v>
+        <v>123640291.7200432</v>
       </c>
       <c r="I84" t="n">
-        <v>11146458428.07166</v>
+        <v>9879870534.401161</v>
       </c>
       <c r="J84" t="n">
         <v>0.1540710305347492</v>
@@ -3319,13 +3319,13 @@
         <v>1.886505995483197</v>
       </c>
       <c r="G85" t="n">
-        <v>1892885.756167829</v>
+        <v>1677794.460727697</v>
       </c>
       <c r="H85" t="n">
-        <v>189288575.6167828</v>
+        <v>167779446.0727697</v>
       </c>
       <c r="I85" t="n">
-        <v>12940397018.01814</v>
+        <v>11469961335.86155</v>
       </c>
       <c r="J85" t="n">
         <v>-0.242195679044257</v>
@@ -3353,13 +3353,13 @@
         <v>2.176923010599811</v>
       </c>
       <c r="G86" t="n">
-        <v>809743.2160934155</v>
+        <v>717730.9450116161</v>
       </c>
       <c r="H86" t="n">
-        <v>48584592.96560494</v>
+        <v>43063856.70069697</v>
       </c>
       <c r="I86" t="n">
-        <v>192185372.6172897</v>
+        <v>170347075.918082</v>
       </c>
       <c r="J86" t="n">
         <v>0.1217130551185047</v>
@@ -3387,13 +3387,13 @@
         <v>2.803339255488408</v>
       </c>
       <c r="G87" t="n">
-        <v>1359978.15872897</v>
+        <v>1205441.910052501</v>
       </c>
       <c r="H87" t="n">
-        <v>108798252.6983176</v>
+        <v>96435352.80420002</v>
       </c>
       <c r="I87" t="n">
-        <v>73662604.92278442</v>
+        <v>65292218.56073949</v>
       </c>
       <c r="J87" t="n">
         <v>-0.3300007082497931</v>
@@ -3421,13 +3421,13 @@
         <v>2.313212370015794</v>
       </c>
       <c r="G88" t="n">
-        <v>781253.7850946437</v>
+        <v>692478.8084982146</v>
       </c>
       <c r="H88" t="n">
-        <v>35156420.32925897</v>
+        <v>31161546.38241966</v>
       </c>
       <c r="I88" t="n">
-        <v>2369110807.930419</v>
+        <v>2099905383.853157</v>
       </c>
       <c r="J88" t="n">
         <v>0.3942829371039798</v>
@@ -3455,13 +3455,13 @@
         <v>2.353526411073462</v>
       </c>
       <c r="G89" t="n">
-        <v>1703176.342965594</v>
+        <v>1509641.997441693</v>
       </c>
       <c r="H89" t="n">
-        <v>127738225.7224196</v>
+        <v>113223149.808127</v>
       </c>
       <c r="I89" t="n">
-        <v>2972662928.564954</v>
+        <v>2634875020.272828</v>
       </c>
       <c r="J89" t="n">
         <v>0.2229042444227899</v>
@@ -3489,13 +3489,13 @@
         <v>1.653622329073557</v>
       </c>
       <c r="G90" t="n">
-        <v>3518518.935720877</v>
+        <v>3118704.634488565</v>
       </c>
       <c r="H90" t="n">
-        <v>562963029.7153403</v>
+        <v>498992741.5181704</v>
       </c>
       <c r="I90" t="n">
-        <v>2308728248.115604</v>
+        <v>2046384180.023636</v>
       </c>
       <c r="J90" t="n">
         <v>-0.4019223458759687</v>
@@ -3523,13 +3523,13 @@
         <v>1.621291185719461</v>
       </c>
       <c r="G91" t="n">
-        <v>3730716.828462308</v>
+        <v>3306790.179461147</v>
       </c>
       <c r="H91" t="n">
-        <v>969986375.4002001</v>
+        <v>859765446.6598983</v>
       </c>
       <c r="I91" t="n">
-        <v>13376070886.35903</v>
+        <v>11856128964.10025</v>
       </c>
       <c r="J91" t="n">
         <v>-1.111236709763408</v>
@@ -3557,13 +3557,13 @@
         <v>2.704362102058114</v>
       </c>
       <c r="G92" t="n">
-        <v>824813.4129277262</v>
+        <v>731088.6939873766</v>
       </c>
       <c r="H92" t="n">
-        <v>13195785.7339291</v>
+        <v>11696329.86945718</v>
       </c>
       <c r="I92" t="n">
-        <v>345942803.1859718</v>
+        <v>306632831.391317</v>
       </c>
       <c r="J92" t="n">
         <v>0.008433295864435024</v>
@@ -3591,13 +3591,13 @@
         <v>2.903794056576392</v>
       </c>
       <c r="G93" t="n">
-        <v>865134.8177891315</v>
+        <v>766828.3203778173</v>
       </c>
       <c r="H93" t="n">
-        <v>12977022.26683698</v>
+        <v>11502424.80566726</v>
       </c>
       <c r="I93" t="n">
-        <v>697749884.2215148</v>
+        <v>618463574.4157681</v>
       </c>
       <c r="J93" t="n">
         <v>0.2987928189149225</v>
@@ -3625,13 +3625,13 @@
         <v>2.106414806033488</v>
       </c>
       <c r="G94" t="n">
-        <v>865134.8177891315</v>
+        <v>766828.3203778173</v>
       </c>
       <c r="H94" t="n">
-        <v>25088909.71588482</v>
+        <v>22238021.29095671</v>
       </c>
       <c r="I94" t="n">
-        <v>954358336.4953076</v>
+        <v>845913243.9998974</v>
       </c>
       <c r="J94" t="n">
         <v>-0.3451456876604662</v>
@@ -3659,13 +3659,13 @@
         <v>2.043090480942521</v>
       </c>
       <c r="G95" t="n">
-        <v>1484209.927069736</v>
+        <v>1315557.046208696</v>
       </c>
       <c r="H95" t="n">
-        <v>222631489.0604604</v>
+        <v>197333556.9313044</v>
       </c>
       <c r="I95" t="n">
-        <v>9966392756.590641</v>
+        <v>8833897400.283381</v>
       </c>
       <c r="J95" t="n">
         <v>-0.2228894695439083</v>
@@ -3693,13 +3693,13 @@
         <v>1.855077351120051</v>
       </c>
       <c r="G96" t="n">
-        <v>1690957.395410284</v>
+        <v>1498811.506241988</v>
       </c>
       <c r="H96" t="n">
-        <v>253643609.3115426</v>
+        <v>224821725.9362983</v>
       </c>
       <c r="I96" t="n">
-        <v>14275128859.80559</v>
+        <v>12653025703.80395</v>
       </c>
       <c r="J96" t="n">
         <v>-0.05633405688587591</v>
@@ -3727,13 +3727,13 @@
         <v>1.670513388775463</v>
       </c>
       <c r="G97" t="n">
-        <v>1963389.199614546</v>
+        <v>1740286.49781535</v>
       </c>
       <c r="H97" t="n">
-        <v>279535758.4180463</v>
+        <v>247771713.385713</v>
       </c>
       <c r="I97" t="n">
-        <v>2397700636.437171</v>
+        <v>2125246509.563191</v>
       </c>
       <c r="J97" t="n">
         <v>-0.4896919372250297</v>
@@ -3761,13 +3761,13 @@
         <v>1.780474223446541</v>
       </c>
       <c r="G98" t="n">
-        <v>1963389.199614546</v>
+        <v>1740286.49781535</v>
       </c>
       <c r="H98" t="n">
-        <v>274874487.9460363</v>
+        <v>243640109.694149</v>
       </c>
       <c r="I98" t="n">
-        <v>2626224155.591627</v>
+        <v>2327802576.845126</v>
       </c>
       <c r="J98" t="n">
         <v>-0.2499201623741735</v>
@@ -3795,13 +3795,13 @@
         <v>2.011201253621685</v>
       </c>
       <c r="G99" t="n">
-        <v>1485352.786834463</v>
+        <v>1316570.041196058</v>
       </c>
       <c r="H99" t="n">
-        <v>63663088.12616313</v>
+        <v>56428961.05211399</v>
       </c>
       <c r="I99" t="n">
-        <v>1729018906.273149</v>
+        <v>1532548033.59688</v>
       </c>
       <c r="J99" t="n">
         <v>0.3145632119546559</v>
@@ -3829,13 +3829,13 @@
         <v>1.97942671109101</v>
       </c>
       <c r="G100" t="n">
-        <v>906301.8578779731</v>
+        <v>803317.4912644143</v>
       </c>
       <c r="H100" t="n">
-        <v>29885994.51403764</v>
+        <v>26490006.5339944</v>
       </c>
       <c r="I100" t="n">
-        <v>5236246575.108992</v>
+        <v>4641244443.884604</v>
       </c>
       <c r="J100" t="n">
         <v>0.6206152799119374</v>
@@ -3863,13 +3863,13 @@
         <v>3.550313974429316</v>
       </c>
       <c r="G101" t="n">
-        <v>809227.4234274246</v>
+        <v>717273.7625984336</v>
       </c>
       <c r="H101" t="n">
-        <v>21849140.43254047</v>
+        <v>19366391.59015771</v>
       </c>
       <c r="I101" t="n">
-        <v>211496094.7527197</v>
+        <v>187463493.2855353</v>
       </c>
       <c r="J101" t="n">
         <v>0.01747954020451694</v>
@@ -3897,13 +3897,13 @@
         <v>6.027772899553292</v>
       </c>
       <c r="G102" t="n">
-        <v>462306.9411155339</v>
+        <v>409774.3471480994</v>
       </c>
       <c r="H102" t="n">
-        <v>13869208.23346602</v>
+        <v>12293230.41444298</v>
       </c>
       <c r="I102" t="n">
-        <v>362875489.5095346</v>
+        <v>321641432.5318469</v>
       </c>
       <c r="J102" t="n">
         <v>0.4867669899500718</v>
@@ -3931,13 +3931,13 @@
         <v>2.345739057351345</v>
       </c>
       <c r="G103" t="n">
-        <v>1321770.522763492</v>
+        <v>1171575.86199783</v>
       </c>
       <c r="H103" t="n">
-        <v>122920065.8875646</v>
+        <v>108952484.3147238</v>
       </c>
       <c r="I103" t="n">
-        <v>23995772976.78061</v>
+        <v>21269099231.23343</v>
       </c>
       <c r="J103" t="n">
         <v>-0.8185617128641272</v>
@@ -3965,13 +3965,13 @@
         <v>4.370135818413353</v>
       </c>
       <c r="G104" t="n">
-        <v>1359978.15872897</v>
+        <v>1205441.910052501</v>
       </c>
       <c r="H104" t="n">
-        <v>108798252.6983176</v>
+        <v>96435352.80420002</v>
       </c>
       <c r="I104" t="n">
-        <v>1306474952.548206</v>
+        <v>1158018349.138294</v>
       </c>
       <c r="J104" t="n">
         <v>0.8031375102129624</v>
@@ -3999,13 +3999,13 @@
         <v>3.271437003499027</v>
       </c>
       <c r="G105" t="n">
-        <v>1850480.06637813</v>
+        <v>1640207.389664024</v>
       </c>
       <c r="H105" t="n">
-        <v>240562408.6291569</v>
+        <v>213226960.6563232</v>
       </c>
       <c r="I105" t="n">
-        <v>2821519964.738987</v>
+        <v>2500906645.975076</v>
       </c>
       <c r="J105" t="n">
         <v>-0.7984587759301017</v>
@@ -4033,13 +4033,13 @@
         <v>2.111058972320168</v>
       </c>
       <c r="G106" t="n">
-        <v>1801863.638150904</v>
+        <v>1597115.315187675</v>
       </c>
       <c r="H106" t="n">
-        <v>270279545.7226356</v>
+        <v>239567297.2781512</v>
       </c>
       <c r="I106" t="n">
-        <v>9380053764.823683</v>
+        <v>8314184940.463885</v>
       </c>
       <c r="J106" t="n">
         <v>-1.17482502842645</v>
@@ -4067,13 +4067,13 @@
         <v>3.04765368496966</v>
       </c>
       <c r="G107" t="n">
-        <v>1632052.249772197</v>
+        <v>1446599.835919092</v>
       </c>
       <c r="H107" t="n">
-        <v>163205224.9772197</v>
+        <v>144659983.5919092</v>
       </c>
       <c r="I107" t="n">
-        <v>3964905907.258588</v>
+        <v>3514368020.800497</v>
       </c>
       <c r="J107" t="n">
         <v>-0.06387731674032879</v>

</xml_diff>